<commit_message>
Auto update AlphaForge data
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -1006,10 +1006,10 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>68.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="F3" t="n">
-        <v>64.59999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 68.9; priority 64.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 68.8; priority 64.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>prezzo 9.4% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 9.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.9, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.4%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.5%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1094,10 +1094,10 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>28.94</v>
+        <v>29.08</v>
       </c>
       <c r="Z3" t="n">
-        <v>40.02</v>
+        <v>40.18</v>
       </c>
       <c r="AA3" t="n">
         <v>21.32</v>
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>17.69</v>
+        <v>17.71</v>
       </c>
       <c r="AH3" t="n">
         <v>51.3</v>
@@ -1130,25 +1130,25 @@
         <v>45.9</v>
       </c>
       <c r="AK3" t="n">
-        <v>61.1</v>
+        <v>60.6</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="AM3" t="n">
-        <v>26.88</v>
+        <v>27.03</v>
       </c>
       <c r="AN3" t="n">
-        <v>17.88</v>
+        <v>17.92</v>
       </c>
       <c r="AO3" t="n">
         <v>0.84</v>
       </c>
       <c r="AP3" t="n">
-        <v>16.1688</v>
+        <v>16.1692</v>
       </c>
       <c r="AQ3" t="n">
-        <v>14.4672</v>
+        <v>14.4673</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
@@ -1161,7 +1161,7 @@
         <v>50.9</v>
       </c>
       <c r="AV3" t="n">
-        <v>61.1</v>
+        <v>60.6</v>
       </c>
       <c r="AW3" t="n">
         <v>756</v>
@@ -1173,10 +1173,10 @@
         <v>18.17</v>
       </c>
       <c r="AZ3" t="n">
-        <v>9.41</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="BA3" t="n">
-        <v>22.28</v>
+        <v>22.41</v>
       </c>
       <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="inlineStr"/>
@@ -2406,10 +2406,10 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>7.67</v>
+        <v>7.69</v>
       </c>
       <c r="Z9" t="n">
-        <v>-15.26</v>
+        <v>-15.25</v>
       </c>
       <c r="AA9" t="n">
         <v>33.93</v>
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="AG9" t="n">
-        <v>26.875</v>
+        <v>26.88</v>
       </c>
       <c r="AH9" t="n">
         <v>22.4</v>
@@ -2442,13 +2442,13 @@
         <v>15.4</v>
       </c>
       <c r="AK9" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="AL9" t="n">
-        <v>11.51</v>
+        <v>11.54</v>
       </c>
       <c r="AM9" t="n">
-        <v>-7.46</v>
+        <v>-7.44</v>
       </c>
       <c r="AN9" t="n">
         <v>-1.98</v>
@@ -2457,7 +2457,7 @@
         <v>-0.06</v>
       </c>
       <c r="AP9" t="n">
-        <v>24.2645</v>
+        <v>24.2646</v>
       </c>
       <c r="AQ9" t="n">
         <v>26.9667</v>
@@ -2473,7 +2473,7 @@
         <v>20.4</v>
       </c>
       <c r="AV9" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="AW9" t="n">
         <v>757</v>
@@ -2485,10 +2485,10 @@
         <v>30.11</v>
       </c>
       <c r="AZ9" t="n">
-        <v>10.76</v>
+        <v>10.78</v>
       </c>
       <c r="BA9" t="n">
-        <v>-0.34</v>
+        <v>-0.32</v>
       </c>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
@@ -2528,10 +2528,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>62</v>
+        <v>62.1</v>
       </c>
       <c r="F10" t="n">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 62.0; priority 19.8; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 62.1; priority 20.2; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2560,17 +2560,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>prezzo 18.3% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 18.2% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 62.0, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.3%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 62.1, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.2%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1527.80 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1526.20 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -2597,7 +2597,7 @@
         <v>1109.5466</v>
       </c>
       <c r="T10" t="n">
-        <v>1527.8</v>
+        <v>1526.2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -2612,10 +2612,10 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>33.42</v>
+        <v>33.28</v>
       </c>
       <c r="Z10" t="n">
-        <v>127.61</v>
+        <v>127.37</v>
       </c>
       <c r="AA10" t="n">
         <v>38.1</v>
@@ -2624,10 +2624,10 @@
         <v>-44.77</v>
       </c>
       <c r="AC10" t="n">
-        <v>58.99</v>
+        <v>58.93</v>
       </c>
       <c r="AD10" t="n">
-        <v>36.85</v>
+        <v>36.81</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
@@ -2636,29 +2636,29 @@
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="n">
-        <v>1527.8</v>
+        <v>1526.2</v>
       </c>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
-        <v>17.02</v>
+        <v>16.9</v>
       </c>
       <c r="AM10" t="n">
-        <v>61.12</v>
+        <v>60.95</v>
       </c>
       <c r="AN10" t="n">
-        <v>32.55</v>
+        <v>32.51</v>
       </c>
       <c r="AO10" t="n">
         <v>0.85</v>
       </c>
       <c r="AP10" t="n">
-        <v>1291.6841</v>
+        <v>1291.6521</v>
       </c>
       <c r="AQ10" t="n">
-        <v>1052.314</v>
+        <v>1052.306</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
@@ -2671,7 +2671,7 @@
         <v>18.5</v>
       </c>
       <c r="AV10" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="AW10" t="n">
         <v>765</v>
@@ -2680,13 +2680,13 @@
         <v>1249</v>
       </c>
       <c r="AY10" t="n">
-        <v>1527.8</v>
+        <v>1526.2</v>
       </c>
       <c r="AZ10" t="n">
-        <v>18.28</v>
+        <v>18.16</v>
       </c>
       <c r="BA10" t="n">
-        <v>45.18</v>
+        <v>45.03</v>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
@@ -2699,7 +2699,7 @@
         </is>
       </c>
       <c r="BD10" t="n">
-        <v>588841156608</v>
+        <v>588224397312</v>
       </c>
       <c r="BE10" t="n">
         <v>29.71</v>
@@ -2723,13 +2723,13 @@
         <v>100</v>
       </c>
       <c r="BL10" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="BM10" t="n">
         <v>18.5</v>
       </c>
       <c r="BN10" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="BO10" t="inlineStr"/>
       <c r="BP10" t="inlineStr">
@@ -3403,7 +3403,7 @@
         <v>76.40000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>76.8</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 76.4; priority 76.8; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 76.4; priority 76.9; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.1%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.0%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>10.53</v>
+        <v>10.46</v>
       </c>
       <c r="Z14" t="n">
-        <v>24.3</v>
+        <v>24.23</v>
       </c>
       <c r="AA14" t="n">
         <v>12.86</v>
@@ -3512,50 +3512,50 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>161.82</v>
+        <v>161.72</v>
       </c>
       <c r="AH14" t="n">
         <v>72.90000000000001</v>
       </c>
       <c r="AI14" t="n">
-        <v>78.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="AJ14" t="n">
         <v>67.7</v>
       </c>
       <c r="AK14" t="n">
-        <v>82.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AL14" t="n">
-        <v>2.02</v>
+        <v>1.95</v>
       </c>
       <c r="AM14" t="n">
-        <v>12.17</v>
+        <v>12.1</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.23</v>
+        <v>17.21</v>
       </c>
       <c r="AO14" t="n">
         <v>1.34</v>
       </c>
       <c r="AP14" t="n">
-        <v>155.4296</v>
+        <v>155.4276</v>
       </c>
       <c r="AQ14" t="n">
-        <v>146.7653</v>
+        <v>146.7648</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>78.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="AU14" t="n">
         <v>67.7</v>
       </c>
       <c r="AV14" t="n">
-        <v>82.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AW14" t="n">
         <v>759</v>
@@ -3567,10 +3567,10 @@
         <v>164.88</v>
       </c>
       <c r="AZ14" t="n">
-        <v>4.11</v>
+        <v>4.05</v>
       </c>
       <c r="BA14" t="n">
-        <v>10.26</v>
+        <v>10.19</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.9%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -3694,10 +3694,10 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>9.859999999999999</v>
+        <v>9.85</v>
       </c>
       <c r="Z15" t="n">
-        <v>22.31</v>
+        <v>22.29</v>
       </c>
       <c r="AA15" t="n">
         <v>13.13</v>
@@ -3718,13 +3718,13 @@
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>122.52</v>
+        <v>122.5</v>
       </c>
       <c r="AH15" t="n">
         <v>71.8</v>
       </c>
       <c r="AI15" t="n">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="AJ15" t="n">
         <v>66.90000000000001</v>
@@ -3733,10 +3733,10 @@
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>2.15</v>
+        <v>2.13</v>
       </c>
       <c r="AM15" t="n">
-        <v>10.34</v>
+        <v>10.32</v>
       </c>
       <c r="AN15" t="n">
         <v>17.12</v>
@@ -3745,17 +3745,17 @@
         <v>1.3</v>
       </c>
       <c r="AP15" t="n">
-        <v>117.9804</v>
+        <v>117.98</v>
       </c>
       <c r="AQ15" t="n">
-        <v>112.2004</v>
+        <v>112.2003</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="AU15" t="n">
         <v>66.90000000000001</v>
@@ -3773,10 +3773,10 @@
         <v>124.27</v>
       </c>
       <c r="AZ15" t="n">
-        <v>3.85</v>
+        <v>3.83</v>
       </c>
       <c r="BA15" t="n">
-        <v>9.199999999999999</v>
+        <v>9.18</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.5%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.4%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -4106,10 +4106,10 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>11.21</v>
+        <v>11.16</v>
       </c>
       <c r="Z17" t="n">
-        <v>23.57</v>
+        <v>23.52</v>
       </c>
       <c r="AA17" t="n">
         <v>14.09</v>
@@ -4130,50 +4130,50 @@
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>692.16</v>
+        <v>691.88</v>
       </c>
       <c r="AH17" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="AI17" t="n">
-        <v>77.59999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="AJ17" t="n">
         <v>64.40000000000001</v>
       </c>
       <c r="AK17" t="n">
-        <v>80.90000000000001</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="AL17" t="n">
-        <v>2.23</v>
+        <v>2.19</v>
       </c>
       <c r="AM17" t="n">
-        <v>10.09</v>
+        <v>10.05</v>
       </c>
       <c r="AN17" t="n">
-        <v>18.37</v>
+        <v>18.36</v>
       </c>
       <c r="AO17" t="n">
         <v>1.3</v>
       </c>
       <c r="AP17" t="n">
-        <v>662.6624</v>
+        <v>662.6568</v>
       </c>
       <c r="AQ17" t="n">
-        <v>629.9932</v>
+        <v>629.9918</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>85</v>
       </c>
       <c r="AT17" t="n">
-        <v>77.59999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="AU17" t="n">
         <v>64.40000000000001</v>
       </c>
       <c r="AV17" t="n">
-        <v>80.90000000000001</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="AW17" t="n">
         <v>759</v>
@@ -4185,10 +4185,10 @@
         <v>703.9400000000001</v>
       </c>
       <c r="AZ17" t="n">
-        <v>4.45</v>
+        <v>4.41</v>
       </c>
       <c r="BA17" t="n">
-        <v>9.869999999999999</v>
+        <v>9.82</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -5132,12 +5132,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>prezzo 5.3% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 5.2% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 55.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -5.3%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 55.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -5.2%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 360.75 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 360.85 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>360.75</v>
+        <v>360.85</v>
       </c>
       <c r="T22" t="n">
         <v>424.57</v>
@@ -5188,16 +5188,16 @@
         </is>
       </c>
       <c r="Y22" t="n">
-        <v>-14.83</v>
+        <v>-14.8</v>
       </c>
       <c r="Z22" t="n">
-        <v>27.63</v>
+        <v>27.66</v>
       </c>
       <c r="AA22" t="n">
         <v>17.78</v>
       </c>
       <c r="AB22" t="n">
-        <v>-17.33</v>
+        <v>-17.31</v>
       </c>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
@@ -5212,13 +5212,13 @@
         </is>
       </c>
       <c r="AG22" t="n">
-        <v>360.75</v>
+        <v>360.85</v>
       </c>
       <c r="AH22" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="AI22" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="AJ22" t="n">
         <v>64.8</v>
@@ -5227,29 +5227,29 @@
         <v>67.40000000000001</v>
       </c>
       <c r="AL22" t="n">
-        <v>-6.67</v>
+        <v>-6.65</v>
       </c>
       <c r="AM22" t="n">
-        <v>3.98</v>
+        <v>4.01</v>
       </c>
       <c r="AN22" t="n">
-        <v>26.96</v>
+        <v>26.97</v>
       </c>
       <c r="AO22" t="n">
         <v>1.52</v>
       </c>
       <c r="AP22" t="n">
-        <v>380.8004</v>
+        <v>380.8024</v>
       </c>
       <c r="AQ22" t="n">
-        <v>362.171</v>
+        <v>362.1715</v>
       </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
         <v>35</v>
       </c>
       <c r="AT22" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="AU22" t="n">
         <v>64.8</v>
@@ -5261,16 +5261,16 @@
         <v>756</v>
       </c>
       <c r="AX22" t="n">
-        <v>360.75</v>
+        <v>360.85</v>
       </c>
       <c r="AY22" t="n">
         <v>386.38</v>
       </c>
       <c r="AZ22" t="n">
-        <v>-5.27</v>
+        <v>-5.24</v>
       </c>
       <c r="BA22" t="n">
-        <v>-0.39</v>
+        <v>-0.36</v>
       </c>
       <c r="BB22" t="inlineStr"/>
       <c r="BC22" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v6_action_portfolio_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -766,24 +766,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>RBOT.MI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>iShares Automation &amp; Robotics UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>66.8</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>66.59999999999999</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -797,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 66.8; priority 66.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 69.6; priority 68.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -812,22 +808,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 8.1% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>AMZN: scenario base Hold / Monitor, score 66.8, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.7%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 69.6, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 8.1%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 274.99 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 18.17 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 199.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 12.94 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -837,156 +833,136 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>199.34</v>
+        <v>12.936</v>
       </c>
       <c r="T2" t="n">
-        <v>274.99</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Amazon.com, Inc.</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+        <v>18.17</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>iShares Automation &amp; Robotics UCITS ETF USD (Acc)</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>14.86</v>
+        <v>27.35</v>
       </c>
       <c r="Z2" t="n">
-        <v>17.95</v>
+        <v>38.29</v>
       </c>
       <c r="AA2" t="n">
-        <v>30.99</v>
+        <v>21.33</v>
       </c>
       <c r="AB2" t="n">
-        <v>-30.88</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>31.64</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>24.86</v>
-      </c>
+        <v>-29.37</v>
+      </c>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr"/>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Robotica e automazione</t>
+        </is>
+      </c>
       <c r="AG2" t="n">
-        <v>245.22</v>
-      </c>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
+        <v>17.472</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>66.40000000000001</v>
+      </c>
       <c r="AL2" t="n">
-        <v>-9.57</v>
+        <v>-0.31</v>
       </c>
       <c r="AM2" t="n">
-        <v>7.03</v>
+        <v>25.32</v>
       </c>
       <c r="AN2" t="n">
-        <v>25.9</v>
+        <v>17.39</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="AP2" t="n">
-        <v>251.9112</v>
+        <v>16.1644</v>
       </c>
       <c r="AQ2" t="n">
-        <v>232.2354</v>
+        <v>14.4661</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>79.5</v>
+        <v>100</v>
       </c>
       <c r="AU2" t="n">
-        <v>38.1</v>
+        <v>50.9</v>
       </c>
       <c r="AV2" t="n">
-        <v>75.8</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AW2" t="n">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="AX2" t="n">
-        <v>245.22</v>
+        <v>16.544</v>
       </c>
       <c r="AY2" t="n">
-        <v>274</v>
+        <v>18.17</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-2.66</v>
+        <v>8.09</v>
       </c>
       <c r="BA2" t="n">
-        <v>5.59</v>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>Internet Retail</t>
-        </is>
-      </c>
-      <c r="BD2" t="n">
-        <v>2637858340864</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>12.22</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>24.29</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="BH2" t="n">
-        <v>53.3</v>
-      </c>
+        <v>20.78</v>
+      </c>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>79.5</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>75.8</v>
-      </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
       <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>USA / Consumer &amp; Cloud</t>
-        </is>
-      </c>
+      <c r="BP2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -996,20 +972,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RBOT.MI</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>iShares Automation &amp; Robotics UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E3" t="n">
-        <v>68.8</v>
+        <v>66.3</v>
       </c>
       <c r="F3" t="n">
-        <v>64.2</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1023,7 +1003,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 68.8; priority 64.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 66.3; priority 65.9; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1038,22 +1018,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>prezzo 9.5% sopra MA50: evitare inseguimento</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.5%.</t>
+          <t>AMZN: scenario base Hold / Monitor, score 66.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.2%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 18.17 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 274.99 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 12.94 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 199.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1063,136 +1043,156 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>12.936</v>
+        <v>199.34</v>
       </c>
       <c r="T3" t="n">
-        <v>18.17</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>iShares Automation &amp; Robotics UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>274.99</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>29.08</v>
+        <v>14.2</v>
       </c>
       <c r="Z3" t="n">
-        <v>40.18</v>
+        <v>14.61</v>
       </c>
       <c r="AA3" t="n">
-        <v>21.32</v>
+        <v>30.97</v>
       </c>
       <c r="AB3" t="n">
-        <v>-29.37</v>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
+        <v>-30.88</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>31.58</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>24.82</v>
+      </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>Robotica e automazione</t>
-        </is>
-      </c>
+          <t>Da monitorare con scenario positivo, base e negativo.</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="n">
-        <v>17.71</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>60.6</v>
-      </c>
+        <v>244.772</v>
+      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="n">
-        <v>1.05</v>
+        <v>-10.23</v>
       </c>
       <c r="AM3" t="n">
-        <v>27.03</v>
+        <v>6.64</v>
       </c>
       <c r="AN3" t="n">
-        <v>17.92</v>
+        <v>25.79</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="AP3" t="n">
-        <v>16.1692</v>
+        <v>252.8198</v>
       </c>
       <c r="AQ3" t="n">
-        <v>14.4673</v>
+        <v>232.3495</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT3" t="n">
-        <v>100</v>
+        <v>77.5</v>
       </c>
       <c r="AU3" t="n">
-        <v>50.9</v>
+        <v>38.1</v>
       </c>
       <c r="AV3" t="n">
-        <v>60.6</v>
+        <v>75</v>
       </c>
       <c r="AW3" t="n">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="AX3" t="n">
-        <v>16.544</v>
+        <v>244.772</v>
       </c>
       <c r="AY3" t="n">
-        <v>18.17</v>
+        <v>274</v>
       </c>
       <c r="AZ3" t="n">
-        <v>9.529999999999999</v>
+        <v>-3.18</v>
       </c>
       <c r="BA3" t="n">
-        <v>22.41</v>
-      </c>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
+        <v>5.35</v>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>Internet Retail</t>
+        </is>
+      </c>
+      <c r="BD3" t="n">
+        <v>2633039347712</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>24.29</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>53.3</v>
+      </c>
       <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
+      <c r="BJ3" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>75</v>
+      </c>
       <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>USA / Consumer &amp; Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1216,10 +1216,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>65.5</v>
+        <v>63.8</v>
       </c>
       <c r="F4" t="n">
-        <v>61.6</v>
+        <v>59.6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1233,12 +1233,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 65.5; priority 61.6; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 63.8; priority 59.6; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>MSFT: scenario base Hold / Monitor, score 65.5, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.8%.</t>
+          <t>MSFT: scenario base Hold / Monitor, score 63.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.7%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Recovery</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S4" t="n">
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>0.79</v>
+        <v>0.43</v>
       </c>
       <c r="Z4" t="n">
-        <v>-11.26</v>
+        <v>-12.86</v>
       </c>
       <c r="AA4" t="n">
         <v>23.97</v>
@@ -1312,57 +1312,57 @@
         <v>-33.91</v>
       </c>
       <c r="AC4" t="n">
-        <v>24.51</v>
+        <v>24.2</v>
       </c>
       <c r="AD4" t="n">
-        <v>21.29</v>
+        <v>21.02</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
+          <t>Trend debole: meglio aspettare stabilizzazione tecnica.</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>411.74</v>
+        <v>406.635</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>-1.93</v>
+        <v>-1.83</v>
       </c>
       <c r="AM4" t="n">
-        <v>-13.99</v>
+        <v>-15.46</v>
       </c>
       <c r="AN4" t="n">
-        <v>8.91</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="AP4" t="n">
-        <v>408.6026</v>
+        <v>409.6153</v>
       </c>
       <c r="AQ4" t="n">
-        <v>453.9891</v>
+        <v>453.517</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="AT4" t="n">
-        <v>39.9</v>
+        <v>38.1</v>
       </c>
       <c r="AU4" t="n">
         <v>44.1</v>
       </c>
       <c r="AV4" t="n">
-        <v>78.2</v>
+        <v>74.2</v>
       </c>
       <c r="AW4" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX4" t="n">
         <v>404.3343</v>
@@ -1371,10 +1371,10 @@
         <v>460.52</v>
       </c>
       <c r="AZ4" t="n">
-        <v>0.77</v>
+        <v>-0.73</v>
       </c>
       <c r="BA4" t="n">
-        <v>-9.31</v>
+        <v>-10.34</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>3058583732224</v>
+        <v>3020624494592</v>
       </c>
       <c r="BE4" t="n">
         <v>39.34</v>
@@ -1408,16 +1408,16 @@
         <v>100</v>
       </c>
       <c r="BK4" t="n">
-        <v>39.9</v>
+        <v>38.1</v>
       </c>
       <c r="BL4" t="n">
-        <v>69.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="BM4" t="n">
         <v>44.1</v>
       </c>
       <c r="BN4" t="n">
-        <v>78.2</v>
+        <v>74.2</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1444,10 +1444,10 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>64.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 64.3; priority 58.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 64.1; priority 58.1; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Hold / Monitor, score 64.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.8%.</t>
+          <t>INRG.MI: scenario base Hold / Monitor, score 64.1, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.1%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1532,13 +1532,13 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>20.41</v>
+        <v>17.17</v>
       </c>
       <c r="Z5" t="n">
-        <v>66.43000000000001</v>
+        <v>61.96</v>
       </c>
       <c r="AA5" t="n">
-        <v>23.17</v>
+        <v>23.22</v>
       </c>
       <c r="AB5" t="n">
         <v>-44.26</v>
@@ -1556,37 +1556,37 @@
         </is>
       </c>
       <c r="AG5" t="n">
-        <v>10.572</v>
+        <v>10.288</v>
       </c>
       <c r="AH5" t="n">
-        <v>31.2</v>
+        <v>30.4</v>
       </c>
       <c r="AI5" t="n">
         <v>100</v>
       </c>
       <c r="AJ5" t="n">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="AK5" t="n">
         <v>82.8</v>
       </c>
       <c r="AL5" t="n">
-        <v>-1.19</v>
+        <v>-3.84</v>
       </c>
       <c r="AM5" t="n">
-        <v>29.13</v>
+        <v>25.66</v>
       </c>
       <c r="AN5" t="n">
-        <v>3.25</v>
+        <v>2.32</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="AP5" t="n">
-        <v>10.1817</v>
+        <v>10.176</v>
       </c>
       <c r="AQ5" t="n">
-        <v>8.756500000000001</v>
+        <v>8.755100000000001</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
@@ -1596,7 +1596,7 @@
         <v>100</v>
       </c>
       <c r="AU5" t="n">
-        <v>36.8</v>
+        <v>36.7</v>
       </c>
       <c r="AV5" t="n">
         <v>82.8</v>
@@ -1611,10 +1611,10 @@
         <v>11.61</v>
       </c>
       <c r="AZ5" t="n">
-        <v>3.83</v>
+        <v>1.1</v>
       </c>
       <c r="BA5" t="n">
-        <v>20.73</v>
+        <v>17.51</v>
       </c>
       <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr"/>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="F6" t="n">
-        <v>39.7</v>
+        <v>40.2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 59.4; priority 39.7; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 59.5; priority 40.2; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1686,12 +1686,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>prezzo 5.6% sotto MA50: attendere recupero</t>
+          <t>prezzo 4.6% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>META: scenario base Hold / Monitor, score 59.4, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -5.6%.</t>
+          <t>META: scenario base Hold / Monitor, score 59.5, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -4.6%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1738,22 +1738,22 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-9.5</v>
+        <v>-9.24</v>
       </c>
       <c r="Z6" t="n">
-        <v>-14.23</v>
+        <v>-14.73</v>
       </c>
       <c r="AA6" t="n">
-        <v>36.3</v>
+        <v>36.28</v>
       </c>
       <c r="AB6" t="n">
         <v>-34.15</v>
       </c>
       <c r="AC6" t="n">
-        <v>21.28</v>
+        <v>21.56</v>
       </c>
       <c r="AD6" t="n">
-        <v>16.19</v>
+        <v>16.4</v>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
@@ -1762,29 +1762,29 @@
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>585.39</v>
+        <v>593.12</v>
       </c>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>-5.09</v>
+        <v>-2.71</v>
       </c>
       <c r="AM6" t="n">
-        <v>-11.36</v>
+        <v>-11.78</v>
       </c>
       <c r="AN6" t="n">
-        <v>30.82</v>
+        <v>31.35</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="AP6" t="n">
-        <v>620.2773999999999</v>
+        <v>621.6254</v>
       </c>
       <c r="AQ6" t="n">
-        <v>660.9453</v>
+        <v>660.2241</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
@@ -1797,10 +1797,10 @@
         <v>29.1</v>
       </c>
       <c r="AV6" t="n">
-        <v>66.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AW6" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX6" t="n">
         <v>585.39</v>
@@ -1809,10 +1809,10 @@
         <v>635.29</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-5.62</v>
+        <v>-4.59</v>
       </c>
       <c r="BA6" t="n">
-        <v>-11.43</v>
+        <v>-10.16</v>
       </c>
       <c r="BB6" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="BD6" t="n">
-        <v>1485967589376</v>
+        <v>1505462714368</v>
       </c>
       <c r="BE6" t="n">
         <v>32.84</v>
@@ -1849,13 +1849,13 @@
         <v>26.3</v>
       </c>
       <c r="BL6" t="n">
-        <v>80.40000000000001</v>
+        <v>79.7</v>
       </c>
       <c r="BM6" t="n">
         <v>29.1</v>
       </c>
       <c r="BN6" t="n">
-        <v>66.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="BO6" t="inlineStr"/>
       <c r="BP6" t="inlineStr">
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>41.3</v>
+        <v>39.5</v>
       </c>
       <c r="F7" t="n">
-        <v>34.9</v>
+        <v>33</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 41.3; priority 34.9; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 39.5; priority 33.0; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 41.3, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.3%.</t>
+          <t>TSLA: scenario base High Risk, score 39.5, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.6%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1970,22 +1970,22 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>2.58</v>
+        <v>-0.03</v>
       </c>
       <c r="Z7" t="n">
-        <v>43.64</v>
+        <v>35.23</v>
       </c>
       <c r="AA7" t="n">
-        <v>57.95</v>
+        <v>57.93</v>
       </c>
       <c r="AB7" t="n">
         <v>-53.77</v>
       </c>
       <c r="AC7" t="n">
-        <v>371.77</v>
+        <v>362.82</v>
       </c>
       <c r="AD7" t="n">
-        <v>163.28</v>
+        <v>159.35</v>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
@@ -1994,36 +1994,36 @@
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="n">
-        <v>408.95</v>
+        <v>399.105</v>
       </c>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-6.83</v>
       </c>
       <c r="AM7" t="n">
-        <v>-10.03</v>
+        <v>-12.28</v>
       </c>
       <c r="AN7" t="n">
-        <v>18.86</v>
+        <v>17.86</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
       <c r="AP7" t="n">
-        <v>396.0254</v>
+        <v>396.7709</v>
       </c>
       <c r="AQ7" t="n">
-        <v>414.5671</v>
+        <v>414.9621</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
         <v>55</v>
       </c>
       <c r="AT7" t="n">
-        <v>58.5</v>
+        <v>51.4</v>
       </c>
       <c r="AU7" t="n">
         <v>0</v>
@@ -2032,7 +2032,7 @@
         <v>78.2</v>
       </c>
       <c r="AW7" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX7" t="n">
         <v>391</v>
@@ -2041,10 +2041,10 @@
         <v>445.27</v>
       </c>
       <c r="AZ7" t="n">
-        <v>3.26</v>
+        <v>0.59</v>
       </c>
       <c r="BA7" t="n">
-        <v>-1.35</v>
+        <v>-3.82</v>
       </c>
       <c r="BB7" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="BD7" t="n">
-        <v>1535903268864</v>
+        <v>1498928119808</v>
       </c>
       <c r="BE7" t="n">
         <v>3.95</v>
@@ -2076,7 +2076,7 @@
         <v>64.40000000000001</v>
       </c>
       <c r="BK7" t="n">
-        <v>58.5</v>
+        <v>51.4</v>
       </c>
       <c r="BL7" t="n">
         <v>0</v>
@@ -2112,10 +2112,10 @@
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>61.9</v>
+        <v>63.3</v>
       </c>
       <c r="F8" t="n">
-        <v>25</v>
+        <v>32.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 61.9; priority 25.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 63.3; priority 32.6; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>prezzo 17.0% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 14.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>SMH: scenario base Hold / Monitor, score 61.9, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 17.0%.</t>
+          <t>SMH: scenario base Hold / Monitor, score 63.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 14.5%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -2200,13 +2200,13 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>51.67</v>
+        <v>48.55</v>
       </c>
       <c r="Z8" t="n">
-        <v>138.77</v>
+        <v>134.28</v>
       </c>
       <c r="AA8" t="n">
-        <v>34.92</v>
+        <v>34.91</v>
       </c>
       <c r="AB8" t="n">
         <v>-35.74</v>
@@ -2224,10 +2224,10 @@
         </is>
       </c>
       <c r="AG8" t="n">
-        <v>598.16</v>
+        <v>590.2506</v>
       </c>
       <c r="AH8" t="n">
-        <v>58.7</v>
+        <v>58.2</v>
       </c>
       <c r="AI8" t="n">
         <v>100</v>
@@ -2236,25 +2236,25 @@
         <v>24.5</v>
       </c>
       <c r="AK8" t="n">
-        <v>30.8</v>
+        <v>40.8</v>
       </c>
       <c r="AL8" t="n">
-        <v>10.75</v>
+        <v>4.19</v>
       </c>
       <c r="AM8" t="n">
-        <v>65.94</v>
+        <v>62.47</v>
       </c>
       <c r="AN8" t="n">
-        <v>60.94</v>
+        <v>60.12</v>
       </c>
       <c r="AO8" t="n">
-        <v>1.75</v>
+        <v>1.72</v>
       </c>
       <c r="AP8" t="n">
-        <v>511.287</v>
+        <v>515.607</v>
       </c>
       <c r="AQ8" t="n">
-        <v>397.8009</v>
+        <v>399.3193</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
@@ -2267,10 +2267,10 @@
         <v>29.5</v>
       </c>
       <c r="AV8" t="n">
-        <v>30.8</v>
+        <v>40.8</v>
       </c>
       <c r="AW8" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX8" t="n">
         <v>543.96</v>
@@ -2279,10 +2279,10 @@
         <v>637.9</v>
       </c>
       <c r="AZ8" t="n">
-        <v>16.99</v>
+        <v>14.48</v>
       </c>
       <c r="BA8" t="n">
-        <v>50.37</v>
+        <v>47.81</v>
       </c>
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr"/>
@@ -2318,10 +2318,10 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="F9" t="n">
-        <v>21.9</v>
+        <v>25.1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2335,12 +2335,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 37.7; priority 21.9; trend: Recovery; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 37.8; priority 25.1; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Extended - wait pullback</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo 10.8% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 9.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base High Risk, score 37.7, trend Recovery. Entry zone: Extended - wait pullback. Distanza da MA50: 10.8%.</t>
+          <t>WCLD.MI: scenario base High Risk, score 37.8, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.5%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -2406,13 +2406,13 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>7.69</v>
+        <v>6.41</v>
       </c>
       <c r="Z9" t="n">
-        <v>-15.25</v>
+        <v>-16.25</v>
       </c>
       <c r="AA9" t="n">
-        <v>33.93</v>
+        <v>33.95</v>
       </c>
       <c r="AB9" t="n">
         <v>-48.6</v>
@@ -2430,50 +2430,50 @@
         </is>
       </c>
       <c r="AG9" t="n">
-        <v>26.88</v>
+        <v>26.56</v>
       </c>
       <c r="AH9" t="n">
-        <v>22.4</v>
+        <v>22.2</v>
       </c>
       <c r="AI9" t="n">
-        <v>52.5</v>
+        <v>49.8</v>
       </c>
       <c r="AJ9" t="n">
         <v>15.4</v>
       </c>
       <c r="AK9" t="n">
-        <v>51.1</v>
+        <v>56.3</v>
       </c>
       <c r="AL9" t="n">
-        <v>11.54</v>
+        <v>10.21</v>
       </c>
       <c r="AM9" t="n">
-        <v>-7.44</v>
+        <v>-8.539999999999999</v>
       </c>
       <c r="AN9" t="n">
-        <v>-1.98</v>
+        <v>-2.37</v>
       </c>
       <c r="AO9" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AP9" t="n">
-        <v>24.2646</v>
+        <v>24.2582</v>
       </c>
       <c r="AQ9" t="n">
-        <v>26.9667</v>
+        <v>26.9651</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>55</v>
       </c>
       <c r="AT9" t="n">
-        <v>52.5</v>
+        <v>49.8</v>
       </c>
       <c r="AU9" t="n">
         <v>20.4</v>
       </c>
       <c r="AV9" t="n">
-        <v>51.1</v>
+        <v>56.3</v>
       </c>
       <c r="AW9" t="n">
         <v>757</v>
@@ -2485,10 +2485,10 @@
         <v>30.11</v>
       </c>
       <c r="AZ9" t="n">
-        <v>10.78</v>
+        <v>9.49</v>
       </c>
       <c r="BA9" t="n">
-        <v>-0.32</v>
+        <v>-1.5</v>
       </c>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
@@ -2528,10 +2528,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>62.1</v>
+        <v>61.6</v>
       </c>
       <c r="F10" t="n">
-        <v>20.2</v>
+        <v>17</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 62.1; priority 20.2; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 61.6; priority 17.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2560,17 +2560,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>prezzo 18.2% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 19.2% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 62.1, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.2%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 61.6, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 19.2%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1526.20 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1539.80 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -2597,7 +2597,7 @@
         <v>1109.5466</v>
       </c>
       <c r="T10" t="n">
-        <v>1526.2</v>
+        <v>1539.8</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -2612,22 +2612,22 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>33.28</v>
+        <v>34.47</v>
       </c>
       <c r="Z10" t="n">
-        <v>127.37</v>
+        <v>129.4</v>
       </c>
       <c r="AA10" t="n">
-        <v>38.1</v>
+        <v>38.11</v>
       </c>
       <c r="AB10" t="n">
         <v>-44.77</v>
       </c>
       <c r="AC10" t="n">
-        <v>58.93</v>
+        <v>59.45</v>
       </c>
       <c r="AD10" t="n">
-        <v>36.81</v>
+        <v>37.14</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
@@ -2636,29 +2636,29 @@
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="n">
-        <v>1526.2</v>
+        <v>1539.8</v>
       </c>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
-        <v>16.9</v>
+        <v>17.94</v>
       </c>
       <c r="AM10" t="n">
-        <v>60.95</v>
+        <v>62.39</v>
       </c>
       <c r="AN10" t="n">
-        <v>32.51</v>
+        <v>32.89</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="AP10" t="n">
-        <v>1291.6521</v>
+        <v>1291.9241</v>
       </c>
       <c r="AQ10" t="n">
-        <v>1052.306</v>
+        <v>1052.374</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
@@ -2668,10 +2668,10 @@
         <v>100</v>
       </c>
       <c r="AU10" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="AV10" t="n">
-        <v>26.1</v>
+        <v>22</v>
       </c>
       <c r="AW10" t="n">
         <v>765</v>
@@ -2680,13 +2680,13 @@
         <v>1249</v>
       </c>
       <c r="AY10" t="n">
-        <v>1526.2</v>
+        <v>1539.8</v>
       </c>
       <c r="AZ10" t="n">
-        <v>18.16</v>
+        <v>19.19</v>
       </c>
       <c r="BA10" t="n">
-        <v>45.03</v>
+        <v>46.32</v>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
@@ -2699,7 +2699,7 @@
         </is>
       </c>
       <c r="BD10" t="n">
-        <v>588224397312</v>
+        <v>593466163200</v>
       </c>
       <c r="BE10" t="n">
         <v>29.71</v>
@@ -2723,13 +2723,13 @@
         <v>100</v>
       </c>
       <c r="BL10" t="n">
-        <v>11.7</v>
+        <v>11.2</v>
       </c>
       <c r="BM10" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="BN10" t="n">
-        <v>26.1</v>
+        <v>22</v>
       </c>
       <c r="BO10" t="inlineStr"/>
       <c r="BP10" t="inlineStr">
@@ -2756,10 +2756,10 @@
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>79.40000000000001</v>
+        <v>79</v>
       </c>
       <c r="F11" t="n">
-        <v>79.7</v>
+        <v>80.2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 79.4; priority 79.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 79.0; priority 80.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Buy Watchlist, score 79.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.3%.</t>
+          <t>EIMI.MI: scenario base Buy Watchlist, score 79.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2844,13 +2844,13 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>16.2</v>
+        <v>14.47</v>
       </c>
       <c r="Z11" t="n">
-        <v>43</v>
+        <v>40.87</v>
       </c>
       <c r="AA11" t="n">
-        <v>16.01</v>
+        <v>15.98</v>
       </c>
       <c r="AB11" t="n">
         <v>-19.17</v>
@@ -2868,50 +2868,50 @@
         </is>
       </c>
       <c r="AG11" t="n">
-        <v>47.305</v>
+        <v>46.6</v>
       </c>
       <c r="AH11" t="n">
-        <v>69</v>
+        <v>68.5</v>
       </c>
       <c r="AI11" t="n">
-        <v>98.40000000000001</v>
+        <v>94.3</v>
       </c>
       <c r="AJ11" t="n">
         <v>65.5</v>
       </c>
       <c r="AK11" t="n">
-        <v>77.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.2</v>
+        <v>-1.29</v>
       </c>
       <c r="AM11" t="n">
-        <v>24.96</v>
+        <v>23.1</v>
       </c>
       <c r="AN11" t="n">
-        <v>18.61</v>
+        <v>18.02</v>
       </c>
       <c r="AO11" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="AP11" t="n">
-        <v>44.9277</v>
+        <v>44.9136</v>
       </c>
       <c r="AQ11" t="n">
-        <v>40.3702</v>
+        <v>40.3666</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>98.40000000000001</v>
+        <v>94.3</v>
       </c>
       <c r="AU11" t="n">
         <v>65.5</v>
       </c>
       <c r="AV11" t="n">
-        <v>77.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AW11" t="n">
         <v>756</v>
@@ -2923,10 +2923,10 @@
         <v>49.485</v>
       </c>
       <c r="AZ11" t="n">
-        <v>5.29</v>
+        <v>3.75</v>
       </c>
       <c r="BA11" t="n">
-        <v>17.18</v>
+        <v>15.44</v>
       </c>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
@@ -2947,69 +2947,73 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3. Interessanti ma da attendere</t>
+          <t>4. Alert / monitoraggio</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>XDEV.MI</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E12" t="n">
-        <v>79.2</v>
+        <v>80.2</v>
       </c>
       <c r="F12" t="n">
-        <v>65.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>🟠 Attendi pullback</t>
+          <t>🟡 Metti alert / monitora</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Non inseguire il prezzo: imposta alert su pullback o tenuta supporto. Supporto 60D: 54.81.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 402.3797. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>score 79.2; priority 65.5; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Normal risk</t>
+          <t>score 80.2; priority 77.9; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Extended - wait pullback</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>prezzo 11.7% sopra MA50: evitare inseguimento</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Accumulate Carefully, score 79.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.7%.</t>
+          <t>GOOGL: scenario base Buy Watchlist, score 80.2, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.6%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 72.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 402.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 54.81 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 273.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -3019,7 +3023,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Buy Watchlist</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -3028,83 +3032,71 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>54.81</v>
+        <v>273.3367</v>
       </c>
       <c r="T12" t="n">
-        <v>72.27</v>
-      </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
+        <v>402.3797</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Monitorare ingresso graduale</t>
+          <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>28.08</v>
+        <v>18.42</v>
       </c>
       <c r="Z12" t="n">
-        <v>62.01</v>
+        <v>110.08</v>
       </c>
       <c r="AA12" t="n">
-        <v>13.61</v>
+        <v>29.71</v>
       </c>
       <c r="AB12" t="n">
-        <v>-17.8</v>
-      </c>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
+        <v>-29.81</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>25.13</v>
+      </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>ETF interessante ma ingresso non ideale: meglio attendere pullback o conferma.</t>
-        </is>
-      </c>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t>Value globale</t>
-        </is>
-      </c>
+          <t>Titolo forte; resta necessario controllare prezzo, trimestrali e size.</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="n">
-        <v>70.93000000000001</v>
-      </c>
-      <c r="AH12" t="n">
-        <v>79.09999999999999</v>
-      </c>
-      <c r="AI12" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>69.40000000000001</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>51.8</v>
-      </c>
+        <v>363.385</v>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="n">
-        <v>6.97</v>
+        <v>-9.279999999999999</v>
       </c>
       <c r="AM12" t="n">
-        <v>38.43</v>
+        <v>13.33</v>
       </c>
       <c r="AN12" t="n">
-        <v>25.9</v>
+        <v>44.5</v>
       </c>
       <c r="AO12" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="AP12" t="n">
-        <v>63.482</v>
+        <v>357.7259</v>
       </c>
       <c r="AQ12" t="n">
-        <v>54.8732</v>
+        <v>305.2903</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
@@ -3114,41 +3106,75 @@
         <v>100</v>
       </c>
       <c r="AU12" t="n">
-        <v>69.40000000000001</v>
+        <v>40.5</v>
       </c>
       <c r="AV12" t="n">
-        <v>51.8</v>
+        <v>82.8</v>
       </c>
       <c r="AW12" t="n">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="AX12" t="n">
-        <v>65.27</v>
+        <v>358.7757</v>
       </c>
       <c r="AY12" t="n">
-        <v>72.27</v>
+        <v>402.3797</v>
       </c>
       <c r="AZ12" t="n">
-        <v>11.73</v>
+        <v>1.58</v>
       </c>
       <c r="BA12" t="n">
-        <v>29.26</v>
-      </c>
-      <c r="BB12" t="inlineStr"/>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="inlineStr"/>
-      <c r="BG12" t="inlineStr"/>
-      <c r="BH12" t="inlineStr"/>
-      <c r="BI12" t="inlineStr"/>
-      <c r="BJ12" t="inlineStr"/>
-      <c r="BK12" t="inlineStr"/>
-      <c r="BL12" t="inlineStr"/>
-      <c r="BM12" t="inlineStr"/>
-      <c r="BN12" t="inlineStr"/>
+        <v>19.03</v>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+      <c r="BD12" t="n">
+        <v>4431456239616</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>37.92</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>38.88</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>24</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>100</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>82.8</v>
+      </c>
       <c r="BO12" t="inlineStr"/>
-      <c r="BP12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr">
+        <is>
+          <t>USA / Internet</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3158,24 +3184,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>VWCE.DE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Alphabet Inc.</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>80.2</v>
+        <v>75.8</v>
       </c>
       <c r="F13" t="n">
-        <v>77.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3184,22 +3206,22 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 402.3797. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 164.88. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 80.2; priority 77.9; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 75.8; priority 76.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -3209,17 +3231,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Buy Watchlist, score 80.2, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.1%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 75.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.3%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 402.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 164.88 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 273.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 140.98 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -3229,7 +3251,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Buy Watchlist</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -3238,149 +3260,127 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>273.3367</v>
+        <v>140.98</v>
       </c>
       <c r="T13" t="n">
-        <v>402.3797</v>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Alphabet Inc.</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
+        <v>164.88</v>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Priorità watchlist</t>
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>18.66</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="Z13" t="n">
-        <v>116.86</v>
+        <v>23.31</v>
       </c>
       <c r="AA13" t="n">
-        <v>29.73</v>
+        <v>12.87</v>
       </c>
       <c r="AB13" t="n">
-        <v>-29.81</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>27.69</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>25.12</v>
-      </c>
+        <v>-21.07</v>
+      </c>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Titolo forte; resta necessario controllare prezzo, trimestrali e size.</t>
-        </is>
-      </c>
-      <c r="AF13" t="inlineStr"/>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Azionario globale</t>
+        </is>
+      </c>
       <c r="AG13" t="n">
-        <v>363.31</v>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+        <v>160.52</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>82.8</v>
+      </c>
       <c r="AL13" t="n">
-        <v>-8.66</v>
+        <v>1.2</v>
       </c>
       <c r="AM13" t="n">
-        <v>14.61</v>
+        <v>11.27</v>
       </c>
       <c r="AN13" t="n">
-        <v>44.56</v>
+        <v>16.92</v>
       </c>
       <c r="AO13" t="n">
-        <v>1.5</v>
+        <v>1.31</v>
       </c>
       <c r="AP13" t="n">
-        <v>355.9417</v>
+        <v>155.4036</v>
       </c>
       <c r="AQ13" t="n">
-        <v>304.4693</v>
+        <v>146.7588</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>100</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AU13" t="n">
-        <v>40.5</v>
+        <v>67.7</v>
       </c>
       <c r="AV13" t="n">
         <v>82.8</v>
       </c>
       <c r="AW13" t="n">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="AX13" t="n">
-        <v>358.7757</v>
+        <v>158.2</v>
       </c>
       <c r="AY13" t="n">
-        <v>402.3797</v>
+        <v>164.88</v>
       </c>
       <c r="AZ13" t="n">
-        <v>2.07</v>
+        <v>3.29</v>
       </c>
       <c r="BA13" t="n">
-        <v>19.33</v>
-      </c>
-      <c r="BB13" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="BC13" t="inlineStr">
-        <is>
-          <t>Internet Content &amp; Information</t>
-        </is>
-      </c>
-      <c r="BD13" t="n">
-        <v>4430541881344</v>
-      </c>
-      <c r="BE13" t="n">
-        <v>37.92</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>38.88</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>20.03</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>24</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>100</v>
-      </c>
-      <c r="BL13" t="n">
-        <v>60.1</v>
-      </c>
-      <c r="BM13" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="BN13" t="n">
-        <v>82.8</v>
-      </c>
+        <v>9.380000000000001</v>
+      </c>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
       <c r="BO13" t="inlineStr"/>
-      <c r="BP13" t="inlineStr">
-        <is>
-          <t>USA / Internet</t>
-        </is>
-      </c>
+      <c r="BP13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3390,20 +3390,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VWCE.DE</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>76.40000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>76.90000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3412,12 +3412,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 164.88. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 124.27. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 76.4; priority 76.9; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.9; priority 75.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3437,17 +3437,17 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.0%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 74.9, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.2%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 164.88 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 124.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 140.98 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 107.50 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -3466,15 +3466,15 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>140.98</v>
+        <v>107.5</v>
       </c>
       <c r="T14" t="n">
-        <v>164.88</v>
+        <v>124.27</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -3488,16 +3488,16 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>10.46</v>
+        <v>9.15</v>
       </c>
       <c r="Z14" t="n">
-        <v>24.23</v>
+        <v>21.51</v>
       </c>
       <c r="AA14" t="n">
-        <v>12.86</v>
+        <v>13.14</v>
       </c>
       <c r="AB14" t="n">
-        <v>-21.07</v>
+        <v>-21.63</v>
       </c>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
@@ -3508,69 +3508,69 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>Azionario globale</t>
+          <t>Azionario globale sviluppato</t>
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>161.72</v>
+        <v>121.72</v>
       </c>
       <c r="AH14" t="n">
-        <v>72.90000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AI14" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="AJ14" t="n">
-        <v>67.7</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AK14" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>1.95</v>
+        <v>1.48</v>
       </c>
       <c r="AM14" t="n">
-        <v>12.1</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.21</v>
+        <v>16.87</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.34</v>
+        <v>1.28</v>
       </c>
       <c r="AP14" t="n">
-        <v>155.4276</v>
+        <v>117.9644</v>
       </c>
       <c r="AQ14" t="n">
-        <v>146.7648</v>
+        <v>112.1964</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="AU14" t="n">
-        <v>67.7</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AV14" t="n">
-        <v>82.59999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AW14" t="n">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="AX14" t="n">
-        <v>158.2</v>
+        <v>120.3</v>
       </c>
       <c r="AY14" t="n">
-        <v>164.88</v>
+        <v>124.27</v>
       </c>
       <c r="AZ14" t="n">
-        <v>4.05</v>
+        <v>3.18</v>
       </c>
       <c r="BA14" t="n">
-        <v>10.19</v>
+        <v>8.49</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3596,21 +3596,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>SXR8.DE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="F15" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="F15" t="n">
-        <v>76</v>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>🟡 Metti alert / monitora</t>
@@ -3618,12 +3618,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 124.27. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 703.94. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 75.4; priority 76.0; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.7; priority 75.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3643,17 +3643,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 124.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 703.94 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 107.50 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 597.92 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3672,15 +3672,15 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>107.5</v>
+        <v>597.92</v>
       </c>
       <c r="T15" t="n">
-        <v>124.27</v>
+        <v>703.9400000000001</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -3694,16 +3694,16 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>9.85</v>
+        <v>10.53</v>
       </c>
       <c r="Z15" t="n">
-        <v>22.29</v>
+        <v>22.81</v>
       </c>
       <c r="AA15" t="n">
-        <v>13.13</v>
+        <v>14.1</v>
       </c>
       <c r="AB15" t="n">
-        <v>-21.63</v>
+        <v>-23.32</v>
       </c>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -3714,69 +3714,69 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Azionario globale sviluppato</t>
+          <t>USA large cap</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>122.5</v>
+        <v>687.92</v>
       </c>
       <c r="AH15" t="n">
-        <v>71.8</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AI15" t="n">
-        <v>75.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AJ15" t="n">
-        <v>66.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AK15" t="n">
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>2.13</v>
+        <v>1.6</v>
       </c>
       <c r="AM15" t="n">
-        <v>10.32</v>
+        <v>9.42</v>
       </c>
       <c r="AN15" t="n">
-        <v>17.12</v>
+        <v>18.13</v>
       </c>
       <c r="AO15" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="AP15" t="n">
-        <v>117.98</v>
+        <v>662.5776</v>
       </c>
       <c r="AQ15" t="n">
-        <v>112.2003</v>
+        <v>629.972</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>75.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AU15" t="n">
-        <v>66.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AV15" t="n">
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="AX15" t="n">
-        <v>120.3</v>
+        <v>680.66</v>
       </c>
       <c r="AY15" t="n">
-        <v>124.27</v>
+        <v>703.9400000000001</v>
       </c>
       <c r="AZ15" t="n">
-        <v>3.83</v>
+        <v>3.82</v>
       </c>
       <c r="BA15" t="n">
-        <v>9.18</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3812,10 +3812,10 @@
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>74.5</v>
+        <v>74.3</v>
       </c>
       <c r="F16" t="n">
-        <v>75.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 74.5; priority 75.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.3; priority 75.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.5%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.2%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -3900,10 +3900,10 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="Z16" t="n">
-        <v>15.8</v>
+        <v>15.47</v>
       </c>
       <c r="AA16" t="n">
         <v>12.85</v>
@@ -3924,13 +3924,13 @@
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>62.85</v>
+        <v>62.67</v>
       </c>
       <c r="AH16" t="n">
         <v>70.09999999999999</v>
       </c>
       <c r="AI16" t="n">
-        <v>69.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AJ16" t="n">
         <v>71.5</v>
@@ -3939,29 +3939,29 @@
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>2.39</v>
+        <v>2.1</v>
       </c>
       <c r="AM16" t="n">
-        <v>10.5</v>
+        <v>10.18</v>
       </c>
       <c r="AN16" t="n">
-        <v>13.81</v>
+        <v>13.7</v>
       </c>
       <c r="AO16" t="n">
         <v>1.07</v>
       </c>
       <c r="AP16" t="n">
-        <v>61.3448</v>
+        <v>61.3412</v>
       </c>
       <c r="AQ16" t="n">
-        <v>58.5815</v>
+        <v>58.5806</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>69.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AU16" t="n">
         <v>71.5</v>
@@ -3979,10 +3979,10 @@
         <v>63.94</v>
       </c>
       <c r="AZ16" t="n">
-        <v>2.45</v>
+        <v>2.17</v>
       </c>
       <c r="BA16" t="n">
-        <v>7.29</v>
+        <v>6.98</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -4008,20 +4008,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SXR8.DE</t>
+          <t>IWQU.MI</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>74.8</v>
+        <v>72.5</v>
       </c>
       <c r="F17" t="n">
-        <v>75.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4030,12 +4030,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 703.94. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 74.96. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 74.8; priority 75.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.5; priority 74.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4055,17 +4055,17 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.4%.</t>
+          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.0%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 703.94 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 74.96 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 597.92 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 66.58 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4084,38 +4084,38 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>597.92</v>
+        <v>66.58</v>
       </c>
       <c r="T17" t="n">
-        <v>703.9400000000001</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Factor</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>11.16</v>
+        <v>7.16</v>
       </c>
       <c r="Z17" t="n">
-        <v>23.52</v>
+        <v>17.75</v>
       </c>
       <c r="AA17" t="n">
-        <v>14.09</v>
+        <v>12.87</v>
       </c>
       <c r="AB17" t="n">
-        <v>-23.32</v>
+        <v>-20.6</v>
       </c>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -4126,69 +4126,69 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>USA large cap</t>
+          <t>Quality globale</t>
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>691.88</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AH17" t="n">
-        <v>70.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="AI17" t="n">
-        <v>77.5</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AJ17" t="n">
-        <v>64.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>81.09999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AL17" t="n">
-        <v>2.19</v>
+        <v>2.33</v>
       </c>
       <c r="AM17" t="n">
-        <v>10.05</v>
+        <v>9.42</v>
       </c>
       <c r="AN17" t="n">
-        <v>18.36</v>
+        <v>14.94</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.3</v>
+        <v>1.16</v>
       </c>
       <c r="AP17" t="n">
-        <v>662.6568</v>
+        <v>71.9044</v>
       </c>
       <c r="AQ17" t="n">
-        <v>629.9918</v>
+        <v>68.7041</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>85</v>
       </c>
       <c r="AT17" t="n">
-        <v>77.5</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AU17" t="n">
-        <v>64.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>81.09999999999999</v>
+        <v>82.8</v>
       </c>
       <c r="AW17" t="n">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="AX17" t="n">
-        <v>680.66</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AY17" t="n">
-        <v>703.9400000000001</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="AZ17" t="n">
-        <v>4.41</v>
+        <v>3.05</v>
       </c>
       <c r="BA17" t="n">
-        <v>9.82</v>
+        <v>7.85</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4214,20 +4214,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IWQU.MI</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E18" t="n">
-        <v>72.8</v>
+        <v>73</v>
       </c>
       <c r="F18" t="n">
-        <v>74.3</v>
+        <v>72.2</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4236,42 +4240,42 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 74.96. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 315.2. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 72.8; priority 74.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.0; priority 72.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Constructive entry zone</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.4%.</t>
+          <t>AAPL: scenario base Accumulate Carefully, score 73.0, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.6%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 74.96 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 315.20 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 66.58 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 246.40 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -4290,127 +4294,149 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>66.58</v>
+        <v>246.403</v>
       </c>
       <c r="T18" t="n">
-        <v>74.95999999999999</v>
-      </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
+        <v>315.2</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Monitorare ingresso graduale</t>
+          <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>7.49</v>
+        <v>12.55</v>
       </c>
       <c r="Z18" t="n">
-        <v>18.12</v>
+        <v>44.39</v>
       </c>
       <c r="AA18" t="n">
-        <v>12.86</v>
+        <v>25.94</v>
       </c>
       <c r="AB18" t="n">
-        <v>-20.6</v>
-      </c>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
+        <v>-33.36</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>35.51</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>30.52</v>
+      </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
-        </is>
-      </c>
-      <c r="AF18" t="inlineStr">
-        <is>
-          <t>Quality globale</t>
-        </is>
-      </c>
+          <t>Business/momentum interessanti ma valutazione tirata: non inseguire senza pullback.</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="n">
-        <v>74.33</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>65</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>70.90000000000001</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>68.09999999999999</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>82.8</v>
-      </c>
+        <v>293.285</v>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
-        <v>2.65</v>
+        <v>0.08</v>
       </c>
       <c r="AM18" t="n">
-        <v>9.76</v>
+        <v>5.4</v>
       </c>
       <c r="AN18" t="n">
-        <v>15.06</v>
+        <v>18.11</v>
       </c>
       <c r="AO18" t="n">
-        <v>1.17</v>
+        <v>0.7</v>
       </c>
       <c r="AP18" t="n">
-        <v>71.90900000000001</v>
+        <v>282.9571</v>
       </c>
       <c r="AQ18" t="n">
-        <v>68.70529999999999</v>
+        <v>265.4899</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>85</v>
       </c>
       <c r="AT18" t="n">
-        <v>70.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="AU18" t="n">
-        <v>68.09999999999999</v>
+        <v>42.2</v>
       </c>
       <c r="AV18" t="n">
         <v>82.8</v>
       </c>
       <c r="AW18" t="n">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="AX18" t="n">
-        <v>72.59999999999999</v>
+        <v>293.285</v>
       </c>
       <c r="AY18" t="n">
-        <v>74.95999999999999</v>
+        <v>315.2</v>
       </c>
       <c r="AZ18" t="n">
-        <v>3.37</v>
+        <v>3.65</v>
       </c>
       <c r="BA18" t="n">
-        <v>8.19</v>
-      </c>
-      <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
-      <c r="BE18" t="inlineStr"/>
-      <c r="BF18" t="inlineStr"/>
-      <c r="BG18" t="inlineStr"/>
-      <c r="BH18" t="inlineStr"/>
-      <c r="BI18" t="inlineStr"/>
-      <c r="BJ18" t="inlineStr"/>
-      <c r="BK18" t="inlineStr"/>
-      <c r="BL18" t="inlineStr"/>
-      <c r="BM18" t="inlineStr"/>
-      <c r="BN18" t="inlineStr"/>
+        <v>10.47</v>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>Consumer Electronics</t>
+        </is>
+      </c>
+      <c r="BD18" t="n">
+        <v>4307581140992</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>27.15</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>141.47</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>79.55</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>36</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="BN18" t="n">
+        <v>82.8</v>
+      </c>
       <c r="BO18" t="inlineStr"/>
-      <c r="BP18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr">
+        <is>
+          <t>USA / Technology</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4420,24 +4446,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>XDEV.MI</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>73.40000000000001</v>
+        <v>80</v>
       </c>
       <c r="F19" t="n">
-        <v>70.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4446,12 +4468,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 315.2. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 72.27. Trigger: prezzo 10.0% sopra MA50: evitare inseguimento.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>score 73.4; priority 70.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 80.0; priority 70.7; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4461,27 +4483,27 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 10.0% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>AAPL: scenario base Accumulate Carefully, score 73.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 6.9%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 80.0, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 10.0%.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 315.20 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 72.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 246.40 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 54.81 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -4491,7 +4513,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Buy Watchlist</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -4500,149 +4522,127 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>246.403</v>
+        <v>54.81</v>
       </c>
       <c r="T19" t="n">
-        <v>315.2</v>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Apple Inc.</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
+        <v>72.27</v>
+      </c>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Xtrackers MSCI World Value UCITS ETF 1C</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y19" t="n">
-        <v>16.14</v>
+        <v>26.04</v>
       </c>
       <c r="Z19" t="n">
-        <v>50.89</v>
+        <v>59.43</v>
       </c>
       <c r="AA19" t="n">
-        <v>25.91</v>
+        <v>13.62</v>
       </c>
       <c r="AB19" t="n">
-        <v>-33.36</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>36.51</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>31.38</v>
-      </c>
+        <v>-17.8</v>
+      </c>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>Business/momentum interessanti ma valutazione tirata: non inseguire senza pullback.</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr"/>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Value globale</t>
+        </is>
+      </c>
       <c r="AG19" t="n">
-        <v>301.54</v>
-      </c>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
+        <v>69.8</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>58.8</v>
+      </c>
       <c r="AL19" t="n">
-        <v>5</v>
+        <v>5.26</v>
       </c>
       <c r="AM19" t="n">
-        <v>7.62</v>
+        <v>36.22</v>
       </c>
       <c r="AN19" t="n">
-        <v>19.25</v>
+        <v>25.23</v>
       </c>
       <c r="AO19" t="n">
-        <v>0.74</v>
+        <v>1.85</v>
       </c>
       <c r="AP19" t="n">
-        <v>282.0628</v>
+        <v>63.4594</v>
       </c>
       <c r="AQ19" t="n">
-        <v>265.1448</v>
+        <v>54.8676</v>
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="n">
         <v>85</v>
       </c>
       <c r="AT19" t="n">
-        <v>89.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="AU19" t="n">
-        <v>42.2</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AV19" t="n">
-        <v>71.09999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="AW19" t="n">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="AX19" t="n">
-        <v>292.68</v>
+        <v>65.27</v>
       </c>
       <c r="AY19" t="n">
-        <v>315.2</v>
+        <v>72.27</v>
       </c>
       <c r="AZ19" t="n">
-        <v>6.91</v>
+        <v>9.99</v>
       </c>
       <c r="BA19" t="n">
-        <v>13.73</v>
-      </c>
-      <c r="BB19" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC19" t="inlineStr">
-        <is>
-          <t>Consumer Electronics</t>
-        </is>
-      </c>
-      <c r="BD19" t="n">
-        <v>4428825362432</v>
-      </c>
-      <c r="BE19" t="n">
-        <v>27.15</v>
-      </c>
-      <c r="BF19" t="n">
-        <v>141.47</v>
-      </c>
-      <c r="BG19" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="BH19" t="n">
-        <v>79.55</v>
-      </c>
-      <c r="BI19" t="n">
-        <v>36</v>
-      </c>
-      <c r="BJ19" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK19" t="n">
-        <v>89.90000000000001</v>
-      </c>
-      <c r="BL19" t="n">
-        <v>41</v>
-      </c>
-      <c r="BM19" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="BN19" t="n">
-        <v>71.09999999999999</v>
-      </c>
+        <v>27.22</v>
+      </c>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
       <c r="BO19" t="inlineStr"/>
-      <c r="BP19" t="inlineStr">
-        <is>
-          <t>USA / Technology</t>
-        </is>
-      </c>
+      <c r="BP19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4662,10 +4662,10 @@
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>68.2</v>
+        <v>68.3</v>
       </c>
       <c r="F20" t="n">
-        <v>70.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 68.2; priority 70.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 68.3; priority 70.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 68.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 68.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.8%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -4750,13 +4750,13 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>-1.95</v>
+        <v>-1.77</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.28</v>
+        <v>0.47</v>
       </c>
       <c r="AA20" t="n">
-        <v>9.56</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AB20" t="n">
         <v>-12.85</v>
@@ -4774,13 +4774,13 @@
         </is>
       </c>
       <c r="AG20" t="n">
-        <v>63.74</v>
+        <v>63.86</v>
       </c>
       <c r="AH20" t="n">
         <v>61.3</v>
       </c>
       <c r="AI20" t="n">
-        <v>48.2</v>
+        <v>48.7</v>
       </c>
       <c r="AJ20" t="n">
         <v>78.3</v>
@@ -4789,29 +4789,29 @@
         <v>82.8</v>
       </c>
       <c r="AL20" t="n">
-        <v>2.71</v>
+        <v>2.9</v>
       </c>
       <c r="AM20" t="n">
-        <v>1.51</v>
+        <v>1.7</v>
       </c>
       <c r="AN20" t="n">
-        <v>6.57</v>
+        <v>6.64</v>
       </c>
       <c r="AO20" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="AP20" t="n">
-        <v>63.3206</v>
+        <v>63.323</v>
       </c>
       <c r="AQ20" t="n">
-        <v>63.1004</v>
+        <v>63.101</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>85</v>
       </c>
       <c r="AT20" t="n">
-        <v>48.2</v>
+        <v>48.7</v>
       </c>
       <c r="AU20" t="n">
         <v>78.3</v>
@@ -4829,10 +4829,10 @@
         <v>64.68000000000001</v>
       </c>
       <c r="AZ20" t="n">
-        <v>0.66</v>
+        <v>0.85</v>
       </c>
       <c r="BA20" t="n">
-        <v>1.01</v>
+        <v>1.2</v>
       </c>
       <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="inlineStr"/>
@@ -4872,10 +4872,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>74.8</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>58.1</v>
+        <v>56.7</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 74.8; priority 58.1; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 73.6; priority 56.7; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.3%.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 73.6, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.6%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4956,22 +4956,22 @@
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>14.37</v>
+        <v>11.59</v>
       </c>
       <c r="Z21" t="n">
-        <v>49.25</v>
+        <v>45.52</v>
       </c>
       <c r="AA21" t="n">
-        <v>46.98</v>
+        <v>46.96</v>
       </c>
       <c r="AB21" t="n">
         <v>-36.88</v>
       </c>
       <c r="AC21" t="n">
-        <v>31.95</v>
+        <v>31.54</v>
       </c>
       <c r="AD21" t="n">
-        <v>16.45</v>
+        <v>16.24</v>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
@@ -4980,36 +4980,36 @@
       </c>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="n">
-        <v>208.64</v>
+        <v>205.94</v>
       </c>
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="n">
-        <v>-1.24</v>
+        <v>-4.19</v>
       </c>
       <c r="AM21" t="n">
-        <v>13.91</v>
+        <v>13.04</v>
       </c>
       <c r="AN21" t="n">
-        <v>76.01000000000001</v>
+        <v>75.11</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.62</v>
+        <v>1.6</v>
       </c>
       <c r="AP21" t="n">
-        <v>203.972</v>
+        <v>204.7443</v>
       </c>
       <c r="AQ21" t="n">
-        <v>188.512</v>
+        <v>188.668</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
         <v>85</v>
       </c>
       <c r="AT21" t="n">
-        <v>90.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="AU21" t="n">
         <v>14.1</v>
@@ -5018,7 +5018,7 @@
         <v>82.8</v>
       </c>
       <c r="AW21" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX21" t="n">
         <v>205.1</v>
@@ -5027,10 +5027,10 @@
         <v>235.4656</v>
       </c>
       <c r="AZ21" t="n">
-        <v>2.29</v>
+        <v>0.57</v>
       </c>
       <c r="BA21" t="n">
-        <v>10.68</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BB21" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         </is>
       </c>
       <c r="BD21" t="n">
-        <v>5053469425664</v>
+        <v>4988072886272</v>
       </c>
       <c r="BE21" t="n">
         <v>62.97</v>
@@ -5064,10 +5064,10 @@
         <v>100</v>
       </c>
       <c r="BK21" t="n">
-        <v>90.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="BL21" t="n">
-        <v>67.59999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="BM21" t="n">
         <v>14.1</v>
@@ -5100,10 +5100,10 @@
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>55.6</v>
+        <v>54.5</v>
       </c>
       <c r="F22" t="n">
-        <v>57.4</v>
+        <v>56.1</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 55.6; priority 57.4; trend: Weak; entry zone: Wait for trend repair; risk flag: Normal risk</t>
+          <t>score 54.5; priority 56.1; trend: Weak; entry zone: Wait for trend repair; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -5132,12 +5132,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>prezzo 5.2% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 6.1% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 55.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -5.2%.</t>
+          <t>SGLD.MI: scenario base Avoid for Now, score 54.5, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -6.1%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 360.85 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 357.35 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="S22" t="n">
-        <v>360.85</v>
+        <v>357.35</v>
       </c>
       <c r="T22" t="n">
         <v>424.57</v>
@@ -5184,20 +5184,20 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Osservare</t>
+          <t>Evitare per ora</t>
         </is>
       </c>
       <c r="Y22" t="n">
-        <v>-14.8</v>
+        <v>-15.63</v>
       </c>
       <c r="Z22" t="n">
-        <v>27.66</v>
+        <v>26.42</v>
       </c>
       <c r="AA22" t="n">
-        <v>17.78</v>
+        <v>17.79</v>
       </c>
       <c r="AB22" t="n">
-        <v>-17.31</v>
+        <v>-18.11</v>
       </c>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr"/>
@@ -5212,65 +5212,65 @@
         </is>
       </c>
       <c r="AG22" t="n">
-        <v>360.85</v>
+        <v>357.35</v>
       </c>
       <c r="AH22" t="n">
-        <v>70.59999999999999</v>
+        <v>69.7</v>
       </c>
       <c r="AI22" t="n">
-        <v>38.6</v>
+        <v>36.5</v>
       </c>
       <c r="AJ22" t="n">
-        <v>64.8</v>
+        <v>64.2</v>
       </c>
       <c r="AK22" t="n">
-        <v>67.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="AL22" t="n">
-        <v>-6.65</v>
+        <v>-7.55</v>
       </c>
       <c r="AM22" t="n">
-        <v>4.01</v>
+        <v>3</v>
       </c>
       <c r="AN22" t="n">
-        <v>26.97</v>
+        <v>26.56</v>
       </c>
       <c r="AO22" t="n">
-        <v>1.52</v>
+        <v>1.49</v>
       </c>
       <c r="AP22" t="n">
-        <v>380.8024</v>
+        <v>380.7324</v>
       </c>
       <c r="AQ22" t="n">
-        <v>362.1715</v>
+        <v>362.154</v>
       </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
         <v>35</v>
       </c>
       <c r="AT22" t="n">
-        <v>38.6</v>
+        <v>36.5</v>
       </c>
       <c r="AU22" t="n">
-        <v>64.8</v>
+        <v>64.2</v>
       </c>
       <c r="AV22" t="n">
-        <v>67.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="AW22" t="n">
         <v>756</v>
       </c>
       <c r="AX22" t="n">
-        <v>360.85</v>
+        <v>357.35</v>
       </c>
       <c r="AY22" t="n">
         <v>386.38</v>
       </c>
       <c r="AZ22" t="n">
-        <v>-5.24</v>
+        <v>-6.14</v>
       </c>
       <c r="BA22" t="n">
-        <v>-0.36</v>
+        <v>-1.33</v>
       </c>
       <c r="BB22" t="inlineStr"/>
       <c r="BC22" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v7_sector_compass_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -776,10 +776,10 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>67.09999999999999</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>70.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 67.1; priority 70.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 68.1; priority 71.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Hold / Monitor, score 67.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.4%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.3%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>2.55</v>
+        <v>3.69</v>
       </c>
       <c r="Z2" t="n">
-        <v>40.66</v>
+        <v>42.56</v>
       </c>
       <c r="AA2" t="n">
-        <v>22.4</v>
+        <v>22.44</v>
       </c>
       <c r="AB2" t="n">
         <v>-29.37</v>
@@ -888,13 +888,13 @@
         </is>
       </c>
       <c r="AG2" t="n">
-        <v>18.32</v>
+        <v>18.652</v>
       </c>
       <c r="AH2" t="n">
-        <v>52.3</v>
+        <v>52.1</v>
       </c>
       <c r="AI2" t="n">
-        <v>79.59999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="AJ2" t="n">
         <v>44.6</v>
@@ -903,29 +903,29 @@
         <v>82.8</v>
       </c>
       <c r="AL2" t="n">
-        <v>6.66</v>
+        <v>7.47</v>
       </c>
       <c r="AM2" t="n">
-        <v>26.43</v>
+        <v>30.18</v>
       </c>
       <c r="AN2" t="n">
-        <v>20.67</v>
+        <v>20.4</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.2427</v>
+        <v>18.2371</v>
       </c>
       <c r="AQ2" t="n">
-        <v>15.7421</v>
+        <v>15.789</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>79.59999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="AU2" t="n">
         <v>49.6</v>
@@ -934,19 +934,19 @@
         <v>82.8</v>
       </c>
       <c r="AW2" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX2" t="n">
-        <v>17.356</v>
+        <v>17.914</v>
       </c>
       <c r="AY2" t="n">
         <v>19.25</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.42</v>
+        <v>2.28</v>
       </c>
       <c r="BA2" t="n">
-        <v>16.38</v>
+        <v>18.13</v>
       </c>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
@@ -1082,7 +1082,7 @@
         <v>-30.88</v>
       </c>
       <c r="AC3" t="n">
-        <v>21.43</v>
+        <v>21.42</v>
       </c>
       <c r="AD3" t="n">
         <v>25.64</v>
@@ -1219,7 +1219,7 @@
         <v>67.7</v>
       </c>
       <c r="F4" t="n">
-        <v>54.6</v>
+        <v>54.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 67.7; priority 54.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 67.7; priority 54.5; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 67.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.6%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 67.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.8%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1300,22 +1300,22 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>6.76</v>
+        <v>1.31</v>
       </c>
       <c r="Z4" t="n">
-        <v>135.2</v>
+        <v>141.23</v>
       </c>
       <c r="AA4" t="n">
-        <v>39.47</v>
+        <v>39.51</v>
       </c>
       <c r="AB4" t="n">
         <v>-44.77</v>
       </c>
       <c r="AC4" t="n">
-        <v>58.79</v>
+        <v>58.54</v>
       </c>
       <c r="AD4" t="n">
-        <v>28.91</v>
+        <v>28.62</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1324,29 +1324,29 @@
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>1486.4</v>
+        <v>1479.2</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>9.119999999999999</v>
+        <v>2.72</v>
       </c>
       <c r="AM4" t="n">
-        <v>20.92</v>
+        <v>22.63</v>
       </c>
       <c r="AN4" t="n">
-        <v>35.41</v>
+        <v>35.2</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="AP4" t="n">
-        <v>1541.8116</v>
+        <v>1538.2795</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1263.4068</v>
+        <v>1266.4162</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
@@ -1359,10 +1359,10 @@
         <v>16.8</v>
       </c>
       <c r="AV4" t="n">
-        <v>74.40000000000001</v>
+        <v>74</v>
       </c>
       <c r="AW4" t="n">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="AX4" t="n">
         <v>1419.6</v>
@@ -1371,10 +1371,10 @@
         <v>1621.2</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-3.59</v>
+        <v>-3.84</v>
       </c>
       <c r="BA4" t="n">
-        <v>17.65</v>
+        <v>16.8</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>573999022080</v>
+        <v>568160681984</v>
       </c>
       <c r="BE4" t="n">
         <v>30.11</v>
@@ -1411,13 +1411,13 @@
         <v>100</v>
       </c>
       <c r="BL4" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="BM4" t="n">
         <v>16.8</v>
       </c>
       <c r="BN4" t="n">
-        <v>74.40000000000001</v>
+        <v>74</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1750,7 +1750,7 @@
         <v>-34.15</v>
       </c>
       <c r="AC6" t="n">
-        <v>21.76</v>
+        <v>21.79</v>
       </c>
       <c r="AD6" t="n">
         <v>16.53</v>
@@ -1840,7 +1840,7 @@
         <v>43</v>
       </c>
       <c r="BI6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="BJ6" t="n">
         <v>100</v>
@@ -1872,20 +1872,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>WCLD.MI</t>
+          <t>INRG.MI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>55.3</v>
+        <v>35.7</v>
       </c>
       <c r="F7" t="n">
-        <v>36.8</v>
+        <v>29.5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1899,12 +1899,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 55.3; priority 36.8; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 35.7; priority 29.5; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Extended - wait pullback</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1914,22 +1914,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>prezzo 11.2% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 7.2% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base Hold / Monitor, score 55.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.2%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 35.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -7.2%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 34.72 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 10.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 8.59 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1939,24 +1939,24 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>24.785</v>
+        <v>8.593</v>
       </c>
       <c r="T7" t="n">
-        <v>34.715</v>
+        <v>10.872</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1970,16 +1970,16 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>23.6</v>
+        <v>-25.23</v>
       </c>
       <c r="Z7" t="n">
-        <v>16.7</v>
+        <v>22.91</v>
       </c>
       <c r="AA7" t="n">
-        <v>34.77</v>
+        <v>24.13</v>
       </c>
       <c r="AB7" t="n">
-        <v>-48.6</v>
+        <v>-35.07</v>
       </c>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -1990,69 +1990,69 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Energia pulita</t>
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>33.575</v>
+        <v>8.680999999999999</v>
       </c>
       <c r="AH7" t="n">
-        <v>26.3</v>
+        <v>33.6</v>
       </c>
       <c r="AI7" t="n">
-        <v>100</v>
+        <v>18.9</v>
       </c>
       <c r="AJ7" t="n">
-        <v>14.4</v>
+        <v>38</v>
       </c>
       <c r="AK7" t="n">
-        <v>54.1</v>
+        <v>64.5</v>
       </c>
       <c r="AL7" t="n">
-        <v>10.99</v>
+        <v>-1.39</v>
       </c>
       <c r="AM7" t="n">
-        <v>52.58</v>
+        <v>-2.46</v>
       </c>
       <c r="AN7" t="n">
-        <v>6.37</v>
+        <v>1.69</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.18</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AP7" t="n">
-        <v>30.2035</v>
+        <v>9.3507</v>
       </c>
       <c r="AQ7" t="n">
-        <v>26.9246</v>
+        <v>9.282</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="AT7" t="n">
-        <v>100</v>
+        <v>18.9</v>
       </c>
       <c r="AU7" t="n">
-        <v>19.4</v>
+        <v>43</v>
       </c>
       <c r="AV7" t="n">
-        <v>54.1</v>
+        <v>64.5</v>
       </c>
       <c r="AW7" t="n">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="AX7" t="n">
-        <v>29.525</v>
+        <v>8.613</v>
       </c>
       <c r="AY7" t="n">
-        <v>34.715</v>
+        <v>9.217000000000001</v>
       </c>
       <c r="AZ7" t="n">
-        <v>11.16</v>
+        <v>-7.16</v>
       </c>
       <c r="BA7" t="n">
-        <v>24.7</v>
+        <v>-6.47</v>
       </c>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
@@ -2078,20 +2078,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E8" t="n">
-        <v>34.6</v>
+        <v>29.8</v>
       </c>
       <c r="F8" t="n">
-        <v>28.3</v>
+        <v>21.1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2105,7 +2109,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 34.6; priority 28.3; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 29.8; priority 21.1; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2120,22 +2124,22 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>prezzo 7.9% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 34.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -7.9%.</t>
+          <t>TSLA: scenario base High Risk, score 29.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.2%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 11.25 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.59 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2145,7 +2149,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>High Risk</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -2154,127 +2158,147 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>8.593</v>
+        <v>298.32</v>
       </c>
       <c r="T8" t="n">
-        <v>11.252</v>
-      </c>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>425.3</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>-24.85</v>
+        <v>-19.97</v>
       </c>
       <c r="Z8" t="n">
-        <v>22.79</v>
+        <v>-0.24</v>
       </c>
       <c r="AA8" t="n">
-        <v>24.1</v>
+        <v>58.26</v>
       </c>
       <c r="AB8" t="n">
-        <v>-35.93</v>
-      </c>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
+        <v>-53.77</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>322.92</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>161.56</v>
+      </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>Energia pulita</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="n">
-        <v>8.68</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>33.1</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>63.4</v>
-      </c>
+        <v>348.75</v>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
-        <v>-0.45</v>
+        <v>12.92</v>
       </c>
       <c r="AM8" t="n">
-        <v>-7.26</v>
+        <v>-13.36</v>
       </c>
       <c r="AN8" t="n">
-        <v>1.49</v>
+        <v>10.73</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.06</v>
+        <v>0.18</v>
       </c>
       <c r="AP8" t="n">
-        <v>9.4244</v>
+        <v>360.4738</v>
       </c>
       <c r="AQ8" t="n">
-        <v>9.281000000000001</v>
+        <v>400.9283</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
         <v>35</v>
       </c>
       <c r="AT8" t="n">
-        <v>16.6</v>
+        <v>14</v>
       </c>
       <c r="AU8" t="n">
-        <v>42.3</v>
+        <v>0</v>
       </c>
       <c r="AV8" t="n">
-        <v>63.4</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AW8" t="n">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="AX8" t="n">
-        <v>8.613</v>
+        <v>319.53</v>
       </c>
       <c r="AY8" t="n">
-        <v>9.217000000000001</v>
+        <v>362.86</v>
       </c>
       <c r="AZ8" t="n">
-        <v>-7.9</v>
+        <v>-3.25</v>
       </c>
       <c r="BA8" t="n">
-        <v>-6.48</v>
-      </c>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
+        <v>-13.01</v>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+      <c r="BD8" t="n">
+        <v>1377404715008</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>18.37</v>
+      </c>
       <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="inlineStr"/>
+      <c r="BJ8" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>14</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>70.40000000000001</v>
+      </c>
       <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>USA / EV</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2284,24 +2308,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>WCLD.MI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>29.8</v>
+        <v>51.3</v>
       </c>
       <c r="F9" t="n">
-        <v>21.1</v>
+        <v>15.7</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2315,12 +2335,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 29.8; priority 21.1; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 51.3; priority 15.7; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Extended - wait pullback</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2330,22 +2350,22 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 18.1% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 29.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.2%.</t>
+          <t>WCLD.MI: scenario base High Risk, score 51.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.1%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 36.17 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -2360,151 +2380,131 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S9" t="n">
-        <v>298.32</v>
+        <v>24.785</v>
       </c>
       <c r="T9" t="n">
-        <v>425.3</v>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+        <v>36.175</v>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X9" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>-19.97</v>
+        <v>24.72</v>
       </c>
       <c r="Z9" t="n">
-        <v>-0.24</v>
+        <v>20.08</v>
       </c>
       <c r="AA9" t="n">
-        <v>58.26</v>
+        <v>35.03</v>
       </c>
       <c r="AB9" t="n">
-        <v>-53.77</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>329.01</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>161.56</v>
-      </c>
+        <v>-48.6</v>
+      </c>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
       <c r="AG9" t="n">
-        <v>348.75</v>
-      </c>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+        <v>36.175</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>26.5</v>
+      </c>
       <c r="AL9" t="n">
-        <v>12.92</v>
+        <v>22.52</v>
       </c>
       <c r="AM9" t="n">
-        <v>-13.36</v>
+        <v>61.17</v>
       </c>
       <c r="AN9" t="n">
-        <v>10.73</v>
+        <v>7.68</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="AP9" t="n">
-        <v>360.4738</v>
+        <v>30.6422</v>
       </c>
       <c r="AQ9" t="n">
-        <v>400.9283</v>
+        <v>26.9892</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="AT9" t="n">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="AU9" t="n">
-        <v>0</v>
+        <v>19.1</v>
       </c>
       <c r="AV9" t="n">
-        <v>70.40000000000001</v>
+        <v>26.5</v>
       </c>
       <c r="AW9" t="n">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="AX9" t="n">
-        <v>319.53</v>
+        <v>31.27</v>
       </c>
       <c r="AY9" t="n">
-        <v>362.86</v>
+        <v>36.175</v>
       </c>
       <c r="AZ9" t="n">
-        <v>-3.25</v>
+        <v>18.06</v>
       </c>
       <c r="BA9" t="n">
-        <v>-13.01</v>
-      </c>
-      <c r="BB9" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="BC9" t="inlineStr">
-        <is>
-          <t>Auto Manufacturers</t>
-        </is>
-      </c>
-      <c r="BD9" t="n">
-        <v>1377404715008</v>
-      </c>
-      <c r="BE9" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="BF9" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="BG9" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="BH9" t="n">
-        <v>18.37</v>
-      </c>
+        <v>34.04</v>
+      </c>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
-      <c r="BJ9" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>14</v>
-      </c>
-      <c r="BL9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN9" t="n">
-        <v>70.40000000000001</v>
-      </c>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
       <c r="BO9" t="inlineStr"/>
-      <c r="BP9" t="inlineStr">
-        <is>
-          <t>USA / EV</t>
-        </is>
-      </c>
+      <c r="BP9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2524,10 +2524,10 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>78.8</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>78.7</v>
+        <v>78.3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 78.8; priority 78.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 78.4; priority 78.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 78.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.2%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 78.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.7%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2612,13 +2612,13 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>2.16</v>
+        <v>0.8</v>
       </c>
       <c r="Z10" t="n">
-        <v>54.68</v>
+        <v>55.71</v>
       </c>
       <c r="AA10" t="n">
-        <v>14.12</v>
+        <v>14.13</v>
       </c>
       <c r="AB10" t="n">
         <v>-17.8</v>
@@ -2636,13 +2636,13 @@
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>72.48999999999999</v>
+        <v>72.84</v>
       </c>
       <c r="AH10" t="n">
-        <v>78.09999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AI10" t="n">
-        <v>81.2</v>
+        <v>80</v>
       </c>
       <c r="AJ10" t="n">
         <v>68.8</v>
@@ -2651,29 +2651,29 @@
         <v>82.8</v>
       </c>
       <c r="AL10" t="n">
-        <v>2.36</v>
+        <v>3.44</v>
       </c>
       <c r="AM10" t="n">
-        <v>24.23</v>
+        <v>24.96</v>
       </c>
       <c r="AN10" t="n">
-        <v>26.24</v>
+        <v>26.14</v>
       </c>
       <c r="AO10" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
       <c r="AP10" t="n">
-        <v>71.616</v>
+        <v>71.61960000000001</v>
       </c>
       <c r="AQ10" t="n">
-        <v>61.4335</v>
+        <v>61.657</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
         <v>85</v>
       </c>
       <c r="AT10" t="n">
-        <v>81.2</v>
+        <v>80</v>
       </c>
       <c r="AU10" t="n">
         <v>68.8</v>
@@ -2682,19 +2682,19 @@
         <v>82.8</v>
       </c>
       <c r="AW10" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX10" t="n">
-        <v>70.2</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="AY10" t="n">
         <v>73.75</v>
       </c>
       <c r="AZ10" t="n">
-        <v>1.22</v>
+        <v>1.7</v>
       </c>
       <c r="BA10" t="n">
-        <v>18</v>
+        <v>18.14</v>
       </c>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2830,7 +2830,7 @@
         <v>-34.5</v>
       </c>
       <c r="AC11" t="n">
-        <v>28.64</v>
+        <v>28.58</v>
       </c>
       <c r="AD11" t="n">
         <v>21.78</v>
@@ -2920,7 +2920,7 @@
         <v>29.12</v>
       </c>
       <c r="BI11" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="BJ11" t="n">
         <v>100</v>
@@ -2929,7 +2929,7 @@
         <v>89.3</v>
       </c>
       <c r="BL11" t="n">
-        <v>63.8</v>
+        <v>63.9</v>
       </c>
       <c r="BM11" t="n">
         <v>41</v>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.6%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.3%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -3050,13 +3050,13 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>5.49</v>
+        <v>5.15</v>
       </c>
       <c r="Z12" t="n">
-        <v>21.58</v>
+        <v>21.35</v>
       </c>
       <c r="AA12" t="n">
-        <v>12.74</v>
+        <v>12.75</v>
       </c>
       <c r="AB12" t="n">
         <v>-16.33</v>
@@ -3074,13 +3074,13 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>65.63</v>
+        <v>65.47</v>
       </c>
       <c r="AH12" t="n">
-        <v>73.40000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="AI12" t="n">
-        <v>66.59999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AJ12" t="n">
         <v>71.59999999999999</v>
@@ -3089,29 +3089,29 @@
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>1.77</v>
+        <v>1.02</v>
       </c>
       <c r="AM12" t="n">
-        <v>5.88</v>
+        <v>7.29</v>
       </c>
       <c r="AN12" t="n">
-        <v>15.97</v>
+        <v>15.78</v>
       </c>
       <c r="AO12" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="AP12" t="n">
-        <v>64.5716</v>
+        <v>64.6536</v>
       </c>
       <c r="AQ12" t="n">
-        <v>60.6324</v>
+        <v>60.7231</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>66.59999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AU12" t="n">
         <v>71.59999999999999</v>
@@ -3120,19 +3120,19 @@
         <v>82.8</v>
       </c>
       <c r="AW12" t="n">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="AX12" t="n">
-        <v>64.73</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="AY12" t="n">
         <v>65.95</v>
       </c>
       <c r="AZ12" t="n">
-        <v>1.64</v>
+        <v>1.26</v>
       </c>
       <c r="BA12" t="n">
-        <v>8.24</v>
+        <v>7.82</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3256,10 +3256,10 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>6.19</v>
+        <v>6.34</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.29</v>
+        <v>7.23</v>
       </c>
       <c r="AA13" t="n">
         <v>9.69</v>
@@ -3280,13 +3280,13 @@
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>67.44</v>
+        <v>67.64</v>
       </c>
       <c r="AH13" t="n">
         <v>64.5</v>
       </c>
       <c r="AI13" t="n">
-        <v>63.3</v>
+        <v>63</v>
       </c>
       <c r="AJ13" t="n">
         <v>78.09999999999999</v>
@@ -3295,29 +3295,29 @@
         <v>82.8</v>
       </c>
       <c r="AL13" t="n">
-        <v>-0.41</v>
+        <v>2.14</v>
       </c>
       <c r="AM13" t="n">
-        <v>4.64</v>
+        <v>3.85</v>
       </c>
       <c r="AN13" t="n">
-        <v>8.42</v>
+        <v>8.44</v>
       </c>
       <c r="AO13" t="n">
         <v>0.87</v>
       </c>
       <c r="AP13" t="n">
-        <v>66.12860000000001</v>
+        <v>66.2912</v>
       </c>
       <c r="AQ13" t="n">
-        <v>64.0175</v>
+        <v>64.0718</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>63.3</v>
+        <v>63</v>
       </c>
       <c r="AU13" t="n">
         <v>78.09999999999999</v>
@@ -3326,19 +3326,19 @@
         <v>82.8</v>
       </c>
       <c r="AW13" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX13" t="n">
-        <v>66.22</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="AY13" t="n">
         <v>67.65000000000001</v>
       </c>
       <c r="AZ13" t="n">
-        <v>1.98</v>
+        <v>2.03</v>
       </c>
       <c r="BA13" t="n">
-        <v>5.35</v>
+        <v>5.57</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3374,10 +3374,10 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>73.2</v>
+        <v>73.3</v>
       </c>
       <c r="F14" t="n">
-        <v>73.5</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3386,12 +3386,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 73.2; priority 73.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.3; priority 73.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3406,12 +3406,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 73.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 73.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.2%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3462,13 +3462,13 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>2.07</v>
+        <v>1.71</v>
       </c>
       <c r="Z14" t="n">
-        <v>22.24</v>
+        <v>22.57</v>
       </c>
       <c r="AA14" t="n">
-        <v>12.99</v>
+        <v>12.98</v>
       </c>
       <c r="AB14" t="n">
         <v>-21.07</v>
@@ -3486,13 +3486,13 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>166.54</v>
+        <v>167.7</v>
       </c>
       <c r="AH14" t="n">
-        <v>73.5</v>
+        <v>73.3</v>
       </c>
       <c r="AI14" t="n">
-        <v>64.7</v>
+        <v>65.2</v>
       </c>
       <c r="AJ14" t="n">
         <v>67.59999999999999</v>
@@ -3501,29 +3501,29 @@
         <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>1.69</v>
+        <v>3.51</v>
       </c>
       <c r="AM14" t="n">
-        <v>10.39</v>
+        <v>11.93</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.98</v>
+        <v>17.74</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
       <c r="AP14" t="n">
-        <v>165.6608</v>
+        <v>165.7396</v>
       </c>
       <c r="AQ14" t="n">
-        <v>153.8556</v>
+        <v>154.0994</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>64.7</v>
+        <v>65.2</v>
       </c>
       <c r="AU14" t="n">
         <v>67.59999999999999</v>
@@ -3532,19 +3532,19 @@
         <v>82.8</v>
       </c>
       <c r="AW14" t="n">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="AX14" t="n">
-        <v>162.02</v>
+        <v>165.1</v>
       </c>
       <c r="AY14" t="n">
         <v>169.62</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.53</v>
+        <v>1.18</v>
       </c>
       <c r="BA14" t="n">
-        <v>8.24</v>
+        <v>8.83</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3570,20 +3570,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWQU.MI</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>72.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="F15" t="n">
-        <v>73.5</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3592,12 +3592,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 78.87. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 72.1; priority 73.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.2; priority 73.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3617,17 +3617,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 73.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.1%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 78.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 73.80 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 120.73 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3646,20 +3646,20 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>73.8</v>
+        <v>120.73</v>
       </c>
       <c r="T15" t="n">
-        <v>78.87</v>
+        <v>129.38</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>Factor</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -3668,16 +3668,16 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>4.74</v>
+        <v>2.66</v>
       </c>
       <c r="Z15" t="n">
-        <v>20.7</v>
+        <v>20.82</v>
       </c>
       <c r="AA15" t="n">
-        <v>12.85</v>
+        <v>13.18</v>
       </c>
       <c r="AB15" t="n">
-        <v>-20.6</v>
+        <v>-21.63</v>
       </c>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -3688,69 +3688,69 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Quality globale</t>
+          <t>Azionario globale sviluppato</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>77.73999999999999</v>
+        <v>127.57</v>
       </c>
       <c r="AH15" t="n">
-        <v>65.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AI15" t="n">
-        <v>67.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="AJ15" t="n">
-        <v>68.09999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AK15" t="n">
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>0.6899999999999999</v>
+        <v>3.14</v>
       </c>
       <c r="AM15" t="n">
-        <v>9.369999999999999</v>
+        <v>12.32</v>
       </c>
       <c r="AN15" t="n">
-        <v>15.62</v>
+        <v>17.55</v>
       </c>
       <c r="AO15" t="n">
-        <v>1.22</v>
+        <v>1.33</v>
       </c>
       <c r="AP15" t="n">
-        <v>77.19</v>
+        <v>126.152</v>
       </c>
       <c r="AQ15" t="n">
-        <v>71.8681</v>
+        <v>117.4156</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>67.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="AU15" t="n">
-        <v>68.09999999999999</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AV15" t="n">
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX15" t="n">
-        <v>76.23</v>
+        <v>126.11</v>
       </c>
       <c r="AY15" t="n">
-        <v>78.87</v>
+        <v>129.38</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.71</v>
+        <v>1.12</v>
       </c>
       <c r="BA15" t="n">
-        <v>8.17</v>
+        <v>8.65</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3776,20 +3776,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>IWQU.MI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>73.09999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>73.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3798,12 +3798,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 78.87. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 73.1; priority 73.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.1; priority 73.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3818,22 +3818,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 73.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
+          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 78.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 120.73 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 73.80 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3852,20 +3852,20 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>120.73</v>
+        <v>73.8</v>
       </c>
       <c r="T16" t="n">
-        <v>129.38</v>
+        <v>78.87</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Factor</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -3874,16 +3874,16 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>2.63</v>
+        <v>4.94</v>
       </c>
       <c r="Z16" t="n">
-        <v>20.6</v>
+        <v>20.31</v>
       </c>
       <c r="AA16" t="n">
-        <v>13.19</v>
+        <v>12.84</v>
       </c>
       <c r="AB16" t="n">
-        <v>-21.63</v>
+        <v>-20.6</v>
       </c>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
@@ -3894,69 +3894,69 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Azionario globale sviluppato</t>
+          <t>Quality globale</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>126.68</v>
+        <v>77.94</v>
       </c>
       <c r="AH16" t="n">
-        <v>72.8</v>
+        <v>65.2</v>
       </c>
       <c r="AI16" t="n">
-        <v>65.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AJ16" t="n">
-        <v>66.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AK16" t="n">
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>1.21</v>
+        <v>2.24</v>
       </c>
       <c r="AM16" t="n">
-        <v>10.91</v>
+        <v>10.18</v>
       </c>
       <c r="AN16" t="n">
-        <v>17.88</v>
+        <v>15.13</v>
       </c>
       <c r="AO16" t="n">
-        <v>1.36</v>
+        <v>1.18</v>
       </c>
       <c r="AP16" t="n">
-        <v>126.0474</v>
+        <v>77.2728</v>
       </c>
       <c r="AQ16" t="n">
-        <v>117.2403</v>
+        <v>71.9829</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>65.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AU16" t="n">
-        <v>66.90000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AV16" t="n">
         <v>82.8</v>
       </c>
       <c r="AW16" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX16" t="n">
-        <v>123.69</v>
+        <v>77.25</v>
       </c>
       <c r="AY16" t="n">
-        <v>129.38</v>
+        <v>78.87</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.5</v>
+        <v>0.86</v>
       </c>
       <c r="BA16" t="n">
-        <v>8.050000000000001</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -3992,10 +3992,10 @@
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>71.8</v>
+        <v>72</v>
       </c>
       <c r="F17" t="n">
-        <v>72.40000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 71.8; priority 72.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.0; priority 72.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4024,12 +4024,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 72.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -4080,10 +4080,10 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>1.54</v>
+        <v>1.72</v>
       </c>
       <c r="Z17" t="n">
-        <v>20.13</v>
+        <v>20.14</v>
       </c>
       <c r="AA17" t="n">
         <v>14.24</v>
@@ -4104,13 +4104,13 @@
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>709.6799999999999</v>
+        <v>716.04</v>
       </c>
       <c r="AH17" t="n">
-        <v>70.3</v>
+        <v>69.8</v>
       </c>
       <c r="AI17" t="n">
-        <v>64.8</v>
+        <v>66.3</v>
       </c>
       <c r="AJ17" t="n">
         <v>64.3</v>
@@ -4119,29 +4119,29 @@
         <v>82.8</v>
       </c>
       <c r="AL17" t="n">
-        <v>0.9399999999999999</v>
+        <v>3.7</v>
       </c>
       <c r="AM17" t="n">
-        <v>12.64</v>
+        <v>14.75</v>
       </c>
       <c r="AN17" t="n">
-        <v>18.35</v>
+        <v>17.98</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.29</v>
+        <v>1.26</v>
       </c>
       <c r="AP17" t="n">
-        <v>708.9284</v>
+        <v>709.4304</v>
       </c>
       <c r="AQ17" t="n">
-        <v>657.8077</v>
+        <v>658.7511</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>85</v>
       </c>
       <c r="AT17" t="n">
-        <v>64.8</v>
+        <v>66.3</v>
       </c>
       <c r="AU17" t="n">
         <v>64.3</v>
@@ -4150,19 +4150,19 @@
         <v>82.8</v>
       </c>
       <c r="AW17" t="n">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="AX17" t="n">
-        <v>690.52</v>
+        <v>707.24</v>
       </c>
       <c r="AY17" t="n">
         <v>727.1799999999999</v>
       </c>
       <c r="AZ17" t="n">
-        <v>0.11</v>
+        <v>0.93</v>
       </c>
       <c r="BA17" t="n">
-        <v>7.89</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4198,10 +4198,10 @@
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>70.3</v>
+        <v>70</v>
       </c>
       <c r="F18" t="n">
-        <v>71.2</v>
+        <v>70.8</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4210,12 +4210,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 70.3; priority 71.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 70.0; priority 70.8; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 70.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 70.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.5%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -4286,10 +4286,10 @@
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>-1.24</v>
+        <v>-3.7</v>
       </c>
       <c r="Z18" t="n">
-        <v>33.91</v>
+        <v>35.85</v>
       </c>
       <c r="AA18" t="n">
         <v>17.07</v>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="AG18" t="n">
-        <v>47.385</v>
+        <v>47.655</v>
       </c>
       <c r="AH18" t="n">
-        <v>67.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AI18" t="n">
-        <v>61.5</v>
+        <v>59.7</v>
       </c>
       <c r="AJ18" t="n">
         <v>64.2</v>
@@ -4325,29 +4325,29 @@
         <v>82.8</v>
       </c>
       <c r="AL18" t="n">
-        <v>5.46</v>
+        <v>6.47</v>
       </c>
       <c r="AM18" t="n">
-        <v>7.94</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="AN18" t="n">
-        <v>19.08</v>
+        <v>19.56</v>
       </c>
       <c r="AO18" t="n">
-        <v>1.12</v>
+        <v>1.15</v>
       </c>
       <c r="AP18" t="n">
-        <v>47.0566</v>
+        <v>46.9617</v>
       </c>
       <c r="AQ18" t="n">
-        <v>43.2389</v>
+        <v>43.3316</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>85</v>
       </c>
       <c r="AT18" t="n">
-        <v>61.5</v>
+        <v>59.7</v>
       </c>
       <c r="AU18" t="n">
         <v>64.2</v>
@@ -4356,19 +4356,19 @@
         <v>82.8</v>
       </c>
       <c r="AW18" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX18" t="n">
-        <v>44.76</v>
+        <v>45.455</v>
       </c>
       <c r="AY18" t="n">
         <v>48.005</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0.7</v>
+        <v>1.48</v>
       </c>
       <c r="BA18" t="n">
-        <v>9.59</v>
+        <v>9.98</v>
       </c>
       <c r="BB18" t="inlineStr"/>
       <c r="BC18" t="inlineStr"/>
@@ -4504,7 +4504,7 @@
         <v>-33.36</v>
       </c>
       <c r="AC19" t="n">
-        <v>36.7</v>
+        <v>36.62</v>
       </c>
       <c r="AD19" t="n">
         <v>33.52</v>
@@ -4603,7 +4603,7 @@
         <v>76.09999999999999</v>
       </c>
       <c r="BL19" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="BM19" t="n">
         <v>41.1</v>
@@ -4826,7 +4826,7 @@
         <v>18.86</v>
       </c>
       <c r="BI20" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="BJ20" t="n">
         <v>100</v>
@@ -4853,53 +4853,49 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2. Rischio da controllare</t>
+          <t>4. Alert / monitoraggio</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SGLD.MI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>Invesco Physical Gold ETC</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>71.7</v>
+        <v>60.4</v>
       </c>
       <c r="F21" t="n">
-        <v>53.7</v>
+        <v>62.4</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>🟥 Solo size piccola</t>
+          <t>🟡 Metti alert / monitora</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 384.93. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 71.7; priority 53.7; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 60.4; priority 62.4; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -4909,17 +4905,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 4.4%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 60.4, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 4.4%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 227.98 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 190.01 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -4929,173 +4925,151 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>190.01</v>
+        <v>337.23</v>
       </c>
       <c r="T21" t="n">
-        <v>227.98</v>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+        <v>384.93</v>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Invesco Physical Gold ETC</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Defensive</t>
+        </is>
+      </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>3.16</v>
+        <v>-1.23</v>
       </c>
       <c r="Z21" t="n">
-        <v>19.96</v>
+        <v>30.92</v>
       </c>
       <c r="AA21" t="n">
-        <v>46.9</v>
+        <v>18.89</v>
       </c>
       <c r="AB21" t="n">
-        <v>-36.88</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>14.34</v>
-      </c>
+        <v>-22.72</v>
+      </c>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF21" t="inlineStr"/>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Oro</t>
+        </is>
+      </c>
       <c r="AG21" t="n">
-        <v>217.55</v>
-      </c>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
-      <c r="AK21" t="inlineStr"/>
+        <v>368</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>76.5</v>
+      </c>
       <c r="AL21" t="n">
-        <v>11.54</v>
+        <v>7.49</v>
       </c>
       <c r="AM21" t="n">
-        <v>22.93</v>
+        <v>-13.6</v>
       </c>
       <c r="AN21" t="n">
-        <v>65.03</v>
+        <v>28.66</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.39</v>
+        <v>1.52</v>
       </c>
       <c r="AP21" t="n">
-        <v>208.42</v>
+        <v>352.3482</v>
       </c>
       <c r="AQ21" t="n">
-        <v>195.6651</v>
+        <v>373.1635</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="AT21" t="n">
-        <v>73.2</v>
+        <v>47.8</v>
       </c>
       <c r="AU21" t="n">
-        <v>14.2</v>
+        <v>59.2</v>
       </c>
       <c r="AV21" t="n">
-        <v>81.2</v>
+        <v>76.5</v>
       </c>
       <c r="AW21" t="n">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="AX21" t="n">
-        <v>206.64</v>
+        <v>337.28</v>
       </c>
       <c r="AY21" t="n">
-        <v>227.98</v>
+        <v>384.93</v>
       </c>
       <c r="AZ21" t="n">
-        <v>4.38</v>
+        <v>4.44</v>
       </c>
       <c r="BA21" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="BB21" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC21" t="inlineStr">
-        <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-      <c r="BD21" t="n">
-        <v>5253179637760</v>
-      </c>
-      <c r="BE21" t="n">
-        <v>63.66</v>
-      </c>
-      <c r="BF21" t="n">
-        <v>117.21</v>
-      </c>
-      <c r="BG21" t="n">
-        <v>105.9</v>
-      </c>
-      <c r="BH21" t="n">
-        <v>16.97</v>
-      </c>
-      <c r="BI21" t="n">
-        <v>44</v>
-      </c>
-      <c r="BJ21" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK21" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="BL21" t="n">
-        <v>75.8</v>
-      </c>
-      <c r="BM21" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="BN21" t="n">
-        <v>81.2</v>
-      </c>
+        <v>-1.38</v>
+      </c>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="inlineStr"/>
+      <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
       <c r="BO21" t="inlineStr"/>
-      <c r="BP21" t="inlineStr">
-        <is>
-          <t>USA / Semiconductors</t>
-        </is>
-      </c>
+      <c r="BP21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5. Solo osservazione</t>
+          <t>2. Rischio da controllare</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5104,54 +5078,54 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>38.5</v>
+        <v>71.8</v>
       </c>
       <c r="F22" t="n">
-        <v>32.3</v>
+        <v>53.7</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>⚪ Evita per ora</t>
+          <t>🟥 Solo size piccola</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Lascia fuori dalla lista operativa finché trend, score o rischio non migliorano.</t>
+          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 71.8; priority 53.7; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Dati prezzo insufficienti.</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 71.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 4.4%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 227.98 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
+          <t>Scenario negativo: perdita area 190.01 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5161,104 +5135,156 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>No Data</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>190.01</v>
+      </c>
+      <c r="T22" t="n">
+        <v>227.98</v>
+      </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Evitare per ora</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>19.96</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-36.88</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>27.47</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>14.21</v>
+      </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
+      <c r="AG22" t="n">
+        <v>217.55</v>
+      </c>
       <c r="AH22" t="inlineStr"/>
       <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr"/>
-      <c r="AQ22" t="inlineStr"/>
+      <c r="AL22" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>22.93</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>65.03</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>208.42</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>195.6651</v>
+      </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>73.2</v>
       </c>
       <c r="AU22" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>753</v>
+      </c>
+      <c r="AX22" t="n">
+        <v>206.64</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>227.98</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC22" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+      <c r="BD22" t="n">
+        <v>5253179637760</v>
+      </c>
+      <c r="BE22" t="n">
+        <v>63.66</v>
+      </c>
+      <c r="BF22" t="n">
+        <v>117.21</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="BH22" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>46</v>
+      </c>
+      <c r="BJ22" t="n">
         <v>100</v>
       </c>
-      <c r="AV22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX22" t="inlineStr"/>
-      <c r="AY22" t="inlineStr"/>
-      <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" t="inlineStr"/>
-      <c r="BB22" t="inlineStr"/>
-      <c r="BC22" t="inlineStr"/>
-      <c r="BD22" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE22" t="inlineStr"/>
-      <c r="BF22" t="inlineStr"/>
-      <c r="BG22" t="inlineStr"/>
-      <c r="BH22" t="inlineStr"/>
-      <c r="BI22" t="inlineStr"/>
-      <c r="BJ22" t="n">
-        <v>50</v>
-      </c>
       <c r="BK22" t="n">
-        <v>0</v>
+        <v>73.2</v>
       </c>
       <c r="BL22" t="n">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="BM22" t="n">
-        <v>100</v>
+        <v>14.2</v>
       </c>
       <c r="BN22" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO22" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
+        <v>81.2</v>
+      </c>
+      <c r="BO22" t="inlineStr"/>
       <c r="BP22" t="inlineStr">
         <is>
-          <t>Italy / Semiconductors</t>
+          <t>USA / Semiconductors</t>
         </is>
       </c>
     </row>
@@ -5270,20 +5296,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EUNA.MI</t>
+          <t>STM.MI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>iShares Core Global Aggregate Bond</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E23" t="n">
-        <v>28.6</v>
+        <v>38.5</v>
       </c>
       <c r="F23" t="n">
-        <v>27.9</v>
+        <v>32.3</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -5297,7 +5327,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -5317,7 +5347,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -5347,17 +5377,13 @@
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>iShares Core Global Aggregate Bond</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>Defensive</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr">
         <is>
           <t>Evitare per ora</t>
@@ -5371,38 +5397,22 @@
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>Obbligazionario globale</t>
-        </is>
-      </c>
+          <t>Da monitorare con scenario positivo, base e negativo.</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>100</v>
-      </c>
-      <c r="AK23" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
       <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
+      <c r="AR23" t="inlineStr"/>
       <c r="AS23" t="n">
         <v>0</v>
       </c>
@@ -5424,19 +5434,39 @@
       <c r="BA23" t="inlineStr"/>
       <c r="BB23" t="inlineStr"/>
       <c r="BC23" t="inlineStr"/>
-      <c r="BD23" t="inlineStr"/>
+      <c r="BD23" t="n">
+        <v>0</v>
+      </c>
       <c r="BE23" t="inlineStr"/>
       <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr"/>
       <c r="BH23" t="inlineStr"/>
       <c r="BI23" t="inlineStr"/>
-      <c r="BJ23" t="inlineStr"/>
-      <c r="BK23" t="inlineStr"/>
-      <c r="BL23" t="inlineStr"/>
-      <c r="BM23" t="inlineStr"/>
-      <c r="BN23" t="inlineStr"/>
-      <c r="BO23" t="inlineStr"/>
-      <c r="BP23" t="inlineStr"/>
+      <c r="BJ23" t="n">
+        <v>50</v>
+      </c>
+      <c r="BK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL23" t="n">
+        <v>50</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>100</v>
+      </c>
+      <c r="BN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO23" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
+      <c r="BP23" t="inlineStr">
+        <is>
+          <t>Italy / Semiconductors</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5446,64 +5476,64 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SGLD.MI</t>
+          <t>EUNA.MI</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
+          <t>iShares Core Global Aggregate Bond</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>65.40000000000001</v>
+        <v>28.6</v>
       </c>
       <c r="F24" t="n">
-        <v>61.3</v>
+        <v>27.9</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>⚪ Osserva</t>
+          <t>⚪ Evita per ora</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
+          <t>Lascia fuori dalla lista operativa finché trend, score o rischio non migliorano.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>score 65.4; priority 61.3; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Normal risk</t>
+          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>Dati prezzo insufficienti.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 65.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 8.0%.</t>
+          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -5513,24 +5543,20 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="S24" t="n">
-        <v>337.23</v>
-      </c>
-      <c r="T24" t="n">
-        <v>384.93</v>
-      </c>
+          <t>No Data</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
+          <t>iShares Core Global Aggregate Bond</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -5540,21 +5566,13 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Osservare</t>
-        </is>
-      </c>
-      <c r="Y24" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>36.47</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>18.79</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>-22.72</v>
-      </c>
+          <t>Evitare per ora</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
@@ -5564,70 +5582,52 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Oro</t>
-        </is>
-      </c>
-      <c r="AG24" t="n">
-        <v>379.54</v>
-      </c>
+          <t>Obbligazionario globale</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="n">
-        <v>69.3</v>
+        <v>34.2</v>
       </c>
       <c r="AI24" t="n">
-        <v>53.6</v>
+        <v>0</v>
       </c>
       <c r="AJ24" t="n">
-        <v>59.3</v>
+        <v>100</v>
       </c>
       <c r="AK24" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>11.42</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>-10.6</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>30.21</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>351.46</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>372.8023</v>
-      </c>
-      <c r="AR24" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
       <c r="AS24" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="AT24" t="n">
-        <v>53.6</v>
+        <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>59.3</v>
+        <v>100</v>
       </c>
       <c r="AV24" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="AW24" t="n">
-        <v>757</v>
-      </c>
-      <c r="AX24" t="n">
-        <v>337.28</v>
-      </c>
-      <c r="AY24" t="n">
-        <v>384.93</v>
-      </c>
-      <c r="AZ24" t="n">
-        <v>7.99</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>1.81</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
       <c r="BB24" t="inlineStr"/>
       <c r="BC24" t="inlineStr"/>
       <c r="BD24" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v9_news_realtime_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -780,10 +780,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>69.09999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>67.3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 69.1; priority 67.0; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 69.4; priority 67.3; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>AMZN: scenario base Accumulate Carefully, score 69.1, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.0%.</t>
+          <t>AMZN: scenario base Accumulate Carefully, score 69.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.6%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -864,22 +864,22 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>-0.62</v>
+        <v>1.76</v>
       </c>
       <c r="Z2" t="n">
-        <v>11.32</v>
+        <v>12.9</v>
       </c>
       <c r="AA2" t="n">
-        <v>32.42</v>
+        <v>32.4</v>
       </c>
       <c r="AB2" t="n">
         <v>-30.88</v>
       </c>
       <c r="AC2" t="n">
-        <v>20.49</v>
+        <v>20.45</v>
       </c>
       <c r="AD2" t="n">
-        <v>24.53</v>
+        <v>24.47</v>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
@@ -888,36 +888,36 @@
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="n">
-        <v>254.92</v>
+        <v>254.41</v>
       </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="n">
-        <v>-10.25</v>
+        <v>-8.289999999999999</v>
       </c>
       <c r="AM2" t="n">
-        <v>22.13</v>
+        <v>17.34</v>
       </c>
       <c r="AN2" t="n">
-        <v>23.09</v>
+        <v>22.97</v>
       </c>
       <c r="AO2" t="n">
         <v>0.71</v>
       </c>
       <c r="AP2" t="n">
-        <v>252.4094</v>
+        <v>252.8154</v>
       </c>
       <c r="AQ2" t="n">
-        <v>238.7866</v>
+        <v>238.8707</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>65.2</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AU2" t="n">
         <v>36.4</v>
@@ -926,19 +926,19 @@
         <v>82.8</v>
       </c>
       <c r="AW2" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX2" t="n">
-        <v>254.92</v>
+        <v>254.41</v>
       </c>
       <c r="AY2" t="n">
         <v>278.09</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.99</v>
+        <v>0.63</v>
       </c>
       <c r="BA2" t="n">
-        <v>6.76</v>
+        <v>6.51</v>
       </c>
       <c r="BB2" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="BD2" t="n">
-        <v>2749647028224</v>
+        <v>2743822450688</v>
       </c>
       <c r="BE2" t="n">
         <v>17.44</v>
@@ -970,10 +970,10 @@
         <v>86.40000000000001</v>
       </c>
       <c r="BK2" t="n">
-        <v>65.2</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="BL2" t="n">
-        <v>69.40000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="BM2" t="n">
         <v>36.4</v>
@@ -1006,10 +1006,10 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>62.3</v>
+        <v>61.7</v>
       </c>
       <c r="F3" t="n">
-        <v>66.7</v>
+        <v>65.8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 62.3; priority 66.7; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 61.7; priority 65.8; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Hold / Monitor, score 62.3, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
+          <t>RBOT.MI: scenario base Hold / Monitor, score 61.7, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.5%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1094,13 +1094,13 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>0.13</v>
+        <v>-0.75</v>
       </c>
       <c r="Z3" t="n">
-        <v>38.02</v>
+        <v>37.46</v>
       </c>
       <c r="AA3" t="n">
-        <v>22.52</v>
+        <v>22.53</v>
       </c>
       <c r="AB3" t="n">
         <v>-29.37</v>
@@ -1118,65 +1118,65 @@
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>18.194</v>
+        <v>17.938</v>
       </c>
       <c r="AH3" t="n">
-        <v>50.9</v>
+        <v>50.6</v>
       </c>
       <c r="AI3" t="n">
-        <v>75.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="AJ3" t="n">
         <v>44.5</v>
       </c>
       <c r="AK3" t="n">
-        <v>79.5</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="AL3" t="n">
-        <v>3.6</v>
+        <v>0.13</v>
       </c>
       <c r="AM3" t="n">
-        <v>27.07</v>
+        <v>28.39</v>
       </c>
       <c r="AN3" t="n">
-        <v>19.18</v>
+        <v>18.68</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="AP3" t="n">
-        <v>18.2209</v>
+        <v>18.2174</v>
       </c>
       <c r="AQ3" t="n">
-        <v>15.8101</v>
+        <v>15.8302</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
         <v>65</v>
       </c>
       <c r="AT3" t="n">
-        <v>75.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="AU3" t="n">
         <v>49.5</v>
       </c>
       <c r="AV3" t="n">
-        <v>79.5</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="AW3" t="n">
         <v>756</v>
       </c>
       <c r="AX3" t="n">
-        <v>18.164</v>
+        <v>17.938</v>
       </c>
       <c r="AY3" t="n">
         <v>19.25</v>
       </c>
       <c r="AZ3" t="n">
-        <v>-0.15</v>
+        <v>-1.53</v>
       </c>
       <c r="BA3" t="n">
-        <v>15.08</v>
+        <v>13.32</v>
       </c>
       <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="inlineStr"/>
@@ -1216,10 +1216,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>64.3</v>
+        <v>65.3</v>
       </c>
       <c r="F4" t="n">
-        <v>50.1</v>
+        <v>51.3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 64.3; priority 50.1; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 65.3; priority 51.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>prezzo 6.3% sotto MA50: attendere recupero</t>
+          <t>prezzo 5.9% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 64.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -6.3%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 65.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.9%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>-4.06</v>
+        <v>-1.4</v>
       </c>
       <c r="Z4" t="n">
-        <v>123.1</v>
+        <v>119.54</v>
       </c>
       <c r="AA4" t="n">
         <v>39.53</v>
@@ -1312,10 +1312,10 @@
         <v>-44.77</v>
       </c>
       <c r="AC4" t="n">
-        <v>56.49</v>
+        <v>56.67</v>
       </c>
       <c r="AD4" t="n">
-        <v>27.76</v>
+        <v>27.85</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1324,42 +1324,42 @@
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>1435.4</v>
+        <v>1440</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>1.11</v>
+        <v>-2.21</v>
       </c>
       <c r="AM4" t="n">
-        <v>20.05</v>
+        <v>21.83</v>
       </c>
       <c r="AN4" t="n">
-        <v>33.54</v>
+        <v>33.32</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="AP4" t="n">
-        <v>1532.0728</v>
+        <v>1529.8342</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1272.2172</v>
+        <v>1275.1098</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
         <v>65</v>
       </c>
       <c r="AT4" t="n">
-        <v>87.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="AU4" t="n">
         <v>16.7</v>
       </c>
       <c r="AV4" t="n">
-        <v>70.3</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AW4" t="n">
         <v>765</v>
@@ -1371,10 +1371,10 @@
         <v>1621.2</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-6.31</v>
+        <v>-5.87</v>
       </c>
       <c r="BA4" t="n">
-        <v>12.83</v>
+        <v>12.93</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>551337132032</v>
+        <v>553103982592</v>
       </c>
       <c r="BE4" t="n">
         <v>30.11</v>
@@ -1402,22 +1402,22 @@
         <v>9.09</v>
       </c>
       <c r="BI4" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="BJ4" t="n">
         <v>100</v>
       </c>
       <c r="BK4" t="n">
-        <v>87.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="BL4" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="BM4" t="n">
         <v>16.7</v>
       </c>
       <c r="BN4" t="n">
-        <v>70.3</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>prezzo 5.7% sotto MA50: attendere recupero</t>
+          <t>prezzo 5.6% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>SMH: scenario base Hold / Monitor, score 57.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.7%.</t>
+          <t>SMH: scenario base Hold / Monitor, score 57.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.6%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1532,13 +1532,13 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>-13.76</v>
+        <v>-13.7</v>
       </c>
       <c r="Z5" t="n">
-        <v>88.40000000000001</v>
+        <v>88.52</v>
       </c>
       <c r="AA5" t="n">
-        <v>36.95</v>
+        <v>36.93</v>
       </c>
       <c r="AB5" t="n">
         <v>-35.74</v>
@@ -1556,50 +1556,50 @@
         </is>
       </c>
       <c r="AG5" t="n">
-        <v>545.22</v>
+        <v>545.5700000000001</v>
       </c>
       <c r="AH5" t="n">
         <v>52</v>
       </c>
       <c r="AI5" t="n">
-        <v>76.5</v>
+        <v>76.7</v>
       </c>
       <c r="AJ5" t="n">
         <v>22.1</v>
       </c>
       <c r="AK5" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="AL5" t="n">
-        <v>-0.04</v>
+        <v>0.02</v>
       </c>
       <c r="AM5" t="n">
-        <v>39.42</v>
+        <v>39.51</v>
       </c>
       <c r="AN5" t="n">
-        <v>52.68</v>
+        <v>52.71</v>
       </c>
       <c r="AO5" t="n">
         <v>1.43</v>
       </c>
       <c r="AP5" t="n">
-        <v>578.1212</v>
+        <v>577.9704</v>
       </c>
       <c r="AQ5" t="n">
-        <v>474.0544</v>
+        <v>474.0167</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
         <v>65</v>
       </c>
       <c r="AT5" t="n">
-        <v>76.5</v>
+        <v>76.7</v>
       </c>
       <c r="AU5" t="n">
         <v>27.1</v>
       </c>
       <c r="AV5" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="AW5" t="n">
         <v>751</v>
@@ -1611,10 +1611,10 @@
         <v>594.0700000000001</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-5.69</v>
+        <v>-5.61</v>
       </c>
       <c r="BA5" t="n">
-        <v>15.01</v>
+        <v>15.1</v>
       </c>
       <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr"/>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>61.3</v>
+        <v>60.7</v>
       </c>
       <c r="F6" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 61.3; priority 42.7; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 60.7; priority 42.6; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>META: scenario base Hold / Monitor, score 61.3, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -2.3%.</t>
+          <t>META: scenario base Hold / Monitor, score 60.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.6%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1738,22 +1738,22 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-3.1</v>
+        <v>-5.33</v>
       </c>
       <c r="Z6" t="n">
-        <v>-21.42</v>
+        <v>-19.58</v>
       </c>
       <c r="AA6" t="n">
-        <v>37.5</v>
+        <v>37.49</v>
       </c>
       <c r="AB6" t="n">
         <v>-34.15</v>
       </c>
       <c r="AC6" t="n">
-        <v>21.78</v>
+        <v>22.19</v>
       </c>
       <c r="AD6" t="n">
-        <v>16.55</v>
+        <v>16.86</v>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
@@ -1762,45 +1762,45 @@
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>578.54</v>
+        <v>589.2495</v>
       </c>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>-1.98</v>
+        <v>0.22</v>
       </c>
       <c r="AM6" t="n">
-        <v>-11.53</v>
+        <v>-11.6</v>
       </c>
       <c r="AN6" t="n">
-        <v>25</v>
+        <v>25.73</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="AP6" t="n">
-        <v>592.3404</v>
+        <v>592.8814</v>
       </c>
       <c r="AQ6" t="n">
-        <v>621.5884</v>
+        <v>621.4931</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
         <v>35</v>
       </c>
       <c r="AT6" t="n">
-        <v>33.4</v>
+        <v>30.7</v>
       </c>
       <c r="AU6" t="n">
         <v>27.7</v>
       </c>
       <c r="AV6" t="n">
-        <v>71.8</v>
+        <v>74.3</v>
       </c>
       <c r="AW6" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX6" t="n">
         <v>543.67</v>
@@ -1809,10 +1809,10 @@
         <v>599.12</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-2.33</v>
+        <v>-0.61</v>
       </c>
       <c r="BA6" t="n">
-        <v>-6.93</v>
+        <v>-5.19</v>
       </c>
       <c r="BB6" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="BD6" t="n">
-        <v>1473834123264</v>
+        <v>1501118070784</v>
       </c>
       <c r="BE6" t="n">
         <v>29.83</v>
@@ -1846,16 +1846,16 @@
         <v>100</v>
       </c>
       <c r="BK6" t="n">
-        <v>33.4</v>
+        <v>30.7</v>
       </c>
       <c r="BL6" t="n">
-        <v>79.3</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="BM6" t="n">
         <v>27.7</v>
       </c>
       <c r="BN6" t="n">
-        <v>71.8</v>
+        <v>74.3</v>
       </c>
       <c r="BO6" t="inlineStr"/>
       <c r="BP6" t="inlineStr">
@@ -1882,10 +1882,10 @@
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>35</v>
+        <v>35.9</v>
       </c>
       <c r="F7" t="n">
-        <v>28.7</v>
+        <v>41.6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 35.0; priority 28.7; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 35.9; priority 41.6; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 35.0, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -7.8%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 35.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -7.8%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.58 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>8.58</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="T7" t="n">
         <v>10.872</v>
@@ -1970,16 +1970,16 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>-25.35</v>
+        <v>-24.1</v>
       </c>
       <c r="Z7" t="n">
-        <v>20.48</v>
+        <v>21.47</v>
       </c>
       <c r="AA7" t="n">
-        <v>24.14</v>
+        <v>24.13</v>
       </c>
       <c r="AB7" t="n">
-        <v>-35.07</v>
+        <v>-34.68</v>
       </c>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
@@ -1994,47 +1994,47 @@
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>8.58</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="AH7" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="AI7" t="n">
-        <v>17.4</v>
+        <v>20.5</v>
       </c>
       <c r="AJ7" t="n">
-        <v>38</v>
+        <v>38.3</v>
       </c>
       <c r="AK7" t="n">
         <v>63.5</v>
       </c>
       <c r="AL7" t="n">
-        <v>-2.6</v>
+        <v>-5.35</v>
       </c>
       <c r="AM7" t="n">
-        <v>-3.69</v>
+        <v>-1.92</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.12</v>
+        <v>1.16</v>
       </c>
       <c r="AO7" t="n">
         <v>0.05</v>
       </c>
       <c r="AP7" t="n">
-        <v>9.306100000000001</v>
+        <v>9.266500000000001</v>
       </c>
       <c r="AQ7" t="n">
-        <v>9.281599999999999</v>
+        <v>9.281000000000001</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
         <v>35</v>
       </c>
       <c r="AT7" t="n">
-        <v>17.4</v>
+        <v>20.5</v>
       </c>
       <c r="AU7" t="n">
-        <v>43</v>
+        <v>43.3</v>
       </c>
       <c r="AV7" t="n">
         <v>63.5</v>
@@ -2043,16 +2043,16 @@
         <v>756</v>
       </c>
       <c r="AX7" t="n">
-        <v>8.58</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="AY7" t="n">
         <v>9.217000000000001</v>
       </c>
       <c r="AZ7" t="n">
-        <v>-7.8</v>
+        <v>-7.84</v>
       </c>
       <c r="BA7" t="n">
-        <v>-7.56</v>
+        <v>-7.98</v>
       </c>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
@@ -2078,24 +2078,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>WCLD.MI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>32.6</v>
+        <v>53.7</v>
       </c>
       <c r="F8" t="n">
-        <v>24.8</v>
+        <v>29</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2109,12 +2105,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 32.6; priority 24.8; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 53.7; priority 29.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Extended - wait pullback</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -2124,22 +2120,22 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo 13.7% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 32.6, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.8%.</t>
+          <t>WCLD.MI: scenario base High Risk, score 53.7, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 13.7%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 36.89 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2154,151 +2150,131 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S8" t="n">
-        <v>298.32</v>
+        <v>24.785</v>
       </c>
       <c r="T8" t="n">
-        <v>425.3</v>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Tesla, Inc.</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+        <v>36.89</v>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X8" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>-15.96</v>
+        <v>23.65</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.66</v>
+        <v>17.12</v>
       </c>
       <c r="AA8" t="n">
-        <v>58.32</v>
+        <v>35.07</v>
       </c>
       <c r="AB8" t="n">
-        <v>-53.77</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>332.79</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>164.96</v>
-      </c>
+        <v>-48.6</v>
+      </c>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
       <c r="AG8" t="n">
-        <v>356.09</v>
-      </c>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+        <v>35.34</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>14</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>44.1</v>
+      </c>
       <c r="AL8" t="n">
-        <v>10.56</v>
+        <v>13.02</v>
       </c>
       <c r="AM8" t="n">
-        <v>-9.26</v>
+        <v>49.68</v>
       </c>
       <c r="AN8" t="n">
-        <v>11.64</v>
+        <v>6.41</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="AP8" t="n">
-        <v>358.8438</v>
+        <v>31.0894</v>
       </c>
       <c r="AQ8" t="n">
-        <v>400.1974</v>
+        <v>27.0478</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="AT8" t="n">
-        <v>23.8</v>
+        <v>100</v>
       </c>
       <c r="AU8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="AV8" t="n">
-        <v>74.09999999999999</v>
+        <v>44.1</v>
       </c>
       <c r="AW8" t="n">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="AX8" t="n">
-        <v>319.53</v>
+        <v>31.92</v>
       </c>
       <c r="AY8" t="n">
-        <v>367.95</v>
+        <v>36.89</v>
       </c>
       <c r="AZ8" t="n">
-        <v>-0.77</v>
+        <v>13.67</v>
       </c>
       <c r="BA8" t="n">
-        <v>-11.02</v>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="BC8" t="inlineStr">
-        <is>
-          <t>Auto Manufacturers</t>
-        </is>
-      </c>
-      <c r="BD8" t="n">
-        <v>1406394302464</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>18.37</v>
-      </c>
+        <v>30.66</v>
+      </c>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN8" t="n">
-        <v>74.09999999999999</v>
-      </c>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
       <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr">
-        <is>
-          <t>USA / EV</t>
-        </is>
-      </c>
+      <c r="BP8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2308,20 +2284,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WCLD.MI</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E9" t="n">
-        <v>52.4</v>
+        <v>31.9</v>
       </c>
       <c r="F9" t="n">
-        <v>22.5</v>
+        <v>24</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2335,12 +2315,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 52.4; priority 22.5; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 31.9; priority 24.0; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Extended - wait pullback</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2350,22 +2330,22 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo 15.8% sopra MA50: evitare inseguimento</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base High Risk, score 52.4, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 15.8%.</t>
+          <t>TSLA: scenario base High Risk, score 31.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -1.1%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 36.89 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 425.30 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 298.32 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -2380,131 +2360,151 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S9" t="n">
-        <v>24.785</v>
+        <v>298.32</v>
       </c>
       <c r="T9" t="n">
-        <v>36.89</v>
-      </c>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>425.3</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>27.11</v>
+        <v>-16.36</v>
       </c>
       <c r="Z9" t="n">
-        <v>18.75</v>
+        <v>7.6</v>
       </c>
       <c r="AA9" t="n">
-        <v>35.07</v>
+        <v>58.28</v>
       </c>
       <c r="AB9" t="n">
-        <v>-48.6</v>
-      </c>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
+        <v>-53.77</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>331.21</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>164.18</v>
+      </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>Cloud</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="n">
-        <v>35.75</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>14</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>35.6</v>
-      </c>
+        <v>354.39</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="n">
-        <v>19.59</v>
+        <v>8.26</v>
       </c>
       <c r="AM9" t="n">
-        <v>55.37</v>
+        <v>-12.7</v>
       </c>
       <c r="AN9" t="n">
-        <v>6.41</v>
+        <v>11.44</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="AP9" t="n">
-        <v>30.8758</v>
+        <v>358.2994</v>
       </c>
       <c r="AQ9" t="n">
-        <v>27.0196</v>
+        <v>399.9594</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="AT9" t="n">
-        <v>100</v>
+        <v>21.4</v>
       </c>
       <c r="AU9" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="AV9" t="n">
-        <v>35.6</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="AW9" t="n">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="AX9" t="n">
-        <v>31.92</v>
+        <v>319.53</v>
       </c>
       <c r="AY9" t="n">
-        <v>36.89</v>
+        <v>367.95</v>
       </c>
       <c r="AZ9" t="n">
-        <v>15.79</v>
+        <v>-1.09</v>
       </c>
       <c r="BA9" t="n">
-        <v>32.31</v>
-      </c>
-      <c r="BB9" t="inlineStr"/>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="inlineStr"/>
-      <c r="BG9" t="inlineStr"/>
-      <c r="BH9" t="inlineStr"/>
+        <v>-11.39</v>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+      <c r="BD9" t="n">
+        <v>1399680139264</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>18.37</v>
+      </c>
       <c r="BI9" t="inlineStr"/>
-      <c r="BJ9" t="inlineStr"/>
-      <c r="BK9" t="inlineStr"/>
-      <c r="BL9" t="inlineStr"/>
-      <c r="BM9" t="inlineStr"/>
-      <c r="BN9" t="inlineStr"/>
+      <c r="BJ9" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>73.59999999999999</v>
+      </c>
       <c r="BO9" t="inlineStr"/>
-      <c r="BP9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>USA / EV</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2524,10 +2524,10 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>78.59999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>78.59999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 78.6; priority 78.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 79.1; priority 79.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 78.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.9%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 79.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.4%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2612,10 +2612,10 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>0.97</v>
+        <v>1.35</v>
       </c>
       <c r="Z10" t="n">
-        <v>56.2</v>
+        <v>56.31</v>
       </c>
       <c r="AA10" t="n">
         <v>14.13</v>
@@ -2636,13 +2636,13 @@
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>72.97</v>
+        <v>72.59</v>
       </c>
       <c r="AH10" t="n">
-        <v>77.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="AI10" t="n">
-        <v>81.2</v>
+        <v>83.3</v>
       </c>
       <c r="AJ10" t="n">
         <v>68.8</v>
@@ -2651,29 +2651,29 @@
         <v>82.8</v>
       </c>
       <c r="AL10" t="n">
-        <v>3.95</v>
+        <v>2.98</v>
       </c>
       <c r="AM10" t="n">
-        <v>26.27</v>
+        <v>28.91</v>
       </c>
       <c r="AN10" t="n">
-        <v>25.87</v>
+        <v>25.53</v>
       </c>
       <c r="AO10" t="n">
-        <v>1.83</v>
+        <v>1.81</v>
       </c>
       <c r="AP10" t="n">
-        <v>71.6122</v>
+        <v>71.6172</v>
       </c>
       <c r="AQ10" t="n">
-        <v>61.7686</v>
+        <v>61.8725</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
         <v>85</v>
       </c>
       <c r="AT10" t="n">
-        <v>81.2</v>
+        <v>83.3</v>
       </c>
       <c r="AU10" t="n">
         <v>68.8</v>
@@ -2685,16 +2685,16 @@
         <v>756</v>
       </c>
       <c r="AX10" t="n">
-        <v>71.81999999999999</v>
+        <v>71.86</v>
       </c>
       <c r="AY10" t="n">
         <v>73.75</v>
       </c>
       <c r="AZ10" t="n">
-        <v>1.9</v>
+        <v>1.36</v>
       </c>
       <c r="BA10" t="n">
-        <v>18.13</v>
+        <v>17.32</v>
       </c>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2734,10 +2734,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>72.8</v>
+        <v>74.2</v>
       </c>
       <c r="F11" t="n">
-        <v>46.4</v>
+        <v>52.2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 72.8; priority 46.4; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Medium-high risk</t>
+          <t>score 74.2; priority 52.2; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>prezzo 15.1% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 13.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>MSFT: scenario base Accumulate Carefully, score 72.8, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 15.1%.</t>
+          <t>MSFT: scenario base Accumulate Carefully, score 74.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 13.4%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2818,22 +2818,22 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>13.74</v>
+        <v>16.41</v>
       </c>
       <c r="Z11" t="n">
-        <v>-0.31</v>
+        <v>-0.89</v>
       </c>
       <c r="AA11" t="n">
-        <v>26.21</v>
+        <v>26.2</v>
       </c>
       <c r="AB11" t="n">
         <v>-34.5</v>
       </c>
       <c r="AC11" t="n">
-        <v>27.9</v>
+        <v>27.68</v>
       </c>
       <c r="AD11" t="n">
-        <v>21.25</v>
+        <v>21.06</v>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
@@ -2842,45 +2842,45 @@
       </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="n">
-        <v>501.02</v>
+        <v>496.5397</v>
       </c>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="n">
-        <v>2.94</v>
+        <v>0.95</v>
       </c>
       <c r="AM11" t="n">
-        <v>24.54</v>
+        <v>23.04</v>
       </c>
       <c r="AN11" t="n">
-        <v>15.52</v>
+        <v>15.15</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="AP11" t="n">
-        <v>435.2328</v>
+        <v>437.6989</v>
       </c>
       <c r="AQ11" t="n">
-        <v>429.3825</v>
+        <v>429.3692</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>83.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="AU11" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="AV11" t="n">
-        <v>38.3</v>
+        <v>45</v>
       </c>
       <c r="AW11" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX11" t="n">
         <v>479.4474</v>
@@ -2889,10 +2889,10 @@
         <v>513.53</v>
       </c>
       <c r="AZ11" t="n">
-        <v>15.12</v>
+        <v>13.45</v>
       </c>
       <c r="BA11" t="n">
-        <v>16.68</v>
+        <v>15.65</v>
       </c>
       <c r="BB11" t="inlineStr">
         <is>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="BD11" t="n">
-        <v>3720346861568</v>
+        <v>3686783516672</v>
       </c>
       <c r="BE11" t="n">
         <v>40.3</v>
@@ -2920,22 +2920,22 @@
         <v>29.12</v>
       </c>
       <c r="BI11" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="BJ11" t="n">
         <v>100</v>
       </c>
       <c r="BK11" t="n">
-        <v>83.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="BL11" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="BM11" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="BN11" t="n">
-        <v>38.3</v>
+        <v>45</v>
       </c>
       <c r="BO11" t="inlineStr"/>
       <c r="BP11" t="inlineStr">
@@ -2952,20 +2952,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EXSA.DE</t>
+          <t>MVOL.MI</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>74.5</v>
+        <v>72.5</v>
       </c>
       <c r="F12" t="n">
-        <v>75.09999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2974,12 +2974,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 65.95. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 67.85. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>score 74.5; priority 75.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.5; priority 74.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2994,22 +2994,22 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.6%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 65.95 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 67.85 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 61.47 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 63.44 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -3028,111 +3028,111 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>61.4745</v>
+        <v>63.44</v>
       </c>
       <c r="T12" t="n">
-        <v>65.95</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Defensive</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>4.79</v>
+        <v>5.95</v>
       </c>
       <c r="Z12" t="n">
-        <v>20.88</v>
+        <v>7.86</v>
       </c>
       <c r="AA12" t="n">
-        <v>12.77</v>
+        <v>9.69</v>
       </c>
       <c r="AB12" t="n">
-        <v>-16.33</v>
+        <v>-12.85</v>
       </c>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>Europa</t>
+          <t>Min volatility</t>
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>64.78</v>
+        <v>67.48999999999999</v>
       </c>
       <c r="AH12" t="n">
-        <v>72.5</v>
+        <v>64.3</v>
       </c>
       <c r="AI12" t="n">
-        <v>67.59999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="AJ12" t="n">
-        <v>71.59999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AK12" t="n">
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.08</v>
+        <v>1.43</v>
       </c>
       <c r="AM12" t="n">
-        <v>9.44</v>
+        <v>3.53</v>
       </c>
       <c r="AN12" t="n">
-        <v>15.36</v>
+        <v>8.33</v>
       </c>
       <c r="AO12" t="n">
-        <v>1.2</v>
+        <v>0.86</v>
       </c>
       <c r="AP12" t="n">
-        <v>64.67740000000001</v>
+        <v>66.43940000000001</v>
       </c>
       <c r="AQ12" t="n">
-        <v>60.7619</v>
+        <v>64.1176</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>67.59999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="AU12" t="n">
-        <v>71.59999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AV12" t="n">
         <v>82.8</v>
       </c>
       <c r="AW12" t="n">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="AX12" t="n">
-        <v>64.78</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="AY12" t="n">
-        <v>65.95</v>
+        <v>67.75</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.16</v>
+        <v>1.58</v>
       </c>
       <c r="BA12" t="n">
-        <v>6.61</v>
+        <v>5.26</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3158,20 +3158,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MVOL.MI</t>
+          <t>VWCE.DE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>72.40000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>74.3</v>
+        <v>73.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3180,12 +3180,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 67.85. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 72.4; priority 74.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.1; priority 73.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3200,22 +3200,22 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.8%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 73.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 67.85 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 169.62 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 63.44 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 159.24 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -3234,20 +3234,20 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>63.44</v>
+        <v>159.24</v>
       </c>
       <c r="T13" t="n">
-        <v>67.84999999999999</v>
+        <v>169.62</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>Defensive</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -3256,89 +3256,89 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>5.99</v>
+        <v>1.4</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.85</v>
+        <v>22.6</v>
       </c>
       <c r="AA13" t="n">
-        <v>9.69</v>
+        <v>13.01</v>
       </c>
       <c r="AB13" t="n">
-        <v>-12.85</v>
+        <v>-21.07</v>
       </c>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Min volatility</t>
+          <t>Azionario globale</t>
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>67.56999999999999</v>
+        <v>166.1</v>
       </c>
       <c r="AH13" t="n">
-        <v>64.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="AI13" t="n">
-        <v>62.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AJ13" t="n">
-        <v>78.09999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="AK13" t="n">
         <v>82.8</v>
       </c>
       <c r="AL13" t="n">
-        <v>1.92</v>
+        <v>0.61</v>
       </c>
       <c r="AM13" t="n">
-        <v>3.03</v>
+        <v>12.47</v>
       </c>
       <c r="AN13" t="n">
-        <v>8.289999999999999</v>
+        <v>17.13</v>
       </c>
       <c r="AO13" t="n">
-        <v>0.86</v>
+        <v>1.32</v>
       </c>
       <c r="AP13" t="n">
-        <v>66.3734</v>
+        <v>165.8124</v>
       </c>
       <c r="AQ13" t="n">
-        <v>64.0964</v>
+        <v>154.3136</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>62.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AU13" t="n">
-        <v>78.09999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="AV13" t="n">
         <v>82.8</v>
       </c>
       <c r="AW13" t="n">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="AX13" t="n">
-        <v>66.66</v>
+        <v>165.62</v>
       </c>
       <c r="AY13" t="n">
-        <v>67.75</v>
+        <v>169.62</v>
       </c>
       <c r="AZ13" t="n">
-        <v>1.8</v>
+        <v>0.17</v>
       </c>
       <c r="BA13" t="n">
-        <v>5.42</v>
+        <v>7.64</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3364,20 +3364,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VWCE.DE</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>72.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="F14" t="n">
-        <v>73.3</v>
+        <v>73.2</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3386,12 +3386,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 72.9; priority 73.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.7; priority 73.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3411,17 +3411,17 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 72.9, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 72.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 169.62 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 159.24 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 120.73 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -3440,15 +3440,15 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>159.24</v>
+        <v>120.73</v>
       </c>
       <c r="T14" t="n">
-        <v>169.62</v>
+        <v>129.38</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -3462,16 +3462,16 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>1.51</v>
+        <v>1.94</v>
       </c>
       <c r="Z14" t="n">
-        <v>22.03</v>
+        <v>20.76</v>
       </c>
       <c r="AA14" t="n">
-        <v>13.01</v>
+        <v>13.21</v>
       </c>
       <c r="AB14" t="n">
-        <v>-21.07</v>
+        <v>-21.63</v>
       </c>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
@@ -3482,69 +3482,69 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>Azionario globale</t>
+          <t>Azionario globale sviluppato</t>
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>166.62</v>
+        <v>126.32</v>
       </c>
       <c r="AH14" t="n">
-        <v>72.59999999999999</v>
+        <v>71.5</v>
       </c>
       <c r="AI14" t="n">
-        <v>64.3</v>
+        <v>65.2</v>
       </c>
       <c r="AJ14" t="n">
-        <v>67.5</v>
+        <v>66.8</v>
       </c>
       <c r="AK14" t="n">
         <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>2.25</v>
+        <v>0.17</v>
       </c>
       <c r="AM14" t="n">
-        <v>11.07</v>
+        <v>12.16</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.29</v>
+        <v>16.99</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.33</v>
+        <v>1.29</v>
       </c>
       <c r="AP14" t="n">
-        <v>165.768</v>
+        <v>126.2476</v>
       </c>
       <c r="AQ14" t="n">
-        <v>154.2116</v>
+        <v>117.5678</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>64.3</v>
+        <v>65.2</v>
       </c>
       <c r="AU14" t="n">
-        <v>67.5</v>
+        <v>66.8</v>
       </c>
       <c r="AV14" t="n">
         <v>82.8</v>
       </c>
       <c r="AW14" t="n">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="AX14" t="n">
-        <v>165.62</v>
+        <v>126.18</v>
       </c>
       <c r="AY14" t="n">
-        <v>169.62</v>
+        <v>129.38</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.51</v>
+        <v>0.06</v>
       </c>
       <c r="BA14" t="n">
-        <v>8.050000000000001</v>
+        <v>7.44</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3570,20 +3570,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>SXR8.DE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>72.59999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F15" t="n">
-        <v>73.09999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3592,12 +3592,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 72.6; priority 73.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.6; priority 72.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3617,17 +3617,17 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 72.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.3%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 120.73 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 681.24 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3646,15 +3646,15 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>120.73</v>
+        <v>681.24</v>
       </c>
       <c r="T15" t="n">
-        <v>129.38</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -3668,16 +3668,16 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>2.16</v>
+        <v>1.4</v>
       </c>
       <c r="Z15" t="n">
-        <v>20.14</v>
+        <v>20.59</v>
       </c>
       <c r="AA15" t="n">
-        <v>13.21</v>
+        <v>14.26</v>
       </c>
       <c r="AB15" t="n">
-        <v>-21.63</v>
+        <v>-23.32</v>
       </c>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -3688,69 +3688,69 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Azionario globale sviluppato</t>
+          <t>USA large cap</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>126.58</v>
+        <v>710.54</v>
       </c>
       <c r="AH15" t="n">
-        <v>71.5</v>
+        <v>69.2</v>
       </c>
       <c r="AI15" t="n">
-        <v>64.7</v>
+        <v>65</v>
       </c>
       <c r="AJ15" t="n">
-        <v>66.8</v>
+        <v>64.2</v>
       </c>
       <c r="AK15" t="n">
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>1.89</v>
+        <v>0.14</v>
       </c>
       <c r="AM15" t="n">
-        <v>11.14</v>
+        <v>13.23</v>
       </c>
       <c r="AN15" t="n">
-        <v>17.07</v>
+        <v>17.56</v>
       </c>
       <c r="AO15" t="n">
-        <v>1.29</v>
+        <v>1.23</v>
       </c>
       <c r="AP15" t="n">
-        <v>126.1956</v>
+        <v>709.9503999999999</v>
       </c>
       <c r="AQ15" t="n">
-        <v>117.495</v>
+        <v>659.5874</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>64.7</v>
+        <v>65</v>
       </c>
       <c r="AU15" t="n">
-        <v>66.8</v>
+        <v>64.2</v>
       </c>
       <c r="AV15" t="n">
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="AX15" t="n">
-        <v>126.18</v>
+        <v>707.24</v>
       </c>
       <c r="AY15" t="n">
-        <v>129.38</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.3</v>
+        <v>0.08</v>
       </c>
       <c r="BA15" t="n">
-        <v>7.73</v>
+        <v>7.72</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3776,20 +3776,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SXR8.DE</t>
+          <t>EIMI.MI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>71.59999999999999</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>72.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3798,12 +3798,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 71.6; priority 72.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.1; priority 72.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3818,22 +3818,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.3%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 71.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.8%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 50.73 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 681.24 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 43.98 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3852,15 +3852,15 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>681.24</v>
+        <v>43.985</v>
       </c>
       <c r="T16" t="n">
-        <v>727.1799999999999</v>
+        <v>50.73</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -3874,16 +3874,16 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>1.42</v>
+        <v>-2.09</v>
       </c>
       <c r="Z16" t="n">
-        <v>19.94</v>
+        <v>35.75</v>
       </c>
       <c r="AA16" t="n">
-        <v>14.27</v>
+        <v>17.06</v>
       </c>
       <c r="AB16" t="n">
-        <v>-23.32</v>
+        <v>-19.17</v>
       </c>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
@@ -3894,17 +3894,17 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>USA large cap</t>
+          <t>Mercati emergenti</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>711.72</v>
+        <v>47.24</v>
       </c>
       <c r="AH16" t="n">
-        <v>69.40000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AI16" t="n">
-        <v>64.8</v>
+        <v>65.3</v>
       </c>
       <c r="AJ16" t="n">
         <v>64.2</v>
@@ -3913,29 +3913,29 @@
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>2.22</v>
+        <v>3.93</v>
       </c>
       <c r="AM16" t="n">
-        <v>13.04</v>
+        <v>15.42</v>
       </c>
       <c r="AN16" t="n">
-        <v>17.64</v>
+        <v>18.48</v>
       </c>
       <c r="AO16" t="n">
-        <v>1.24</v>
+        <v>1.08</v>
       </c>
       <c r="AP16" t="n">
-        <v>709.6932</v>
+        <v>46.8739</v>
       </c>
       <c r="AQ16" t="n">
-        <v>659.191</v>
+        <v>43.4172</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>64.8</v>
+        <v>65.3</v>
       </c>
       <c r="AU16" t="n">
         <v>64.2</v>
@@ -3944,19 +3944,19 @@
         <v>82.8</v>
       </c>
       <c r="AW16" t="n">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="AX16" t="n">
-        <v>707.24</v>
+        <v>46.37</v>
       </c>
       <c r="AY16" t="n">
-        <v>727.1799999999999</v>
+        <v>48.005</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.29</v>
+        <v>0.78</v>
       </c>
       <c r="BA16" t="n">
-        <v>7.97</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -3982,20 +3982,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EIMI.MI</t>
+          <t>EXSA.DE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
+          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>70.5</v>
+        <v>70.3</v>
       </c>
       <c r="F17" t="n">
-        <v>71.40000000000001</v>
+        <v>72</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 65.95. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 70.5; priority 71.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 70.3; priority 72.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4024,22 +4024,22 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 70.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.7%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 70.3, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.2%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 50.73 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 65.95 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 43.98 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 61.47 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4054,19 +4054,19 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>43.985</v>
+        <v>61.4745</v>
       </c>
       <c r="T17" t="n">
-        <v>50.73</v>
+        <v>65.95</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
+          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -4080,16 +4080,16 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>-2.52</v>
+        <v>3.78</v>
       </c>
       <c r="Z17" t="n">
-        <v>36.09</v>
+        <v>20.12</v>
       </c>
       <c r="AA17" t="n">
-        <v>17.05</v>
+        <v>12.77</v>
       </c>
       <c r="AB17" t="n">
-        <v>-19.17</v>
+        <v>-16.33</v>
       </c>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -4100,69 +4100,69 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Mercati emergenti</t>
+          <t>Europa</t>
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>47.685</v>
+        <v>64.55</v>
       </c>
       <c r="AH17" t="n">
-        <v>67.7</v>
+        <v>72.5</v>
       </c>
       <c r="AI17" t="n">
-        <v>62.1</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AJ17" t="n">
-        <v>64.2</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>82.8</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AL17" t="n">
-        <v>5.13</v>
+        <v>-0.77</v>
       </c>
       <c r="AM17" t="n">
-        <v>11.09</v>
+        <v>7.67</v>
       </c>
       <c r="AN17" t="n">
-        <v>19</v>
+        <v>15.26</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.11</v>
+        <v>1.2</v>
       </c>
       <c r="AP17" t="n">
-        <v>46.9043</v>
+        <v>64.7086</v>
       </c>
       <c r="AQ17" t="n">
-        <v>43.377</v>
+        <v>60.8023</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT17" t="n">
-        <v>62.1</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AU17" t="n">
-        <v>64.2</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>82.8</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AW17" t="n">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="AX17" t="n">
-        <v>46.37</v>
+        <v>64.55</v>
       </c>
       <c r="AY17" t="n">
-        <v>48.005</v>
+        <v>65.95</v>
       </c>
       <c r="AZ17" t="n">
-        <v>1.66</v>
+        <v>-0.25</v>
       </c>
       <c r="BA17" t="n">
-        <v>9.93</v>
+        <v>6.16</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4202,10 +4202,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>70.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>70.5</v>
+        <v>71.2</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 70.7; priority 70.5; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 71.4; priority 71.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>AAPL: scenario base Accumulate Carefully, score 70.7, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 4.0%.</t>
+          <t>AAPL: scenario base Accumulate Carefully, score 71.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.6%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -4286,22 +4286,22 @@
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>3.24</v>
+        <v>4.72</v>
       </c>
       <c r="Z18" t="n">
-        <v>40.58</v>
+        <v>41.83</v>
       </c>
       <c r="AA18" t="n">
-        <v>26.9</v>
+        <v>26.88</v>
       </c>
       <c r="AB18" t="n">
         <v>-33.36</v>
       </c>
       <c r="AC18" t="n">
-        <v>37.33</v>
+        <v>37.28</v>
       </c>
       <c r="AD18" t="n">
-        <v>34.09</v>
+        <v>34.03</v>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
@@ -4310,45 +4310,45 @@
       </c>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="n">
-        <v>325.13</v>
+        <v>324.61</v>
       </c>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
-        <v>7.25</v>
+        <v>5.01</v>
       </c>
       <c r="AM18" t="n">
-        <v>23.49</v>
+        <v>23.87</v>
       </c>
       <c r="AN18" t="n">
-        <v>20.36</v>
+        <v>20.26</v>
       </c>
       <c r="AO18" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="AP18" t="n">
-        <v>312.7607</v>
+        <v>313.372</v>
       </c>
       <c r="AQ18" t="n">
-        <v>282.6264</v>
+        <v>282.8884</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>85</v>
       </c>
       <c r="AT18" t="n">
-        <v>78.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="AU18" t="n">
-        <v>41</v>
+        <v>41.1</v>
       </c>
       <c r="AV18" t="n">
         <v>82.8</v>
       </c>
       <c r="AW18" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX18" t="n">
         <v>302.25</v>
@@ -4357,10 +4357,10 @@
         <v>325.13</v>
       </c>
       <c r="AZ18" t="n">
-        <v>3.95</v>
+        <v>3.6</v>
       </c>
       <c r="BA18" t="n">
-        <v>15.04</v>
+        <v>14.76</v>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
       <c r="BD18" t="n">
-        <v>4745005629440</v>
+        <v>4738438397952</v>
       </c>
       <c r="BE18" t="n">
         <v>27.62</v>
@@ -4388,19 +4388,19 @@
         <v>78.44</v>
       </c>
       <c r="BI18" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="BJ18" t="n">
         <v>100</v>
       </c>
       <c r="BK18" t="n">
-        <v>78.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="BL18" t="n">
-        <v>36.1</v>
+        <v>36.3</v>
       </c>
       <c r="BM18" t="n">
-        <v>41</v>
+        <v>41.1</v>
       </c>
       <c r="BN18" t="n">
         <v>82.8</v>
@@ -4430,10 +4430,10 @@
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>67.8</v>
+        <v>67.5</v>
       </c>
       <c r="F19" t="n">
-        <v>70.5</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>score 67.8; priority 70.5; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 67.5; priority 70.1; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Hold / Monitor, score 67.8, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.2%.</t>
+          <t>IWQU.MI: scenario base Hold / Monitor, score 67.5, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.5%.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 73.80 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 74.01 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -4496,7 +4496,7 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>73.8</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="T19" t="n">
         <v>78.87</v>
@@ -4518,13 +4518,13 @@
         </is>
       </c>
       <c r="Y19" t="n">
-        <v>3.95</v>
+        <v>2.91</v>
       </c>
       <c r="Z19" t="n">
-        <v>19.8</v>
+        <v>20.15</v>
       </c>
       <c r="AA19" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="AB19" t="n">
         <v>-20.6</v>
@@ -4542,65 +4542,65 @@
         </is>
       </c>
       <c r="AG19" t="n">
-        <v>77.16</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="AH19" t="n">
-        <v>64.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="AI19" t="n">
-        <v>65.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AJ19" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AK19" t="n">
-        <v>79.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="AL19" t="n">
-        <v>1.14</v>
+        <v>-0.38</v>
       </c>
       <c r="AM19" t="n">
-        <v>8.75</v>
+        <v>9.58</v>
       </c>
       <c r="AN19" t="n">
-        <v>14.58</v>
+        <v>14.46</v>
       </c>
       <c r="AO19" t="n">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="AP19" t="n">
-        <v>77.3058</v>
+        <v>77.3442</v>
       </c>
       <c r="AQ19" t="n">
-        <v>72.0343</v>
+        <v>72.0821</v>
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="n">
         <v>65</v>
       </c>
       <c r="AT19" t="n">
-        <v>65.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AU19" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AV19" t="n">
-        <v>79.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="AW19" t="n">
         <v>756</v>
       </c>
       <c r="AX19" t="n">
-        <v>77.16</v>
+        <v>76.98999999999999</v>
       </c>
       <c r="AY19" t="n">
         <v>78.87</v>
       </c>
       <c r="AZ19" t="n">
-        <v>-0.19</v>
+        <v>-0.46</v>
       </c>
       <c r="BA19" t="n">
-        <v>7.12</v>
+        <v>6.81</v>
       </c>
       <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="inlineStr"/>
@@ -4640,10 +4640,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>71.2</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>65.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 71.2; priority 65.5; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 71.6; priority 65.9; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Accumulate Carefully, score 71.2, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -4.0%.</t>
+          <t>GOOGL: scenario base Accumulate Carefully, score 71.6, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.9%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -4724,13 +4724,13 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>-7.36</v>
+        <v>-6.59</v>
       </c>
       <c r="Z20" t="n">
-        <v>57.8</v>
+        <v>59.01</v>
       </c>
       <c r="AA20" t="n">
-        <v>30.61</v>
+        <v>30.59</v>
       </c>
       <c r="AB20" t="n">
         <v>-29.81</v>
@@ -4739,7 +4739,7 @@
         <v>16.82</v>
       </c>
       <c r="AD20" t="n">
-        <v>22.59</v>
+        <v>22.61</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
@@ -4748,57 +4748,57 @@
       </c>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="n">
-        <v>335.02</v>
+        <v>335.12</v>
       </c>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>-10.3</v>
+        <v>-11.26</v>
       </c>
       <c r="AM20" t="n">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
       <c r="AN20" t="n">
-        <v>35.8</v>
+        <v>35.76</v>
       </c>
       <c r="AO20" t="n">
         <v>1.17</v>
       </c>
       <c r="AP20" t="n">
-        <v>348.9108</v>
+        <v>348.6906</v>
       </c>
       <c r="AQ20" t="n">
-        <v>334.8123</v>
+        <v>335.0978</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>65</v>
       </c>
       <c r="AT20" t="n">
-        <v>60.4</v>
+        <v>61.9</v>
       </c>
       <c r="AU20" t="n">
         <v>39.4</v>
       </c>
       <c r="AV20" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="AW20" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX20" t="n">
         <v>335.02</v>
       </c>
       <c r="AY20" t="n">
-        <v>362.43</v>
+        <v>357.75</v>
       </c>
       <c r="AZ20" t="n">
-        <v>-3.98</v>
+        <v>-3.89</v>
       </c>
       <c r="BA20" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="BD20" t="n">
-        <v>4097272709120</v>
+        <v>4099535273984</v>
       </c>
       <c r="BE20" t="n">
         <v>54.77</v>
@@ -4826,13 +4826,13 @@
         <v>18.86</v>
       </c>
       <c r="BI20" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="BJ20" t="n">
         <v>100</v>
       </c>
       <c r="BK20" t="n">
-        <v>60.4</v>
+        <v>61.9</v>
       </c>
       <c r="BL20" t="n">
         <v>76.40000000000001</v>
@@ -4841,7 +4841,7 @@
         <v>39.4</v>
       </c>
       <c r="BN20" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="BO20" t="inlineStr"/>
       <c r="BP20" t="inlineStr">
@@ -4872,10 +4872,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>70</v>
+        <v>71.3</v>
       </c>
       <c r="F21" t="n">
-        <v>52</v>
+        <v>52.8</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 70.0; priority 52.0; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 71.3; priority 52.8; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 70.0, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 4.1%.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 71.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.0%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4956,22 +4956,22 @@
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>-2.3</v>
+        <v>2.38</v>
       </c>
       <c r="Z21" t="n">
-        <v>25</v>
+        <v>28.76</v>
       </c>
       <c r="AA21" t="n">
-        <v>46.96</v>
+        <v>46.93</v>
       </c>
       <c r="AB21" t="n">
         <v>-36.88</v>
       </c>
       <c r="AC21" t="n">
-        <v>27.52</v>
+        <v>27.76</v>
       </c>
       <c r="AD21" t="n">
-        <v>14.12</v>
+        <v>14.25</v>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
@@ -4980,45 +4980,45 @@
       </c>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="n">
-        <v>217.44</v>
+        <v>219.6045</v>
       </c>
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="n">
-        <v>5.23</v>
+        <v>3.62</v>
       </c>
       <c r="AM21" t="n">
-        <v>20.91</v>
+        <v>20.12</v>
       </c>
       <c r="AN21" t="n">
-        <v>65.48999999999999</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="AP21" t="n">
-        <v>208.7976</v>
+        <v>209.1889</v>
       </c>
       <c r="AQ21" t="n">
-        <v>195.9239</v>
+        <v>196.0888</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
         <v>85</v>
       </c>
       <c r="AT21" t="n">
-        <v>65.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="AU21" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="AV21" t="n">
-        <v>82.2</v>
+        <v>78.8</v>
       </c>
       <c r="AW21" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX21" t="n">
         <v>208.48</v>
@@ -5027,10 +5027,10 @@
         <v>227.98</v>
       </c>
       <c r="AZ21" t="n">
-        <v>4.14</v>
+        <v>4.96</v>
       </c>
       <c r="BA21" t="n">
-        <v>10.98</v>
+        <v>11.97</v>
       </c>
       <c r="BB21" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         </is>
       </c>
       <c r="BD21" t="n">
-        <v>5250523594752</v>
+        <v>5301836185600</v>
       </c>
       <c r="BE21" t="n">
         <v>63.66</v>
@@ -5064,16 +5064,16 @@
         <v>100</v>
       </c>
       <c r="BK21" t="n">
-        <v>65.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="BL21" t="n">
-        <v>76.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="BM21" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="BN21" t="n">
-        <v>82.2</v>
+        <v>78.8</v>
       </c>
       <c r="BO21" t="inlineStr"/>
       <c r="BP21" t="inlineStr">
@@ -5456,10 +5456,10 @@
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>59.6</v>
+        <v>59.5</v>
       </c>
       <c r="F24" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>score 59.6; priority 61.9; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 59.5; priority 61.8; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 59.6, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.7%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 59.5, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.2%.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -5544,13 +5544,13 @@
         </is>
       </c>
       <c r="Y24" t="n">
-        <v>-1.65</v>
+        <v>-2.55</v>
       </c>
       <c r="Z24" t="n">
-        <v>28.76</v>
+        <v>27.19</v>
       </c>
       <c r="AA24" t="n">
-        <v>18.97</v>
+        <v>18.91</v>
       </c>
       <c r="AB24" t="n">
         <v>-22.72</v>
@@ -5568,13 +5568,13 @@
         </is>
       </c>
       <c r="AG24" t="n">
-        <v>362.11</v>
+        <v>360.7</v>
       </c>
       <c r="AH24" t="n">
-        <v>66.7</v>
+        <v>66.5</v>
       </c>
       <c r="AI24" t="n">
-        <v>44.7</v>
+        <v>44.1</v>
       </c>
       <c r="AJ24" t="n">
         <v>59.1</v>
@@ -5583,29 +5583,29 @@
         <v>78.2</v>
       </c>
       <c r="AL24" t="n">
-        <v>7.21</v>
+        <v>6.94</v>
       </c>
       <c r="AM24" t="n">
-        <v>-17.02</v>
+        <v>-15.16</v>
       </c>
       <c r="AN24" t="n">
-        <v>27.84</v>
+        <v>27.64</v>
       </c>
       <c r="AO24" t="n">
-        <v>1.47</v>
+        <v>1.46</v>
       </c>
       <c r="AP24" t="n">
-        <v>352.74</v>
+        <v>353.0616</v>
       </c>
       <c r="AQ24" t="n">
-        <v>373.3167</v>
+        <v>373.4025</v>
       </c>
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="n">
         <v>55</v>
       </c>
       <c r="AT24" t="n">
-        <v>44.7</v>
+        <v>44.1</v>
       </c>
       <c r="AU24" t="n">
         <v>59.1</v>
@@ -5617,16 +5617,16 @@
         <v>756</v>
       </c>
       <c r="AX24" t="n">
-        <v>340.64</v>
+        <v>354.48</v>
       </c>
       <c r="AY24" t="n">
         <v>384.93</v>
       </c>
       <c r="AZ24" t="n">
-        <v>2.66</v>
+        <v>2.16</v>
       </c>
       <c r="BA24" t="n">
-        <v>-3</v>
+        <v>-3.4</v>
       </c>
       <c r="BB24" t="inlineStr"/>
       <c r="BC24" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v9_1_investing_ui_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -780,10 +780,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>69.40000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>67.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 69.4; priority 67.3; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 69.6; priority 67.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>AMZN: scenario base Accumulate Carefully, score 69.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.6%.</t>
+          <t>AMZN: scenario base Accumulate Carefully, score 69.6, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 1.1%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -864,10 +864,10 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>1.76</v>
+        <v>2.24</v>
       </c>
       <c r="Z2" t="n">
-        <v>12.9</v>
+        <v>13.44</v>
       </c>
       <c r="AA2" t="n">
         <v>32.4</v>
@@ -876,10 +876,10 @@
         <v>-30.88</v>
       </c>
       <c r="AC2" t="n">
-        <v>20.45</v>
+        <v>20.55</v>
       </c>
       <c r="AD2" t="n">
-        <v>24.47</v>
+        <v>24.59</v>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
@@ -888,36 +888,36 @@
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="n">
-        <v>254.41</v>
+        <v>255.615</v>
       </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="n">
-        <v>-8.289999999999999</v>
+        <v>-7.86</v>
       </c>
       <c r="AM2" t="n">
-        <v>17.34</v>
+        <v>17.89</v>
       </c>
       <c r="AN2" t="n">
-        <v>22.97</v>
+        <v>23.16</v>
       </c>
       <c r="AO2" t="n">
         <v>0.71</v>
       </c>
       <c r="AP2" t="n">
-        <v>252.8154</v>
+        <v>252.8395</v>
       </c>
       <c r="AQ2" t="n">
-        <v>238.8707</v>
+        <v>238.8768</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>66.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="AU2" t="n">
         <v>36.4</v>
@@ -929,16 +929,16 @@
         <v>752</v>
       </c>
       <c r="AX2" t="n">
-        <v>254.41</v>
+        <v>254.92</v>
       </c>
       <c r="AY2" t="n">
         <v>278.09</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.63</v>
+        <v>1.09</v>
       </c>
       <c r="BA2" t="n">
-        <v>6.51</v>
+        <v>7</v>
       </c>
       <c r="BB2" t="inlineStr">
         <is>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="BD2" t="n">
-        <v>2743822450688</v>
+        <v>2756873814016</v>
       </c>
       <c r="BE2" t="n">
         <v>17.44</v>
@@ -970,10 +970,10 @@
         <v>86.40000000000001</v>
       </c>
       <c r="BK2" t="n">
-        <v>66.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="BL2" t="n">
-        <v>69.5</v>
+        <v>69.2</v>
       </c>
       <c r="BM2" t="n">
         <v>36.4</v>
@@ -1006,10 +1006,10 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>61.7</v>
+        <v>61.4</v>
       </c>
       <c r="F3" t="n">
-        <v>65.8</v>
+        <v>65.5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>score 61.7; priority 65.8; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 61.4; priority 65.5; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Hold / Monitor, score 61.7, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.5%.</t>
+          <t>RBOT.MI: scenario base Hold / Monitor, score 61.4, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.9%.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1094,13 +1094,13 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>-0.75</v>
+        <v>-1.08</v>
       </c>
       <c r="Z3" t="n">
-        <v>37.46</v>
+        <v>37</v>
       </c>
       <c r="AA3" t="n">
-        <v>22.53</v>
+        <v>22.55</v>
       </c>
       <c r="AB3" t="n">
         <v>-29.37</v>
@@ -1118,65 +1118,65 @@
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>17.938</v>
+        <v>17.878</v>
       </c>
       <c r="AH3" t="n">
-        <v>50.6</v>
+        <v>50.4</v>
       </c>
       <c r="AI3" t="n">
-        <v>75.3</v>
+        <v>74.5</v>
       </c>
       <c r="AJ3" t="n">
-        <v>44.5</v>
+        <v>44.4</v>
       </c>
       <c r="AK3" t="n">
-        <v>77.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.13</v>
+        <v>-0.2</v>
       </c>
       <c r="AM3" t="n">
-        <v>28.39</v>
+        <v>27.96</v>
       </c>
       <c r="AN3" t="n">
-        <v>18.68</v>
+        <v>18.55</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="AP3" t="n">
-        <v>18.2174</v>
+        <v>18.2162</v>
       </c>
       <c r="AQ3" t="n">
-        <v>15.8302</v>
+        <v>15.8299</v>
       </c>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="n">
         <v>65</v>
       </c>
       <c r="AT3" t="n">
-        <v>75.3</v>
+        <v>74.5</v>
       </c>
       <c r="AU3" t="n">
-        <v>49.5</v>
+        <v>49.4</v>
       </c>
       <c r="AV3" t="n">
-        <v>77.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="AW3" t="n">
         <v>756</v>
       </c>
       <c r="AX3" t="n">
-        <v>17.938</v>
+        <v>17.878</v>
       </c>
       <c r="AY3" t="n">
         <v>19.25</v>
       </c>
       <c r="AZ3" t="n">
-        <v>-1.53</v>
+        <v>-1.86</v>
       </c>
       <c r="BA3" t="n">
-        <v>13.32</v>
+        <v>12.94</v>
       </c>
       <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="inlineStr"/>
@@ -1216,10 +1216,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>65.3</v>
+        <v>64.7</v>
       </c>
       <c r="F4" t="n">
-        <v>51.3</v>
+        <v>50.3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 65.3; priority 51.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 64.7; priority 50.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>prezzo 5.9% sotto MA50: attendere recupero</t>
+          <t>prezzo 6.7% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 65.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.9%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 64.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -6.7%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1300,10 +1300,10 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>-1.4</v>
+        <v>-2.32</v>
       </c>
       <c r="Z4" t="n">
-        <v>119.54</v>
+        <v>117.5</v>
       </c>
       <c r="AA4" t="n">
         <v>39.53</v>
@@ -1312,10 +1312,10 @@
         <v>-44.77</v>
       </c>
       <c r="AC4" t="n">
-        <v>56.67</v>
+        <v>56.14</v>
       </c>
       <c r="AD4" t="n">
-        <v>27.85</v>
+        <v>27.59</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1324,57 +1324,57 @@
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>1440</v>
+        <v>1426.6</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>-2.21</v>
+        <v>-3.12</v>
       </c>
       <c r="AM4" t="n">
-        <v>21.83</v>
+        <v>20.7</v>
       </c>
       <c r="AN4" t="n">
-        <v>33.32</v>
+        <v>32.91</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="AP4" t="n">
-        <v>1529.8342</v>
+        <v>1529.5662</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1275.1098</v>
+        <v>1275.0428</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
         <v>65</v>
       </c>
       <c r="AT4" t="n">
-        <v>91</v>
+        <v>88.5</v>
       </c>
       <c r="AU4" t="n">
         <v>16.7</v>
       </c>
       <c r="AV4" t="n">
-        <v>70.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="AW4" t="n">
         <v>765</v>
       </c>
       <c r="AX4" t="n">
-        <v>1435.4</v>
+        <v>1426.6</v>
       </c>
       <c r="AY4" t="n">
         <v>1621.2</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-5.87</v>
+        <v>-6.73</v>
       </c>
       <c r="BA4" t="n">
-        <v>12.93</v>
+        <v>11.89</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>553103982592</v>
+        <v>547957047296</v>
       </c>
       <c r="BE4" t="n">
         <v>30.11</v>
@@ -1408,16 +1408,16 @@
         <v>100</v>
       </c>
       <c r="BK4" t="n">
-        <v>91</v>
+        <v>88.5</v>
       </c>
       <c r="BL4" t="n">
-        <v>24.5</v>
+        <v>24.9</v>
       </c>
       <c r="BM4" t="n">
         <v>16.7</v>
       </c>
       <c r="BN4" t="n">
-        <v>70.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>57</v>
+        <v>56.9</v>
       </c>
       <c r="F5" t="n">
         <v>47</v>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 57.0; priority 47.0; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 56.9; priority 47.0; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>prezzo 5.6% sotto MA50: attendere recupero</t>
+          <t>prezzo 5.0% sotto MA50: attendere recupero</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>SMH: scenario base Hold / Monitor, score 57.0, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.6%.</t>
+          <t>SMH: scenario base Hold / Monitor, score 56.9, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -5.0%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>-13.7</v>
+        <v>-14.14</v>
       </c>
       <c r="Z5" t="n">
-        <v>88.52</v>
+        <v>91.78</v>
       </c>
       <c r="AA5" t="n">
         <v>36.93</v>
@@ -1556,53 +1556,53 @@
         </is>
       </c>
       <c r="AG5" t="n">
-        <v>545.5700000000001</v>
+        <v>547.7098999999999</v>
       </c>
       <c r="AH5" t="n">
         <v>52</v>
       </c>
       <c r="AI5" t="n">
-        <v>76.7</v>
+        <v>75.5</v>
       </c>
       <c r="AJ5" t="n">
         <v>22.1</v>
       </c>
       <c r="AK5" t="n">
-        <v>71.3</v>
+        <v>72.2</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.02</v>
+        <v>-4.86</v>
       </c>
       <c r="AM5" t="n">
-        <v>39.51</v>
+        <v>37.24</v>
       </c>
       <c r="AN5" t="n">
-        <v>52.71</v>
+        <v>52.83</v>
       </c>
       <c r="AO5" t="n">
         <v>1.43</v>
       </c>
       <c r="AP5" t="n">
-        <v>577.9704</v>
+        <v>576.6344</v>
       </c>
       <c r="AQ5" t="n">
-        <v>474.0167</v>
+        <v>475.0742</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
         <v>65</v>
       </c>
       <c r="AT5" t="n">
-        <v>76.7</v>
+        <v>75.5</v>
       </c>
       <c r="AU5" t="n">
         <v>27.1</v>
       </c>
       <c r="AV5" t="n">
-        <v>71.3</v>
+        <v>72.2</v>
       </c>
       <c r="AW5" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="AX5" t="n">
         <v>545.22</v>
@@ -1611,10 +1611,10 @@
         <v>594.0700000000001</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-5.61</v>
+        <v>-5.02</v>
       </c>
       <c r="BA5" t="n">
-        <v>15.1</v>
+        <v>15.29</v>
       </c>
       <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr"/>
@@ -1654,10 +1654,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>60.7</v>
+        <v>62.7</v>
       </c>
       <c r="F6" t="n">
-        <v>42.6</v>
+        <v>45</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 60.7; priority 42.6; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 62.7; priority 45.0; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1686,12 +1686,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>META: scenario base Hold / Monitor, score 60.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.6%.</t>
+          <t>META: scenario base Hold / Monitor, score 62.7, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.9%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="S6" t="n">
@@ -1738,22 +1738,22 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-5.33</v>
+        <v>-3.9</v>
       </c>
       <c r="Z6" t="n">
-        <v>-19.58</v>
+        <v>-18.37</v>
       </c>
       <c r="AA6" t="n">
-        <v>37.49</v>
+        <v>37.52</v>
       </c>
       <c r="AB6" t="n">
         <v>-34.15</v>
       </c>
       <c r="AC6" t="n">
-        <v>22.19</v>
+        <v>22.54</v>
       </c>
       <c r="AD6" t="n">
-        <v>16.86</v>
+        <v>17.12</v>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
@@ -1762,42 +1762,42 @@
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>589.2495</v>
+        <v>598.13</v>
       </c>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>0.22</v>
+        <v>1.73</v>
       </c>
       <c r="AM6" t="n">
-        <v>-11.6</v>
+        <v>-10.26</v>
       </c>
       <c r="AN6" t="n">
-        <v>25.73</v>
+        <v>26.36</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="AP6" t="n">
-        <v>592.8814</v>
+        <v>593.059</v>
       </c>
       <c r="AQ6" t="n">
-        <v>621.4931</v>
+        <v>621.5375</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="AT6" t="n">
-        <v>30.7</v>
+        <v>33.8</v>
       </c>
       <c r="AU6" t="n">
         <v>27.7</v>
       </c>
       <c r="AV6" t="n">
-        <v>74.3</v>
+        <v>78.2</v>
       </c>
       <c r="AW6" t="n">
         <v>752</v>
@@ -1809,10 +1809,10 @@
         <v>599.12</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-0.61</v>
+        <v>0.9</v>
       </c>
       <c r="BA6" t="n">
-        <v>-5.19</v>
+        <v>-3.72</v>
       </c>
       <c r="BB6" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="BD6" t="n">
-        <v>1501118070784</v>
+        <v>1524325810176</v>
       </c>
       <c r="BE6" t="n">
         <v>29.83</v>
@@ -1846,16 +1846,16 @@
         <v>100</v>
       </c>
       <c r="BK6" t="n">
-        <v>30.7</v>
+        <v>33.8</v>
       </c>
       <c r="BL6" t="n">
-        <v>78.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BM6" t="n">
         <v>27.7</v>
       </c>
       <c r="BN6" t="n">
-        <v>74.3</v>
+        <v>78.2</v>
       </c>
       <c r="BO6" t="inlineStr"/>
       <c r="BP6" t="inlineStr">
@@ -1882,10 +1882,10 @@
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="F7" t="n">
-        <v>41.6</v>
+        <v>41.4</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 35.9; priority 41.6; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 35.8; priority 41.4; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>prezzo 7.8% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo 8.0% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 35.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -7.8%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 35.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -8.0%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 8.53 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>8.539999999999999</v>
+        <v>8.525</v>
       </c>
       <c r="T7" t="n">
         <v>10.872</v>
@@ -1970,13 +1970,13 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>-24.1</v>
+        <v>-24.24</v>
       </c>
       <c r="Z7" t="n">
-        <v>21.47</v>
+        <v>21.26</v>
       </c>
       <c r="AA7" t="n">
-        <v>24.13</v>
+        <v>24.14</v>
       </c>
       <c r="AB7" t="n">
         <v>-34.68</v>
@@ -1994,34 +1994,34 @@
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>8.539999999999999</v>
+        <v>8.525</v>
       </c>
       <c r="AH7" t="n">
         <v>33.4</v>
       </c>
       <c r="AI7" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="AJ7" t="n">
         <v>38.3</v>
       </c>
       <c r="AK7" t="n">
-        <v>63.5</v>
+        <v>63.3</v>
       </c>
       <c r="AL7" t="n">
-        <v>-5.35</v>
+        <v>-5.52</v>
       </c>
       <c r="AM7" t="n">
-        <v>-1.92</v>
+        <v>-2.09</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.16</v>
+        <v>1.1</v>
       </c>
       <c r="AO7" t="n">
         <v>0.05</v>
       </c>
       <c r="AP7" t="n">
-        <v>9.266500000000001</v>
+        <v>9.2662</v>
       </c>
       <c r="AQ7" t="n">
         <v>9.281000000000001</v>
@@ -2031,28 +2031,28 @@
         <v>35</v>
       </c>
       <c r="AT7" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="AU7" t="n">
         <v>43.3</v>
       </c>
       <c r="AV7" t="n">
-        <v>63.5</v>
+        <v>63.3</v>
       </c>
       <c r="AW7" t="n">
         <v>756</v>
       </c>
       <c r="AX7" t="n">
-        <v>8.539999999999999</v>
+        <v>8.525</v>
       </c>
       <c r="AY7" t="n">
         <v>9.217000000000001</v>
       </c>
       <c r="AZ7" t="n">
-        <v>-7.84</v>
+        <v>-8</v>
       </c>
       <c r="BA7" t="n">
-        <v>-7.98</v>
+        <v>-8.15</v>
       </c>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
@@ -2088,10 +2088,10 @@
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>53.7</v>
+        <v>54.5</v>
       </c>
       <c r="F8" t="n">
-        <v>29</v>
+        <v>33.5</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>score 53.7; priority 29.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
+          <t>score 54.5; priority 33.5; trend: Bullish; entry zone: Extended - wait pullback; risk flag: High risk</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>prezzo 13.7% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 12.2% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base High Risk, score 53.7, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 13.7%.</t>
+          <t>WCLD.MI: scenario base High Risk, score 54.5, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 12.2%.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -2176,13 +2176,13 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>23.65</v>
+        <v>22.03</v>
       </c>
       <c r="Z8" t="n">
-        <v>17.12</v>
+        <v>15.58</v>
       </c>
       <c r="AA8" t="n">
-        <v>35.07</v>
+        <v>35.11</v>
       </c>
       <c r="AB8" t="n">
         <v>-48.6</v>
@@ -2200,10 +2200,10 @@
         </is>
       </c>
       <c r="AG8" t="n">
-        <v>35.34</v>
+        <v>34.875</v>
       </c>
       <c r="AH8" t="n">
-        <v>26.2</v>
+        <v>26</v>
       </c>
       <c r="AI8" t="n">
         <v>100</v>
@@ -2212,25 +2212,25 @@
         <v>14</v>
       </c>
       <c r="AK8" t="n">
-        <v>44.1</v>
+        <v>49.9</v>
       </c>
       <c r="AL8" t="n">
-        <v>13.02</v>
+        <v>11.53</v>
       </c>
       <c r="AM8" t="n">
-        <v>49.68</v>
+        <v>47.71</v>
       </c>
       <c r="AN8" t="n">
-        <v>6.41</v>
+        <v>5.94</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="AP8" t="n">
-        <v>31.0894</v>
+        <v>31.0801</v>
       </c>
       <c r="AQ8" t="n">
-        <v>27.0478</v>
+        <v>27.0455</v>
       </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="n">
@@ -2243,7 +2243,7 @@
         <v>19</v>
       </c>
       <c r="AV8" t="n">
-        <v>44.1</v>
+        <v>49.9</v>
       </c>
       <c r="AW8" t="n">
         <v>757</v>
@@ -2255,10 +2255,10 @@
         <v>36.89</v>
       </c>
       <c r="AZ8" t="n">
-        <v>13.67</v>
+        <v>12.21</v>
       </c>
       <c r="BA8" t="n">
-        <v>30.66</v>
+        <v>28.95</v>
       </c>
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr"/>
@@ -2298,10 +2298,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>23.8</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 31.9; priority 24.0; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
+          <t>score 31.8; priority 23.8; trend: Weak; entry zone: Wait for trend repair; risk flag: High risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>TSLA: scenario base High Risk, score 31.9, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -1.1%.</t>
+          <t>TSLA: scenario base High Risk, score 31.8, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -1.3%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -2382,10 +2382,10 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>-16.36</v>
+        <v>-16.55</v>
       </c>
       <c r="Z9" t="n">
-        <v>7.6</v>
+        <v>7.35</v>
       </c>
       <c r="AA9" t="n">
         <v>58.28</v>
@@ -2394,10 +2394,10 @@
         <v>-53.77</v>
       </c>
       <c r="AC9" t="n">
-        <v>331.21</v>
+        <v>330.39</v>
       </c>
       <c r="AD9" t="n">
-        <v>164.18</v>
+        <v>163.77</v>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
@@ -2406,42 +2406,42 @@
       </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="n">
-        <v>354.39</v>
+        <v>353.57</v>
       </c>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="n">
-        <v>8.26</v>
+        <v>8.01</v>
       </c>
       <c r="AM9" t="n">
-        <v>-12.7</v>
+        <v>-12.9</v>
       </c>
       <c r="AN9" t="n">
-        <v>11.44</v>
+        <v>11.36</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="AP9" t="n">
-        <v>358.2994</v>
+        <v>358.283</v>
       </c>
       <c r="AQ9" t="n">
-        <v>399.9594</v>
+        <v>399.9553</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>35</v>
       </c>
       <c r="AT9" t="n">
-        <v>21.4</v>
+        <v>20.9</v>
       </c>
       <c r="AU9" t="n">
         <v>0</v>
       </c>
       <c r="AV9" t="n">
-        <v>73.59999999999999</v>
+        <v>73.3</v>
       </c>
       <c r="AW9" t="n">
         <v>752</v>
@@ -2453,10 +2453,10 @@
         <v>367.95</v>
       </c>
       <c r="AZ9" t="n">
-        <v>-1.09</v>
+        <v>-1.33</v>
       </c>
       <c r="BA9" t="n">
-        <v>-11.39</v>
+        <v>-11.61</v>
       </c>
       <c r="BB9" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="BD9" t="n">
-        <v>1399680139264</v>
+        <v>1396243955712</v>
       </c>
       <c r="BE9" t="n">
         <v>3.67</v>
@@ -2488,7 +2488,7 @@
         <v>69.90000000000001</v>
       </c>
       <c r="BK9" t="n">
-        <v>21.4</v>
+        <v>20.9</v>
       </c>
       <c r="BL9" t="n">
         <v>0</v>
@@ -2497,7 +2497,7 @@
         <v>0</v>
       </c>
       <c r="BN9" t="n">
-        <v>73.59999999999999</v>
+        <v>73.3</v>
       </c>
       <c r="BO9" t="inlineStr"/>
       <c r="BP9" t="inlineStr">
@@ -2612,10 +2612,10 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="Z10" t="n">
-        <v>56.31</v>
+        <v>56.37</v>
       </c>
       <c r="AA10" t="n">
         <v>14.13</v>
@@ -2636,13 +2636,13 @@
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>72.59</v>
+        <v>72.62</v>
       </c>
       <c r="AH10" t="n">
         <v>77.2</v>
       </c>
       <c r="AI10" t="n">
-        <v>83.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="AJ10" t="n">
         <v>68.8</v>
@@ -2651,29 +2651,29 @@
         <v>82.8</v>
       </c>
       <c r="AL10" t="n">
-        <v>2.98</v>
+        <v>3.02</v>
       </c>
       <c r="AM10" t="n">
-        <v>28.91</v>
+        <v>28.96</v>
       </c>
       <c r="AN10" t="n">
-        <v>25.53</v>
+        <v>25.54</v>
       </c>
       <c r="AO10" t="n">
         <v>1.81</v>
       </c>
       <c r="AP10" t="n">
-        <v>71.6172</v>
+        <v>71.6178</v>
       </c>
       <c r="AQ10" t="n">
-        <v>61.8725</v>
+        <v>61.8727</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
         <v>85</v>
       </c>
       <c r="AT10" t="n">
-        <v>83.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="AU10" t="n">
         <v>68.8</v>
@@ -2691,10 +2691,10 @@
         <v>73.75</v>
       </c>
       <c r="AZ10" t="n">
-        <v>1.36</v>
+        <v>1.4</v>
       </c>
       <c r="BA10" t="n">
-        <v>17.32</v>
+        <v>17.37</v>
       </c>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2734,10 +2734,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>74.2</v>
+        <v>74.3</v>
       </c>
       <c r="F11" t="n">
-        <v>52.2</v>
+        <v>51</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 74.2; priority 52.2; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Medium-high risk</t>
+          <t>score 74.3; priority 51.0; trend: Bullish; entry zone: Extended - wait pullback; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>prezzo 13.5% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 13.9% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>MSFT: scenario base Accumulate Carefully, score 74.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 13.4%.</t>
+          <t>MSFT: scenario base Accumulate Carefully, score 74.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 13.9%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2818,22 +2818,22 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>16.41</v>
+        <v>16.93</v>
       </c>
       <c r="Z11" t="n">
-        <v>-0.89</v>
+        <v>-0.45</v>
       </c>
       <c r="AA11" t="n">
-        <v>26.2</v>
+        <v>26.19</v>
       </c>
       <c r="AB11" t="n">
         <v>-34.5</v>
       </c>
       <c r="AC11" t="n">
-        <v>27.68</v>
+        <v>27.8</v>
       </c>
       <c r="AD11" t="n">
-        <v>21.06</v>
+        <v>21.16</v>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
@@ -2842,42 +2842,42 @@
       </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="n">
-        <v>496.5397</v>
+        <v>498.73</v>
       </c>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="n">
-        <v>0.95</v>
+        <v>1.39</v>
       </c>
       <c r="AM11" t="n">
-        <v>23.04</v>
+        <v>23.58</v>
       </c>
       <c r="AN11" t="n">
-        <v>15.15</v>
+        <v>15.32</v>
       </c>
       <c r="AO11" t="n">
         <v>0.58</v>
       </c>
       <c r="AP11" t="n">
-        <v>437.6989</v>
+        <v>437.7427</v>
       </c>
       <c r="AQ11" t="n">
-        <v>429.3692</v>
+        <v>429.3802</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>86.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="AU11" t="n">
         <v>41</v>
       </c>
       <c r="AV11" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="AW11" t="n">
         <v>752</v>
@@ -2889,10 +2889,10 @@
         <v>513.53</v>
       </c>
       <c r="AZ11" t="n">
-        <v>13.45</v>
+        <v>13.93</v>
       </c>
       <c r="BA11" t="n">
-        <v>15.65</v>
+        <v>16.15</v>
       </c>
       <c r="BB11" t="inlineStr">
         <is>
@@ -2905,7 +2905,7 @@
         </is>
       </c>
       <c r="BD11" t="n">
-        <v>3686783516672</v>
+        <v>3703342628864</v>
       </c>
       <c r="BE11" t="n">
         <v>40.3</v>
@@ -2926,16 +2926,16 @@
         <v>100</v>
       </c>
       <c r="BK11" t="n">
-        <v>86.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="BL11" t="n">
-        <v>66</v>
+        <v>65.7</v>
       </c>
       <c r="BM11" t="n">
         <v>41</v>
       </c>
       <c r="BN11" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="BO11" t="inlineStr"/>
       <c r="BP11" t="inlineStr">
@@ -2962,10 +2962,10 @@
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>72.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>74.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>score 72.5; priority 74.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 72.4; priority 74.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.6%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.5%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -3050,10 +3050,10 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>5.95</v>
+        <v>5.87</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.86</v>
+        <v>7.78</v>
       </c>
       <c r="AA12" t="n">
         <v>9.69</v>
@@ -3074,13 +3074,13 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>67.48999999999999</v>
+        <v>67.44</v>
       </c>
       <c r="AH12" t="n">
         <v>64.3</v>
       </c>
       <c r="AI12" t="n">
-        <v>62.4</v>
+        <v>62.2</v>
       </c>
       <c r="AJ12" t="n">
         <v>78.09999999999999</v>
@@ -3089,29 +3089,29 @@
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>1.43</v>
+        <v>1.35</v>
       </c>
       <c r="AM12" t="n">
-        <v>3.53</v>
+        <v>3.45</v>
       </c>
       <c r="AN12" t="n">
-        <v>8.33</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AO12" t="n">
         <v>0.86</v>
       </c>
       <c r="AP12" t="n">
-        <v>66.43940000000001</v>
+        <v>66.4384</v>
       </c>
       <c r="AQ12" t="n">
-        <v>64.1176</v>
+        <v>64.1173</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>62.4</v>
+        <v>62.2</v>
       </c>
       <c r="AU12" t="n">
         <v>78.09999999999999</v>
@@ -3129,10 +3129,10 @@
         <v>67.75</v>
       </c>
       <c r="AZ12" t="n">
-        <v>1.58</v>
+        <v>1.51</v>
       </c>
       <c r="BA12" t="n">
-        <v>5.26</v>
+        <v>5.18</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 73.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 73.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.3%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -3256,10 +3256,10 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="Z13" t="n">
-        <v>22.6</v>
+        <v>22.72</v>
       </c>
       <c r="AA13" t="n">
         <v>13.01</v>
@@ -3280,13 +3280,13 @@
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>166.1</v>
+        <v>166.26</v>
       </c>
       <c r="AH13" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="AI13" t="n">
-        <v>65.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="AJ13" t="n">
         <v>67.5</v>
@@ -3295,29 +3295,29 @@
         <v>82.8</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.61</v>
+        <v>0.7</v>
       </c>
       <c r="AM13" t="n">
-        <v>12.47</v>
+        <v>12.58</v>
       </c>
       <c r="AN13" t="n">
-        <v>17.13</v>
+        <v>17.17</v>
       </c>
       <c r="AO13" t="n">
         <v>1.32</v>
       </c>
       <c r="AP13" t="n">
-        <v>165.8124</v>
+        <v>165.8156</v>
       </c>
       <c r="AQ13" t="n">
-        <v>154.3136</v>
+        <v>154.3144</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>65.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="AU13" t="n">
         <v>67.5</v>
@@ -3335,10 +3335,10 @@
         <v>169.62</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="BA13" t="n">
-        <v>7.64</v>
+        <v>7.74</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3462,10 +3462,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>1.94</v>
+        <v>2</v>
       </c>
       <c r="Z14" t="n">
-        <v>20.76</v>
+        <v>20.83</v>
       </c>
       <c r="AA14" t="n">
         <v>13.21</v>
@@ -3486,13 +3486,13 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>126.32</v>
+        <v>126.39</v>
       </c>
       <c r="AH14" t="n">
         <v>71.5</v>
       </c>
       <c r="AI14" t="n">
-        <v>65.2</v>
+        <v>65.3</v>
       </c>
       <c r="AJ14" t="n">
         <v>66.8</v>
@@ -3501,29 +3501,29 @@
         <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="AM14" t="n">
-        <v>12.16</v>
+        <v>12.23</v>
       </c>
       <c r="AN14" t="n">
-        <v>16.99</v>
+        <v>17.01</v>
       </c>
       <c r="AO14" t="n">
         <v>1.29</v>
       </c>
       <c r="AP14" t="n">
-        <v>126.2476</v>
+        <v>126.249</v>
       </c>
       <c r="AQ14" t="n">
-        <v>117.5678</v>
+        <v>117.5682</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>65.2</v>
+        <v>65.3</v>
       </c>
       <c r="AU14" t="n">
         <v>66.8</v>
@@ -3541,10 +3541,10 @@
         <v>129.38</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="BA14" t="n">
-        <v>7.44</v>
+        <v>7.5</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3570,20 +3570,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SXR8.DE</t>
+          <t>EIMI.MI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>71.59999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3592,12 +3592,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 71.6; priority 72.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.4; priority 72.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3612,22 +3612,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 71.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.1%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 50.73 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 681.24 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 43.98 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3646,15 +3646,15 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>681.24</v>
+        <v>43.985</v>
       </c>
       <c r="T15" t="n">
-        <v>727.1799999999999</v>
+        <v>50.73</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -3668,16 +3668,16 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>1.4</v>
+        <v>-1.75</v>
       </c>
       <c r="Z15" t="n">
-        <v>20.59</v>
+        <v>36.22</v>
       </c>
       <c r="AA15" t="n">
-        <v>14.26</v>
+        <v>17.06</v>
       </c>
       <c r="AB15" t="n">
-        <v>-23.32</v>
+        <v>-19.17</v>
       </c>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
@@ -3688,17 +3688,17 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>USA large cap</t>
+          <t>Mercati emergenti</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>710.54</v>
+        <v>47.405</v>
       </c>
       <c r="AH15" t="n">
-        <v>69.2</v>
+        <v>67.3</v>
       </c>
       <c r="AI15" t="n">
-        <v>65</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AJ15" t="n">
         <v>64.2</v>
@@ -3707,29 +3707,29 @@
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>0.14</v>
+        <v>4.29</v>
       </c>
       <c r="AM15" t="n">
-        <v>13.23</v>
+        <v>15.82</v>
       </c>
       <c r="AN15" t="n">
-        <v>17.56</v>
+        <v>18.62</v>
       </c>
       <c r="AO15" t="n">
-        <v>1.23</v>
+        <v>1.09</v>
       </c>
       <c r="AP15" t="n">
-        <v>709.9503999999999</v>
+        <v>46.8772</v>
       </c>
       <c r="AQ15" t="n">
-        <v>659.5874</v>
+        <v>43.4181</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>65</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AU15" t="n">
         <v>64.2</v>
@@ -3738,19 +3738,19 @@
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="AX15" t="n">
-        <v>707.24</v>
+        <v>46.37</v>
       </c>
       <c r="AY15" t="n">
-        <v>727.1799999999999</v>
+        <v>48.005</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.08</v>
+        <v>1.13</v>
       </c>
       <c r="BA15" t="n">
-        <v>7.72</v>
+        <v>9.18</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3776,20 +3776,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EIMI.MI</t>
+          <t>SXR8.DE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>71.09999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>72.09999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3798,12 +3798,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 50.73. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 71.1; priority 72.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.6; priority 72.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3818,22 +3818,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 71.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.8%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 71.6, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 50.73 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 43.98 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 681.24 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3852,15 +3852,15 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>43.985</v>
+        <v>681.24</v>
       </c>
       <c r="T16" t="n">
-        <v>50.73</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>iShares Core MSCI EM IMI UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -3874,16 +3874,16 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>-2.09</v>
+        <v>1.4</v>
       </c>
       <c r="Z16" t="n">
-        <v>35.75</v>
+        <v>20.6</v>
       </c>
       <c r="AA16" t="n">
-        <v>17.06</v>
+        <v>14.26</v>
       </c>
       <c r="AB16" t="n">
-        <v>-19.17</v>
+        <v>-23.32</v>
       </c>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
@@ -3894,17 +3894,17 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Mercati emergenti</t>
+          <t>USA large cap</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>47.24</v>
+        <v>710.58</v>
       </c>
       <c r="AH16" t="n">
-        <v>67.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="AI16" t="n">
-        <v>65.3</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AJ16" t="n">
         <v>64.2</v>
@@ -3913,29 +3913,29 @@
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>3.93</v>
+        <v>0.15</v>
       </c>
       <c r="AM16" t="n">
-        <v>15.42</v>
+        <v>13.24</v>
       </c>
       <c r="AN16" t="n">
-        <v>18.48</v>
+        <v>17.56</v>
       </c>
       <c r="AO16" t="n">
-        <v>1.08</v>
+        <v>1.23</v>
       </c>
       <c r="AP16" t="n">
-        <v>46.8739</v>
+        <v>709.9512</v>
       </c>
       <c r="AQ16" t="n">
-        <v>43.4172</v>
+        <v>659.5876</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>65.3</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AU16" t="n">
         <v>64.2</v>
@@ -3944,19 +3944,19 @@
         <v>82.8</v>
       </c>
       <c r="AW16" t="n">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="AX16" t="n">
-        <v>46.37</v>
+        <v>707.24</v>
       </c>
       <c r="AY16" t="n">
-        <v>48.005</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.78</v>
+        <v>0.09</v>
       </c>
       <c r="BA16" t="n">
-        <v>8.800000000000001</v>
+        <v>7.73</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -3992,10 +3992,10 @@
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>70.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 70.3; priority 72.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 70.4; priority 72.1; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 70.3, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.2%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 70.4, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.2%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -4080,10 +4080,10 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>3.78</v>
+        <v>3.85</v>
       </c>
       <c r="Z17" t="n">
-        <v>20.12</v>
+        <v>20.2</v>
       </c>
       <c r="AA17" t="n">
         <v>12.77</v>
@@ -4104,65 +4104,65 @@
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>64.55</v>
+        <v>64.59</v>
       </c>
       <c r="AH17" t="n">
         <v>72.5</v>
       </c>
       <c r="AI17" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AJ17" t="n">
         <v>71.59999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>79.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="AL17" t="n">
-        <v>-0.77</v>
+        <v>-0.71</v>
       </c>
       <c r="AM17" t="n">
-        <v>7.67</v>
+        <v>7.73</v>
       </c>
       <c r="AN17" t="n">
-        <v>15.26</v>
+        <v>15.29</v>
       </c>
       <c r="AO17" t="n">
         <v>1.2</v>
       </c>
       <c r="AP17" t="n">
-        <v>64.7086</v>
+        <v>64.7094</v>
       </c>
       <c r="AQ17" t="n">
-        <v>60.8023</v>
+        <v>60.8025</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>65</v>
       </c>
       <c r="AT17" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="AU17" t="n">
         <v>71.59999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>79.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="AW17" t="n">
         <v>759</v>
       </c>
       <c r="AX17" t="n">
-        <v>64.55</v>
+        <v>64.59</v>
       </c>
       <c r="AY17" t="n">
         <v>65.95</v>
       </c>
       <c r="AZ17" t="n">
-        <v>-0.25</v>
+        <v>-0.18</v>
       </c>
       <c r="BA17" t="n">
-        <v>6.16</v>
+        <v>6.23</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4202,10 +4202,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>71.40000000000001</v>
+        <v>71.3</v>
       </c>
       <c r="F18" t="n">
-        <v>71.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>score 71.4; priority 71.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 71.3; priority 71.1; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>AAPL: scenario base Accumulate Carefully, score 71.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.6%.</t>
+          <t>AAPL: scenario base Accumulate Carefully, score 71.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.4%.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -4286,10 +4286,10 @@
         </is>
       </c>
       <c r="Y18" t="n">
-        <v>4.72</v>
+        <v>4.52</v>
       </c>
       <c r="Z18" t="n">
-        <v>41.83</v>
+        <v>41.56</v>
       </c>
       <c r="AA18" t="n">
         <v>26.88</v>
@@ -4298,10 +4298,10 @@
         <v>-33.36</v>
       </c>
       <c r="AC18" t="n">
-        <v>37.28</v>
+        <v>37.2</v>
       </c>
       <c r="AD18" t="n">
-        <v>34.03</v>
+        <v>33.96</v>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
@@ -4310,36 +4310,36 @@
       </c>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="n">
-        <v>324.61</v>
+        <v>324</v>
       </c>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
-        <v>5.01</v>
+        <v>4.82</v>
       </c>
       <c r="AM18" t="n">
-        <v>23.87</v>
+        <v>23.64</v>
       </c>
       <c r="AN18" t="n">
-        <v>20.26</v>
+        <v>20.19</v>
       </c>
       <c r="AO18" t="n">
         <v>0.75</v>
       </c>
       <c r="AP18" t="n">
-        <v>313.372</v>
+        <v>313.3598</v>
       </c>
       <c r="AQ18" t="n">
-        <v>282.8884</v>
+        <v>282.8853</v>
       </c>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="n">
         <v>85</v>
       </c>
       <c r="AT18" t="n">
-        <v>81.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AU18" t="n">
         <v>41.1</v>
@@ -4357,10 +4357,10 @@
         <v>325.13</v>
       </c>
       <c r="AZ18" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="BA18" t="n">
-        <v>14.76</v>
+        <v>14.53</v>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
       <c r="BD18" t="n">
-        <v>4738438397952</v>
+        <v>4728828198912</v>
       </c>
       <c r="BE18" t="n">
         <v>27.62</v>
@@ -4394,10 +4394,10 @@
         <v>100</v>
       </c>
       <c r="BK18" t="n">
-        <v>81.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="BL18" t="n">
-        <v>36.3</v>
+        <v>36.5</v>
       </c>
       <c r="BM18" t="n">
         <v>41.1</v>
@@ -4430,10 +4430,10 @@
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>70.09999999999999</v>
+        <v>70</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>score 67.5; priority 70.1; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 67.4; priority 70.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Hold / Monitor, score 67.5, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.5%.</t>
+          <t>IWQU.MI: scenario base Hold / Monitor, score 67.4, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.5%.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -4518,10 +4518,10 @@
         </is>
       </c>
       <c r="Y19" t="n">
-        <v>2.91</v>
+        <v>2.89</v>
       </c>
       <c r="Z19" t="n">
-        <v>20.15</v>
+        <v>20.12</v>
       </c>
       <c r="AA19" t="n">
         <v>12.87</v>
@@ -4542,65 +4542,65 @@
         </is>
       </c>
       <c r="AG19" t="n">
-        <v>76.98999999999999</v>
+        <v>76.97</v>
       </c>
       <c r="AH19" t="n">
         <v>64.09999999999999</v>
       </c>
       <c r="AI19" t="n">
-        <v>64.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AJ19" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AK19" t="n">
-        <v>79.09999999999999</v>
+        <v>79</v>
       </c>
       <c r="AL19" t="n">
-        <v>-0.38</v>
+        <v>-0.4</v>
       </c>
       <c r="AM19" t="n">
-        <v>9.58</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="AN19" t="n">
-        <v>14.46</v>
+        <v>14.45</v>
       </c>
       <c r="AO19" t="n">
         <v>1.12</v>
       </c>
       <c r="AP19" t="n">
-        <v>77.3442</v>
+        <v>77.3438</v>
       </c>
       <c r="AQ19" t="n">
-        <v>72.0821</v>
+        <v>72.08199999999999</v>
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="n">
         <v>65</v>
       </c>
       <c r="AT19" t="n">
-        <v>64.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AU19" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AV19" t="n">
-        <v>79.09999999999999</v>
+        <v>79</v>
       </c>
       <c r="AW19" t="n">
         <v>756</v>
       </c>
       <c r="AX19" t="n">
-        <v>76.98999999999999</v>
+        <v>76.97</v>
       </c>
       <c r="AY19" t="n">
         <v>78.87</v>
       </c>
       <c r="AZ19" t="n">
-        <v>-0.46</v>
+        <v>-0.48</v>
       </c>
       <c r="BA19" t="n">
-        <v>6.81</v>
+        <v>6.78</v>
       </c>
       <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="inlineStr"/>
@@ -4640,10 +4640,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>71.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="F20" t="n">
-        <v>65.90000000000001</v>
+        <v>67</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 71.6; priority 65.9; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 72.3; priority 67.0; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Accumulate Carefully, score 71.6, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.9%.</t>
+          <t>GOOGL: scenario base Accumulate Carefully, score 72.3, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.8%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -4724,22 +4724,22 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>-6.59</v>
+        <v>-5.54</v>
       </c>
       <c r="Z20" t="n">
-        <v>59.01</v>
+        <v>60.8</v>
       </c>
       <c r="AA20" t="n">
-        <v>30.59</v>
+        <v>30.6</v>
       </c>
       <c r="AB20" t="n">
         <v>-29.81</v>
       </c>
       <c r="AC20" t="n">
-        <v>16.82</v>
+        <v>17.01</v>
       </c>
       <c r="AD20" t="n">
-        <v>22.61</v>
+        <v>22.86</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
@@ -4748,42 +4748,42 @@
       </c>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="n">
-        <v>335.12</v>
+        <v>338.89</v>
       </c>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>-11.26</v>
+        <v>-10.26</v>
       </c>
       <c r="AM20" t="n">
-        <v>10.7</v>
+        <v>11.94</v>
       </c>
       <c r="AN20" t="n">
-        <v>35.76</v>
+        <v>36.27</v>
       </c>
       <c r="AO20" t="n">
-        <v>1.17</v>
+        <v>1.19</v>
       </c>
       <c r="AP20" t="n">
-        <v>348.6906</v>
+        <v>348.766</v>
       </c>
       <c r="AQ20" t="n">
-        <v>335.0978</v>
+        <v>335.1167</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>65</v>
       </c>
       <c r="AT20" t="n">
-        <v>61.9</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="AU20" t="n">
         <v>39.4</v>
       </c>
       <c r="AV20" t="n">
-        <v>73.90000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="AW20" t="n">
         <v>752</v>
@@ -4795,10 +4795,10 @@
         <v>357.75</v>
       </c>
       <c r="AZ20" t="n">
-        <v>-3.89</v>
+        <v>-2.83</v>
       </c>
       <c r="BA20" t="n">
-        <v>0.01</v>
+        <v>1.13</v>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="BD20" t="n">
-        <v>4099535273984</v>
+        <v>4145458708480</v>
       </c>
       <c r="BE20" t="n">
         <v>54.77</v>
@@ -4832,16 +4832,16 @@
         <v>100</v>
       </c>
       <c r="BK20" t="n">
-        <v>61.9</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="BL20" t="n">
-        <v>76.40000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="BM20" t="n">
         <v>39.4</v>
       </c>
       <c r="BN20" t="n">
-        <v>73.90000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="BO20" t="inlineStr"/>
       <c r="BP20" t="inlineStr">
@@ -4853,53 +4853,49 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2. Rischio da controllare</t>
+          <t>4. Alert / monitoraggio</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SGLD.MI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>Invesco Physical Gold ETC</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>71.3</v>
+        <v>60.1</v>
       </c>
       <c r="F21" t="n">
-        <v>52.8</v>
+        <v>62.4</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>🟥 Solo size piccola</t>
+          <t>🟡 Metti alert / monitora</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 384.93. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 71.3; priority 52.8; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 60.1; priority 62.4; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Constructive entry zone</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Normal risk</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -4909,17 +4905,17 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 71.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.0%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 60.1, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 3.1%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 227.98 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 190.01 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -4929,173 +4925,151 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>190.01</v>
+        <v>337.23</v>
       </c>
       <c r="T21" t="n">
-        <v>227.98</v>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>NVIDIA Corporation</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+        <v>384.93</v>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Invesco Physical Gold ETC</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Defensive</t>
+        </is>
+      </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Ridurre size / solo monitoraggio</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>2.38</v>
+        <v>-1.6</v>
       </c>
       <c r="Z21" t="n">
-        <v>28.76</v>
+        <v>28.44</v>
       </c>
       <c r="AA21" t="n">
-        <v>46.93</v>
+        <v>18.89</v>
       </c>
       <c r="AB21" t="n">
-        <v>-36.88</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>27.76</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>14.25</v>
-      </c>
+        <v>-22.72</v>
+      </c>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF21" t="inlineStr"/>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Oro</t>
+        </is>
+      </c>
       <c r="AG21" t="n">
-        <v>219.6045</v>
-      </c>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
-      <c r="AK21" t="inlineStr"/>
+        <v>364.23</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>78.2</v>
+      </c>
       <c r="AL21" t="n">
-        <v>3.62</v>
+        <v>7.99</v>
       </c>
       <c r="AM21" t="n">
-        <v>20.12</v>
+        <v>-14.33</v>
       </c>
       <c r="AN21" t="n">
-        <v>65.93000000000001</v>
+        <v>28.05</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.4</v>
+        <v>1.48</v>
       </c>
       <c r="AP21" t="n">
-        <v>209.1889</v>
+        <v>353.1322</v>
       </c>
       <c r="AQ21" t="n">
-        <v>196.0888</v>
+        <v>373.4202</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="AT21" t="n">
-        <v>72.59999999999999</v>
+        <v>46.3</v>
       </c>
       <c r="AU21" t="n">
-        <v>14.2</v>
+        <v>59.2</v>
       </c>
       <c r="AV21" t="n">
-        <v>78.8</v>
+        <v>78.2</v>
       </c>
       <c r="AW21" t="n">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="AX21" t="n">
-        <v>208.48</v>
+        <v>354.48</v>
       </c>
       <c r="AY21" t="n">
-        <v>227.98</v>
+        <v>384.93</v>
       </c>
       <c r="AZ21" t="n">
-        <v>4.96</v>
+        <v>3.14</v>
       </c>
       <c r="BA21" t="n">
-        <v>11.97</v>
-      </c>
-      <c r="BB21" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC21" t="inlineStr">
-        <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-      <c r="BD21" t="n">
-        <v>5301836185600</v>
-      </c>
-      <c r="BE21" t="n">
-        <v>63.66</v>
-      </c>
-      <c r="BF21" t="n">
-        <v>117.21</v>
-      </c>
-      <c r="BG21" t="n">
-        <v>105.9</v>
-      </c>
-      <c r="BH21" t="n">
-        <v>16.97</v>
-      </c>
-      <c r="BI21" t="n">
-        <v>46</v>
-      </c>
-      <c r="BJ21" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK21" t="n">
-        <v>72.59999999999999</v>
-      </c>
-      <c r="BL21" t="n">
-        <v>75.59999999999999</v>
-      </c>
-      <c r="BM21" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="BN21" t="n">
-        <v>78.8</v>
-      </c>
+        <v>-2.46</v>
+      </c>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="inlineStr"/>
+      <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
       <c r="BO21" t="inlineStr"/>
-      <c r="BP21" t="inlineStr">
-        <is>
-          <t>USA / Semiconductors</t>
-        </is>
-      </c>
+      <c r="BP21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5. Solo osservazione</t>
+          <t>2. Rischio da controllare</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5104,54 +5078,54 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>38.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>32.3</v>
+        <v>52</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>⚪ Evita per ora</t>
+          <t>🟥 Solo size piccola</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Lascia fuori dalla lista operativa finché trend, score o rischio non migliorano.</t>
+          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 71.4; priority 52.0; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>No Data</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Dati prezzo insufficienti.</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 71.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 6.2%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 227.98 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
+          <t>Scenario negativo: perdita area 190.01 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5161,104 +5135,156 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Accumulate Carefully</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>No Data</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>190.01</v>
+      </c>
+      <c r="T22" t="n">
+        <v>227.98</v>
+      </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>STM.MI</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Evitare per ora</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>46.94</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>-36.88</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>14.43</v>
+      </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Da monitorare con scenario positivo, base e negativo.</t>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
+      <c r="AG22" t="n">
+        <v>222.27</v>
+      </c>
       <c r="AH22" t="inlineStr"/>
       <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr"/>
-      <c r="AL22" t="inlineStr"/>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr"/>
-      <c r="AQ22" t="inlineStr"/>
+      <c r="AL22" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>21.58</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>66.61</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>209.2422</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>196.1021</v>
+      </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="AU22" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>752</v>
+      </c>
+      <c r="AX22" t="n">
+        <v>208.48</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>227.98</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>13.34</v>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC22" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+      <c r="BD22" t="n">
+        <v>5367878123520</v>
+      </c>
+      <c r="BE22" t="n">
+        <v>63.66</v>
+      </c>
+      <c r="BF22" t="n">
+        <v>117.21</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="BH22" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>46</v>
+      </c>
+      <c r="BJ22" t="n">
         <v>100</v>
       </c>
-      <c r="AV22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX22" t="inlineStr"/>
-      <c r="AY22" t="inlineStr"/>
-      <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" t="inlineStr"/>
-      <c r="BB22" t="inlineStr"/>
-      <c r="BC22" t="inlineStr"/>
-      <c r="BD22" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE22" t="inlineStr"/>
-      <c r="BF22" t="inlineStr"/>
-      <c r="BG22" t="inlineStr"/>
-      <c r="BH22" t="inlineStr"/>
-      <c r="BI22" t="inlineStr"/>
-      <c r="BJ22" t="n">
-        <v>50</v>
-      </c>
       <c r="BK22" t="n">
-        <v>0</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="BL22" t="n">
-        <v>50</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="BM22" t="n">
-        <v>100</v>
+        <v>14.2</v>
       </c>
       <c r="BN22" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO22" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
+        <v>73.8</v>
+      </c>
+      <c r="BO22" t="inlineStr"/>
       <c r="BP22" t="inlineStr">
         <is>
-          <t>Italy / Semiconductors</t>
+          <t>USA / Semiconductors</t>
         </is>
       </c>
     </row>
@@ -5270,20 +5296,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EUNA.MI</t>
+          <t>STM.MI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>iShares Core Global Aggregate Bond</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E23" t="n">
-        <v>28.6</v>
+        <v>38.5</v>
       </c>
       <c r="F23" t="n">
-        <v>27.9</v>
+        <v>32.3</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -5297,7 +5327,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
+          <t>score 38.5; priority 32.3; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -5317,7 +5347,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -5347,17 +5377,13 @@
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>iShares Core Global Aggregate Bond</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>Defensive</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>STM.MI</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr">
         <is>
           <t>Evitare per ora</t>
@@ -5371,38 +5397,22 @@
       <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>Obbligazionario globale</t>
-        </is>
-      </c>
+          <t>Da monitorare con scenario positivo, base e negativo.</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="AI23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ23" t="n">
-        <v>100</v>
-      </c>
-      <c r="AK23" t="n">
-        <v>0</v>
-      </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
       <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>Nessun dato prezzo disponibile</t>
-        </is>
-      </c>
+      <c r="AR23" t="inlineStr"/>
       <c r="AS23" t="n">
         <v>0</v>
       </c>
@@ -5424,19 +5434,39 @@
       <c r="BA23" t="inlineStr"/>
       <c r="BB23" t="inlineStr"/>
       <c r="BC23" t="inlineStr"/>
-      <c r="BD23" t="inlineStr"/>
+      <c r="BD23" t="n">
+        <v>0</v>
+      </c>
       <c r="BE23" t="inlineStr"/>
       <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr"/>
       <c r="BH23" t="inlineStr"/>
       <c r="BI23" t="inlineStr"/>
-      <c r="BJ23" t="inlineStr"/>
-      <c r="BK23" t="inlineStr"/>
-      <c r="BL23" t="inlineStr"/>
-      <c r="BM23" t="inlineStr"/>
-      <c r="BN23" t="inlineStr"/>
-      <c r="BO23" t="inlineStr"/>
-      <c r="BP23" t="inlineStr"/>
+      <c r="BJ23" t="n">
+        <v>50</v>
+      </c>
+      <c r="BK23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL23" t="n">
+        <v>50</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>100</v>
+      </c>
+      <c r="BN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO23" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
+      <c r="BP23" t="inlineStr">
+        <is>
+          <t>Italy / Semiconductors</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5446,64 +5476,64 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SGLD.MI</t>
+          <t>EUNA.MI</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
+          <t>iShares Core Global Aggregate Bond</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>59.5</v>
+        <v>28.6</v>
       </c>
       <c r="F24" t="n">
-        <v>61.8</v>
+        <v>27.9</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>⚪ Osserva</t>
+          <t>⚪ Evita per ora</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Tieni in osservazione senza azione immediata; rivaluta dopo aggiornamento dati o news rilevanti.</t>
+          <t>Lascia fuori dalla lista operativa finché trend, score o rischio non migliorano.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>score 59.5; priority 61.8; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 28.6; priority 27.9; trend: No Data; entry zone: No Data; risk flag: No Data</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Constructive entry zone</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Normal risk</t>
+          <t>No Data</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma</t>
+          <t>Dati prezzo insufficienti.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 59.5, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.2%.</t>
+          <t>EUNA.MI: scenario base Avoid for Now, score 28.6, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 384.93 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 337.23 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -5513,24 +5543,20 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Recovery</t>
-        </is>
-      </c>
-      <c r="S24" t="n">
-        <v>337.23</v>
-      </c>
-      <c r="T24" t="n">
-        <v>384.93</v>
-      </c>
+          <t>No Data</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Invesco Physical Gold ETC</t>
+          <t>iShares Core Global Aggregate Bond</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -5540,21 +5566,13 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Osservare</t>
-        </is>
-      </c>
-      <c r="Y24" t="n">
-        <v>-2.55</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>27.19</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>18.91</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>-22.72</v>
-      </c>
+          <t>Evitare per ora</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
@@ -5564,70 +5582,52 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>Oro</t>
-        </is>
-      </c>
-      <c r="AG24" t="n">
-        <v>360.7</v>
-      </c>
+          <t>Obbligazionario globale</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="n">
-        <v>66.5</v>
+        <v>34.2</v>
       </c>
       <c r="AI24" t="n">
-        <v>44.1</v>
+        <v>0</v>
       </c>
       <c r="AJ24" t="n">
-        <v>59.1</v>
+        <v>100</v>
       </c>
       <c r="AK24" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>6.94</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>-15.16</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>27.64</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>353.0616</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>373.4025</v>
-      </c>
-      <c r="AR24" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>Nessun dato prezzo disponibile</t>
+        </is>
+      </c>
       <c r="AS24" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AT24" t="n">
-        <v>44.1</v>
+        <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>59.1</v>
+        <v>100</v>
       </c>
       <c r="AV24" t="n">
-        <v>78.2</v>
+        <v>0</v>
       </c>
       <c r="AW24" t="n">
-        <v>756</v>
-      </c>
-      <c r="AX24" t="n">
-        <v>354.48</v>
-      </c>
-      <c r="AY24" t="n">
-        <v>384.93</v>
-      </c>
-      <c r="AZ24" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>-3.4</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
       <c r="BB24" t="inlineStr"/>
       <c r="BC24" t="inlineStr"/>
       <c r="BD24" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v10_decision_cockpit_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -776,10 +776,10 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>68.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="F2" t="n">
-        <v>71.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 68.1; priority 71.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 69.2; priority 72.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.8%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 69.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -864,10 +864,10 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>4.22</v>
+        <v>7.48</v>
       </c>
       <c r="Z2" t="n">
-        <v>43.3</v>
+        <v>41.94</v>
       </c>
       <c r="AA2" t="n">
         <v>22.49</v>
@@ -888,13 +888,13 @@
         </is>
       </c>
       <c r="AG2" t="n">
-        <v>18.36</v>
+        <v>18.37</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.3</v>
+        <v>51.7</v>
       </c>
       <c r="AI2" t="n">
-        <v>84.7</v>
+        <v>88.8</v>
       </c>
       <c r="AJ2" t="n">
         <v>44.5</v>
@@ -903,29 +903,29 @@
         <v>82.8</v>
       </c>
       <c r="AL2" t="n">
-        <v>-1.39</v>
+        <v>-2.14</v>
       </c>
       <c r="AM2" t="n">
-        <v>29.97</v>
+        <v>29.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>19.55</v>
+        <v>20.04</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.2064</v>
+        <v>18.2048</v>
       </c>
       <c r="AQ2" t="n">
-        <v>15.8741</v>
+        <v>15.9218</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
         <v>85</v>
       </c>
       <c r="AT2" t="n">
-        <v>84.7</v>
+        <v>88.8</v>
       </c>
       <c r="AU2" t="n">
         <v>49.5</v>
@@ -934,7 +934,7 @@
         <v>82.8</v>
       </c>
       <c r="AW2" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX2" t="n">
         <v>17.976</v>
@@ -943,10 +943,10 @@
         <v>19.25</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.84</v>
+        <v>0.91</v>
       </c>
       <c r="BA2" t="n">
-        <v>15.66</v>
+        <v>15.38</v>
       </c>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
@@ -1192,10 +1192,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>65.90000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>52.6</v>
+        <v>53.2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 65.9; priority 52.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 66.1; priority 53.2; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 65.9, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -3.7%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 66.1, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.4%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1276,22 +1276,22 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>-2.6</v>
+        <v>-1.33</v>
       </c>
       <c r="Z4" t="n">
-        <v>116.19</v>
+        <v>119.8</v>
       </c>
       <c r="AA4" t="n">
-        <v>39.53</v>
+        <v>39.52</v>
       </c>
       <c r="AB4" t="n">
         <v>-44.77</v>
       </c>
       <c r="AC4" t="n">
-        <v>57.59</v>
+        <v>58.5</v>
       </c>
       <c r="AD4" t="n">
-        <v>28.38</v>
+        <v>28.73</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1300,45 +1300,45 @@
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>1467.4</v>
+        <v>1485.4</v>
       </c>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
-        <v>-1.78</v>
+        <v>-0.91</v>
       </c>
       <c r="AM4" t="n">
-        <v>28.3</v>
+        <v>24.21</v>
       </c>
       <c r="AN4" t="n">
-        <v>34.04</v>
+        <v>36.41</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AP4" t="n">
-        <v>1524.3985</v>
+        <v>1521.9053</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1280.7529</v>
+        <v>1284.0297</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
         <v>65</v>
       </c>
       <c r="AT4" t="n">
-        <v>92.40000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="AU4" t="n">
         <v>16.8</v>
       </c>
       <c r="AV4" t="n">
-        <v>74.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="AW4" t="n">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="AX4" t="n">
         <v>1423.4</v>
@@ -1347,10 +1347,10 @@
         <v>1621.2</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-3.74</v>
+        <v>-2.4</v>
       </c>
       <c r="BA4" t="n">
-        <v>14.57</v>
+        <v>15.68</v>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="BD4" t="n">
-        <v>563628343296</v>
+        <v>570542129152</v>
       </c>
       <c r="BE4" t="n">
         <v>30.11</v>
@@ -1384,16 +1384,16 @@
         <v>100</v>
       </c>
       <c r="BK4" t="n">
-        <v>92.40000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="BL4" t="n">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
       <c r="BM4" t="n">
         <v>16.8</v>
       </c>
       <c r="BN4" t="n">
-        <v>74.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="BO4" t="inlineStr"/>
       <c r="BP4" t="inlineStr">
@@ -1410,24 +1410,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>INRG.MI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Meta Platforms, Inc.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>66.2</v>
+        <v>42.5</v>
       </c>
       <c r="F5" t="n">
-        <v>48.8</v>
+        <v>49.3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1441,37 +1437,37 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 66.2; priority 48.8; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 42.5; priority 49.3; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>META: scenario base Hold / Monitor, score 66.2, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.6%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 42.5, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -3.2%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 681.31 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 10.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 539.03 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1481,158 +1477,136 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Recovery</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>539.03</v>
+        <v>8.541</v>
       </c>
       <c r="T5" t="n">
-        <v>681.3099999999999</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Meta Platforms, Inc.</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+        <v>10.872</v>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>4.1</v>
+        <v>-10.61</v>
       </c>
       <c r="Z5" t="n">
-        <v>-17.35</v>
+        <v>26.69</v>
       </c>
       <c r="AA5" t="n">
-        <v>37.49</v>
+        <v>24.12</v>
       </c>
       <c r="AB5" t="n">
-        <v>-34.15</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>23.22</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>17.64</v>
-      </c>
+        <v>-34.52</v>
+      </c>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Energia pulita</t>
+        </is>
+      </c>
       <c r="AG5" t="n">
-        <v>616.77</v>
-      </c>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
+        <v>8.863</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>70.5</v>
+      </c>
       <c r="AL5" t="n">
-        <v>4.56</v>
+        <v>-2.54</v>
       </c>
       <c r="AM5" t="n">
-        <v>-4.19</v>
+        <v>-2.18</v>
       </c>
       <c r="AN5" t="n">
-        <v>27.59</v>
+        <v>3.54</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.74</v>
+        <v>0.15</v>
       </c>
       <c r="AP5" t="n">
-        <v>595.4915999999999</v>
+        <v>9.1534</v>
       </c>
       <c r="AQ5" t="n">
-        <v>621.6067</v>
+        <v>9.2888</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="AT5" t="n">
-        <v>48.9</v>
+        <v>40.5</v>
       </c>
       <c r="AU5" t="n">
-        <v>27.7</v>
+        <v>43.4</v>
       </c>
       <c r="AV5" t="n">
-        <v>78.2</v>
+        <v>70.5</v>
       </c>
       <c r="AW5" t="n">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="AX5" t="n">
-        <v>543.67</v>
+        <v>8.541</v>
       </c>
       <c r="AY5" t="n">
-        <v>616.77</v>
+        <v>9.217000000000001</v>
       </c>
       <c r="AZ5" t="n">
-        <v>3.57</v>
+        <v>-3.17</v>
       </c>
       <c r="BA5" t="n">
-        <v>-0.78</v>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>Internet Content &amp; Information</t>
-        </is>
-      </c>
-      <c r="BD5" t="n">
-        <v>1571225468928</v>
-      </c>
-      <c r="BE5" t="n">
-        <v>29.83</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>29.85</v>
-      </c>
-      <c r="BG5" t="n">
-        <v>28</v>
-      </c>
-      <c r="BH5" t="n">
-        <v>43</v>
-      </c>
-      <c r="BI5" t="n">
-        <v>34</v>
-      </c>
-      <c r="BJ5" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>76</v>
-      </c>
-      <c r="BM5" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="BN5" t="n">
-        <v>78.2</v>
-      </c>
+        <v>-4.58</v>
+      </c>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
       <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr">
-        <is>
-          <t>USA / Social &amp; AI</t>
-        </is>
-      </c>
+      <c r="BP5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1642,20 +1616,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>META</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>39.7</v>
+        <v>66.2</v>
       </c>
       <c r="F6" t="n">
-        <v>46.3</v>
+        <v>48.8</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1669,37 +1647,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 39.7; priority 46.3; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 66.2; priority 48.8; trend: Recovery; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>prezzo 4.7% sotto MA50: attendere recupero; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 39.7, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -4.7%.</t>
+          <t>META: scenario base Hold / Monitor, score 66.2, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.6%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 10.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 681.31 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 539.03 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1709,136 +1687,158 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Recovery</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>8.541</v>
+        <v>539.03</v>
       </c>
       <c r="T6" t="n">
-        <v>10.872</v>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>681.3099999999999</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>-17.19</v>
+        <v>4.1</v>
       </c>
       <c r="Z6" t="n">
-        <v>26.56</v>
+        <v>-17.35</v>
       </c>
       <c r="AA6" t="n">
-        <v>24.15</v>
+        <v>37.49</v>
       </c>
       <c r="AB6" t="n">
-        <v>-34.68</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
+        <v>-34.15</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>17.64</v>
+      </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>Energia pulita</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
-        <v>8.765000000000001</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>34</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>68.2</v>
-      </c>
+        <v>616.77</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
-        <v>-3.37</v>
+        <v>4.56</v>
       </c>
       <c r="AM6" t="n">
-        <v>-0.35</v>
+        <v>-4.19</v>
       </c>
       <c r="AN6" t="n">
-        <v>2.04</v>
+        <v>27.59</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.08</v>
+        <v>0.74</v>
       </c>
       <c r="AP6" t="n">
-        <v>9.1991</v>
+        <v>595.4915999999999</v>
       </c>
       <c r="AQ6" t="n">
-        <v>9.283899999999999</v>
+        <v>621.6067</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="AT6" t="n">
-        <v>32.4</v>
+        <v>48.9</v>
       </c>
       <c r="AU6" t="n">
-        <v>43.3</v>
+        <v>27.7</v>
       </c>
       <c r="AV6" t="n">
-        <v>68.2</v>
+        <v>78.2</v>
       </c>
       <c r="AW6" t="n">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="AX6" t="n">
-        <v>8.541</v>
+        <v>543.67</v>
       </c>
       <c r="AY6" t="n">
-        <v>9.217000000000001</v>
+        <v>616.77</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-4.72</v>
+        <v>3.57</v>
       </c>
       <c r="BA6" t="n">
-        <v>-5.59</v>
-      </c>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
+        <v>-0.78</v>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+      <c r="BD6" t="n">
+        <v>1571225468928</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>29.83</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>29.85</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>28</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>43</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>34</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>76</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>78.2</v>
+      </c>
       <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>USA / Social &amp; AI</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1858,10 +1858,10 @@
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>55.8</v>
+        <v>57.1</v>
       </c>
       <c r="F7" t="n">
-        <v>40.2</v>
+        <v>46.8</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>score 55.8; priority 40.2; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 57.1; priority 46.8; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1890,12 +1890,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>prezzo 10.0% sopra MA50: evitare inseguimento</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base Hold / Monitor, score 55.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 10.0%.</t>
+          <t>WCLD.MI: scenario base Hold / Monitor, score 57.1, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 7.9%.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1946,13 +1946,13 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>27.63</v>
+        <v>29.32</v>
       </c>
       <c r="Z7" t="n">
-        <v>18.3</v>
+        <v>15.37</v>
       </c>
       <c r="AA7" t="n">
-        <v>35.04</v>
+        <v>35.1</v>
       </c>
       <c r="AB7" t="n">
         <v>-48.6</v>
@@ -1970,37 +1970,37 @@
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>34.625</v>
+        <v>34.295</v>
       </c>
       <c r="AH7" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="AI7" t="n">
         <v>100</v>
       </c>
       <c r="AJ7" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="AK7" t="n">
-        <v>58.6</v>
+        <v>67.3</v>
       </c>
       <c r="AL7" t="n">
-        <v>6.52</v>
+        <v>3.81</v>
       </c>
       <c r="AM7" t="n">
-        <v>38.72</v>
+        <v>39.64</v>
       </c>
       <c r="AN7" t="n">
-        <v>5.67</v>
+        <v>5.61</v>
       </c>
       <c r="AO7" t="n">
         <v>0.16</v>
       </c>
       <c r="AP7" t="n">
-        <v>31.4648</v>
+        <v>31.7959</v>
       </c>
       <c r="AQ7" t="n">
-        <v>27.0987</v>
+        <v>27.1592</v>
       </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="n">
@@ -2010,25 +2010,25 @@
         <v>100</v>
       </c>
       <c r="AU7" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="AV7" t="n">
-        <v>58.6</v>
+        <v>67.3</v>
       </c>
       <c r="AW7" t="n">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="AX7" t="n">
-        <v>33.035</v>
+        <v>33.575</v>
       </c>
       <c r="AY7" t="n">
         <v>36.89</v>
       </c>
       <c r="AZ7" t="n">
-        <v>10.04</v>
+        <v>7.86</v>
       </c>
       <c r="BA7" t="n">
-        <v>27.77</v>
+        <v>26.27</v>
       </c>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
@@ -2164,7 +2164,7 @@
         <v>-53.77</v>
       </c>
       <c r="AC8" t="n">
-        <v>324.84</v>
+        <v>321.89</v>
       </c>
       <c r="AD8" t="n">
         <v>164.03</v>
@@ -2294,10 +2294,10 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>81.2</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>81.2</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 81.2; priority 81.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 82.4; priority 82.4; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 81.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.5%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 82.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 74.14 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 74.47 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -2363,7 +2363,7 @@
         <v>69.45</v>
       </c>
       <c r="T9" t="n">
-        <v>74.14</v>
+        <v>74.47</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>5.19</v>
+        <v>8.1</v>
       </c>
       <c r="Z9" t="n">
-        <v>60.58</v>
+        <v>59.62</v>
       </c>
       <c r="AA9" t="n">
-        <v>14.15</v>
+        <v>14.14</v>
       </c>
       <c r="AB9" t="n">
         <v>-17.8</v>
@@ -2406,13 +2406,13 @@
         </is>
       </c>
       <c r="AG9" t="n">
-        <v>74.14</v>
+        <v>74.47</v>
       </c>
       <c r="AH9" t="n">
-        <v>78.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="AI9" t="n">
-        <v>91</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="AJ9" t="n">
         <v>68.8</v>
@@ -2421,29 +2421,29 @@
         <v>82.8</v>
       </c>
       <c r="AL9" t="n">
-        <v>3.07</v>
+        <v>3.37</v>
       </c>
       <c r="AM9" t="n">
-        <v>30.99</v>
+        <v>31.36</v>
       </c>
       <c r="AN9" t="n">
-        <v>26.34</v>
+        <v>26.75</v>
       </c>
       <c r="AO9" t="n">
-        <v>1.86</v>
+        <v>1.89</v>
       </c>
       <c r="AP9" t="n">
-        <v>71.6688</v>
+        <v>71.7462</v>
       </c>
       <c r="AQ9" t="n">
-        <v>62.0988</v>
+        <v>62.3391</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>85</v>
       </c>
       <c r="AT9" t="n">
-        <v>91</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="AU9" t="n">
         <v>68.8</v>
@@ -2452,19 +2452,19 @@
         <v>82.8</v>
       </c>
       <c r="AW9" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX9" t="n">
         <v>71.86</v>
       </c>
       <c r="AY9" t="n">
-        <v>74.14</v>
+        <v>74.47</v>
       </c>
       <c r="AZ9" t="n">
-        <v>3.45</v>
+        <v>3.8</v>
       </c>
       <c r="BA9" t="n">
-        <v>19.39</v>
+        <v>19.46</v>
       </c>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
@@ -2600,7 +2600,7 @@
         <v>-34.5</v>
       </c>
       <c r="AC10" t="n">
-        <v>27.82</v>
+        <v>27.85</v>
       </c>
       <c r="AD10" t="n">
         <v>21.2</v>
@@ -2690,7 +2690,7 @@
         <v>29.12</v>
       </c>
       <c r="BI10" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="BJ10" t="n">
         <v>100</v>
@@ -2735,7 +2735,7 @@
         <v>75</v>
       </c>
       <c r="F11" t="n">
-        <v>75.59999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 75.0; priority 75.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 75.0; priority 75.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 75.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.4%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 75.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 63.03 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 63.18 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>63.0272</v>
+        <v>63.18</v>
       </c>
       <c r="T11" t="n">
         <v>65.95</v>
@@ -2820,10 +2820,10 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>5.08</v>
+        <v>5.59</v>
       </c>
       <c r="Z11" t="n">
-        <v>22.09</v>
+        <v>21.3</v>
       </c>
       <c r="AA11" t="n">
         <v>12.76</v>
@@ -2844,13 +2844,13 @@
         </is>
       </c>
       <c r="AG11" t="n">
-        <v>65</v>
+        <v>64.91</v>
       </c>
       <c r="AH11" t="n">
-        <v>72.7</v>
+        <v>73</v>
       </c>
       <c r="AI11" t="n">
-        <v>69.2</v>
+        <v>68.8</v>
       </c>
       <c r="AJ11" t="n">
         <v>71.59999999999999</v>
@@ -2859,29 +2859,29 @@
         <v>82.8</v>
       </c>
       <c r="AL11" t="n">
-        <v>-0.84</v>
+        <v>-1.53</v>
       </c>
       <c r="AM11" t="n">
-        <v>10.92</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="AN11" t="n">
-        <v>15.48</v>
+        <v>15.76</v>
       </c>
       <c r="AO11" t="n">
-        <v>1.21</v>
+        <v>1.23</v>
       </c>
       <c r="AP11" t="n">
-        <v>64.762</v>
+        <v>64.82599999999999</v>
       </c>
       <c r="AQ11" t="n">
-        <v>60.8913</v>
+        <v>60.9924</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>69.2</v>
+        <v>68.8</v>
       </c>
       <c r="AU11" t="n">
         <v>71.59999999999999</v>
@@ -2890,7 +2890,7 @@
         <v>82.8</v>
       </c>
       <c r="AW11" t="n">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="AX11" t="n">
         <v>64.53</v>
@@ -2899,10 +2899,10 @@
         <v>65.95</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.37</v>
+        <v>0.13</v>
       </c>
       <c r="BA11" t="n">
-        <v>6.75</v>
+        <v>6.42</v>
       </c>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
@@ -2938,10 +2938,10 @@
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>74</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>75</v>
+        <v>75.3</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>score 74.0; priority 75.0; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.4; priority 75.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 74.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.0%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 74.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.3%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -3026,10 +3026,10 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>3.83</v>
+        <v>5.3</v>
       </c>
       <c r="Z12" t="n">
-        <v>38.68</v>
+        <v>38.64</v>
       </c>
       <c r="AA12" t="n">
         <v>17.06</v>
@@ -3050,13 +3050,13 @@
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>48.24</v>
+        <v>48.38</v>
       </c>
       <c r="AH12" t="n">
-        <v>68</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AI12" t="n">
-        <v>76</v>
+        <v>76.8</v>
       </c>
       <c r="AJ12" t="n">
         <v>64.2</v>
@@ -3065,29 +3065,29 @@
         <v>82.8</v>
       </c>
       <c r="AL12" t="n">
-        <v>3.13</v>
+        <v>3.93</v>
       </c>
       <c r="AM12" t="n">
-        <v>18.21</v>
+        <v>16.16</v>
       </c>
       <c r="AN12" t="n">
-        <v>19.25</v>
+        <v>20.06</v>
       </c>
       <c r="AO12" t="n">
-        <v>1.13</v>
+        <v>1.18</v>
       </c>
       <c r="AP12" t="n">
-        <v>46.852</v>
+        <v>46.8524</v>
       </c>
       <c r="AQ12" t="n">
-        <v>43.5122</v>
+        <v>43.6109</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
         <v>85</v>
       </c>
       <c r="AT12" t="n">
-        <v>76</v>
+        <v>76.8</v>
       </c>
       <c r="AU12" t="n">
         <v>64.2</v>
@@ -3096,19 +3096,19 @@
         <v>82.8</v>
       </c>
       <c r="AW12" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX12" t="n">
         <v>46.37</v>
       </c>
       <c r="AY12" t="n">
-        <v>48.24</v>
+        <v>48.38</v>
       </c>
       <c r="AZ12" t="n">
-        <v>2.96</v>
+        <v>3.26</v>
       </c>
       <c r="BA12" t="n">
-        <v>10.87</v>
+        <v>10.94</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3144,10 +3144,10 @@
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>74.3</v>
+        <v>74.8</v>
       </c>
       <c r="F13" t="n">
-        <v>74.7</v>
+        <v>75.2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 74.3; priority 74.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.8; priority 75.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.2%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.1%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -3228,14 +3228,14 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Monitorare ingresso graduale</t>
+          <t>Priorità watchlist</t>
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>3.91</v>
+        <v>5.43</v>
       </c>
       <c r="Z13" t="n">
-        <v>24.91</v>
+        <v>23.19</v>
       </c>
       <c r="AA13" t="n">
         <v>12.99</v>
@@ -3259,10 +3259,10 @@
         <v>167.88</v>
       </c>
       <c r="AH13" t="n">
-        <v>73</v>
+        <v>73.3</v>
       </c>
       <c r="AI13" t="n">
-        <v>69.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="AJ13" t="n">
         <v>67.59999999999999</v>
@@ -3271,29 +3271,29 @@
         <v>82.8</v>
       </c>
       <c r="AL13" t="n">
-        <v>-0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="AM13" t="n">
-        <v>13.17</v>
+        <v>13.02</v>
       </c>
       <c r="AN13" t="n">
-        <v>17.49</v>
+        <v>17.78</v>
       </c>
       <c r="AO13" t="n">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="AP13" t="n">
-        <v>165.9368</v>
+        <v>166.1128</v>
       </c>
       <c r="AQ13" t="n">
-        <v>154.5522</v>
+        <v>154.8109</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
         <v>85</v>
       </c>
       <c r="AT13" t="n">
-        <v>69.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="AU13" t="n">
         <v>67.59999999999999</v>
@@ -3302,7 +3302,7 @@
         <v>82.8</v>
       </c>
       <c r="AW13" t="n">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="AX13" t="n">
         <v>165.62</v>
@@ -3311,10 +3311,10 @@
         <v>169.62</v>
       </c>
       <c r="AZ13" t="n">
-        <v>1.17</v>
+        <v>1.06</v>
       </c>
       <c r="BA13" t="n">
-        <v>8.619999999999999</v>
+        <v>8.44</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3350,10 +3350,10 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>73.7</v>
+        <v>74.3</v>
       </c>
       <c r="F14" t="n">
-        <v>74.2</v>
+        <v>74.8</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 73.7; priority 74.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.3; priority 74.8; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 73.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.8%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 74.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 122.82 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 123.69 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="S14" t="n">
-        <v>122.82</v>
+        <v>123.69</v>
       </c>
       <c r="T14" t="n">
         <v>129.38</v>
@@ -3438,10 +3438,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>3.89</v>
+        <v>5.51</v>
       </c>
       <c r="Z14" t="n">
-        <v>22.88</v>
+        <v>21.01</v>
       </c>
       <c r="AA14" t="n">
         <v>13.19</v>
@@ -3462,13 +3462,13 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>127.44</v>
+        <v>127.38</v>
       </c>
       <c r="AH14" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AI14" t="n">
-        <v>68.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AJ14" t="n">
         <v>66.90000000000001</v>
@@ -3477,29 +3477,29 @@
         <v>82.8</v>
       </c>
       <c r="AL14" t="n">
-        <v>-0.64</v>
+        <v>-1</v>
       </c>
       <c r="AM14" t="n">
-        <v>12.53</v>
+        <v>12.72</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.28</v>
+        <v>17.49</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.31</v>
+        <v>1.33</v>
       </c>
       <c r="AP14" t="n">
-        <v>126.3618</v>
+        <v>126.514</v>
       </c>
       <c r="AQ14" t="n">
-        <v>117.7367</v>
+        <v>117.9225</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
         <v>85</v>
       </c>
       <c r="AT14" t="n">
-        <v>68.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AU14" t="n">
         <v>66.90000000000001</v>
@@ -3508,7 +3508,7 @@
         <v>82.8</v>
       </c>
       <c r="AW14" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX14" t="n">
         <v>126.18</v>
@@ -3517,10 +3517,10 @@
         <v>129.38</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.85</v>
+        <v>0.68</v>
       </c>
       <c r="BA14" t="n">
-        <v>8.24</v>
+        <v>8.02</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3546,20 +3546,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MVOL.MI</t>
+          <t>SXR8.DE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>72.2</v>
+        <v>73</v>
       </c>
       <c r="F15" t="n">
-        <v>74.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3568,12 +3568,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 67.85. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 72.2; priority 74.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.0; priority 73.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3588,22 +3588,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 72.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 1.3%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 73.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 67.85 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 63.44 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 690.52 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -3622,20 +3622,20 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>63.44</v>
+        <v>690.52</v>
       </c>
       <c r="T15" t="n">
-        <v>67.84999999999999</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
+          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>Defensive</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -3644,89 +3644,89 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>5.38</v>
+        <v>4.83</v>
       </c>
       <c r="Z15" t="n">
-        <v>7.46</v>
+        <v>20.34</v>
       </c>
       <c r="AA15" t="n">
-        <v>9.68</v>
+        <v>14.25</v>
       </c>
       <c r="AB15" t="n">
-        <v>-12.85</v>
+        <v>-23.32</v>
       </c>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
+          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>Min volatility</t>
+          <t>USA large cap</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>67.43000000000001</v>
+        <v>714.64</v>
       </c>
       <c r="AH15" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>70</v>
+      </c>
+      <c r="AJ15" t="n">
         <v>64.2</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>78.09999999999999</v>
       </c>
       <c r="AK15" t="n">
         <v>82.8</v>
       </c>
       <c r="AL15" t="n">
-        <v>1.03</v>
+        <v>-1.16</v>
       </c>
       <c r="AM15" t="n">
-        <v>3.45</v>
+        <v>13.65</v>
       </c>
       <c r="AN15" t="n">
-        <v>8.27</v>
+        <v>17.98</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.85</v>
+        <v>1.26</v>
       </c>
       <c r="AP15" t="n">
-        <v>66.5558</v>
+        <v>711.3064000000001</v>
       </c>
       <c r="AQ15" t="n">
-        <v>64.1626</v>
+        <v>661.5135</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
         <v>85</v>
       </c>
       <c r="AT15" t="n">
-        <v>61.5</v>
+        <v>70</v>
       </c>
       <c r="AU15" t="n">
-        <v>78.09999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="AV15" t="n">
         <v>82.8</v>
       </c>
       <c r="AW15" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="AX15" t="n">
-        <v>67.06999999999999</v>
+        <v>707.24</v>
       </c>
       <c r="AY15" t="n">
-        <v>67.75</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="AZ15" t="n">
-        <v>1.31</v>
+        <v>0.47</v>
       </c>
       <c r="BA15" t="n">
-        <v>5.09</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3752,12 +3752,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWQU.MI</t>
+          <t>MVOL.MI</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -3765,7 +3765,7 @@
         <v>71.7</v>
       </c>
       <c r="F16" t="n">
-        <v>73.3</v>
+        <v>73.7</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3774,12 +3774,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 78.87. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 67.85. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>score 71.7; priority 73.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 71.7; priority 73.7; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3794,22 +3794,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi</t>
+          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.1%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 71.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 78.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 67.85 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 75.27 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 63.44 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3828,20 +3828,20 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>75.27</v>
+        <v>63.44</v>
       </c>
       <c r="T16" t="n">
-        <v>78.87</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Minimum Volatility UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Factor</t>
+          <t>Defensive</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -3850,89 +3850,89 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>4.06</v>
+        <v>4.63</v>
       </c>
       <c r="Z16" t="n">
-        <v>22.03</v>
+        <v>6.52</v>
       </c>
       <c r="AA16" t="n">
-        <v>12.85</v>
+        <v>9.69</v>
       </c>
       <c r="AB16" t="n">
-        <v>-20.6</v>
+        <v>-12.85</v>
       </c>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>Da monitorare: non è un segnale automatico di acquisto.</t>
+          <t>Strumento utile per bilanciare volatilità e rischio macro.</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Quality globale</t>
+          <t>Min volatility</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>77.48</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="AH16" t="n">
-        <v>64.5</v>
+        <v>63.6</v>
       </c>
       <c r="AI16" t="n">
-        <v>67.3</v>
+        <v>60.1</v>
       </c>
       <c r="AJ16" t="n">
-        <v>68.09999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AK16" t="n">
         <v>82.8</v>
       </c>
       <c r="AL16" t="n">
-        <v>-1.2</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="AM16" t="n">
-        <v>10.21</v>
+        <v>3.31</v>
       </c>
       <c r="AN16" t="n">
-        <v>14.66</v>
+        <v>7.98</v>
       </c>
       <c r="AO16" t="n">
-        <v>1.14</v>
+        <v>0.82</v>
       </c>
       <c r="AP16" t="n">
-        <v>77.4118</v>
+        <v>66.66419999999999</v>
       </c>
       <c r="AQ16" t="n">
-        <v>72.1867</v>
+        <v>64.2088</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
         <v>85</v>
       </c>
       <c r="AT16" t="n">
-        <v>67.3</v>
+        <v>60.1</v>
       </c>
       <c r="AU16" t="n">
-        <v>68.09999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AV16" t="n">
         <v>82.8</v>
       </c>
       <c r="AW16" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX16" t="n">
-        <v>77.16</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="AY16" t="n">
-        <v>78.87</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.09</v>
+        <v>0.73</v>
       </c>
       <c r="BA16" t="n">
-        <v>7.33</v>
+        <v>4.58</v>
       </c>
       <c r="BB16" t="inlineStr"/>
       <c r="BC16" t="inlineStr"/>
@@ -3958,20 +3958,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SXR8.DE</t>
+          <t>IWQU.MI</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>72.40000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>73.09999999999999</v>
+        <v>71</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3980,12 +3980,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 727.18. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 78.87. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 72.4; priority 73.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 68.4; priority 71.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4005,17 +4005,17 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 72.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
+          <t>IWQU.MI: scenario base Accumulate Carefully, score 68.4, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 727.18 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 78.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 690.52 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 75.30 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4030,24 +4030,24 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>690.52</v>
+        <v>75.3</v>
       </c>
       <c r="T17" t="n">
-        <v>727.1799999999999</v>
+        <v>78.87</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>iShares Core S&amp;P 500 UCITS ETF USD (Acc)</t>
+          <t>iShares Edge MSCI World Quality Factor UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Factor</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -4056,16 +4056,16 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>3.18</v>
+        <v>4.55</v>
       </c>
       <c r="Z17" t="n">
-        <v>22.55</v>
+        <v>19.78</v>
       </c>
       <c r="AA17" t="n">
-        <v>14.25</v>
+        <v>12.85</v>
       </c>
       <c r="AB17" t="n">
-        <v>-23.32</v>
+        <v>-20.6</v>
       </c>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
@@ -4076,69 +4076,69 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>USA large cap</t>
+          <t>Quality globale</t>
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>715.3</v>
+        <v>77.38</v>
       </c>
       <c r="AH17" t="n">
-        <v>69.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="AI17" t="n">
-        <v>68</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AJ17" t="n">
-        <v>64.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>82.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AL17" t="n">
-        <v>-0.99</v>
+        <v>-1.44</v>
       </c>
       <c r="AM17" t="n">
-        <v>13.12</v>
+        <v>10.54</v>
       </c>
       <c r="AN17" t="n">
-        <v>17.77</v>
+        <v>14.96</v>
       </c>
       <c r="AO17" t="n">
-        <v>1.25</v>
+        <v>1.16</v>
       </c>
       <c r="AP17" t="n">
-        <v>710.5252</v>
+        <v>77.47880000000001</v>
       </c>
       <c r="AQ17" t="n">
-        <v>660.5142</v>
+        <v>72.29949999999999</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT17" t="n">
-        <v>68</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AU17" t="n">
-        <v>64.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>82.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AW17" t="n">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="AX17" t="n">
-        <v>707.24</v>
+        <v>77.16</v>
       </c>
       <c r="AY17" t="n">
-        <v>727.1799999999999</v>
+        <v>78.87</v>
       </c>
       <c r="AZ17" t="n">
-        <v>0.67</v>
+        <v>-0.13</v>
       </c>
       <c r="BA17" t="n">
-        <v>8.289999999999999</v>
+        <v>7.03</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4274,10 +4274,10 @@
         <v>-33.36</v>
       </c>
       <c r="AC18" t="n">
-        <v>36.65</v>
+        <v>36.61</v>
       </c>
       <c r="AD18" t="n">
-        <v>33.54</v>
+        <v>33.42</v>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
@@ -4364,7 +4364,7 @@
         <v>78.44</v>
       </c>
       <c r="BI18" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="BJ18" t="n">
         <v>100</v>
@@ -4373,7 +4373,7 @@
         <v>79.09999999999999</v>
       </c>
       <c r="BL18" t="n">
-        <v>37.7</v>
+        <v>37.9</v>
       </c>
       <c r="BM18" t="n">
         <v>41</v>
@@ -4640,10 +4640,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>70.7</v>
+        <v>70.8</v>
       </c>
       <c r="F20" t="n">
-        <v>65.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4652,12 +4652,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 377.65. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 377.4074. Trigger: prezzo vicino a MA50: monitorare conferma.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 70.7; priority 65.3; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
+          <t>score 70.8; priority 65.4; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4677,17 +4677,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>GOOGL: scenario base Accumulate Carefully, score 70.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.9%.</t>
+          <t>GOOGL: scenario base Accumulate Carefully, score 70.8, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.8%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 377.65 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 377.41 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 317.69 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 317.49 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -4706,10 +4706,10 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>317.69</v>
+        <v>317.4859</v>
       </c>
       <c r="T20" t="n">
-        <v>377.65</v>
+        <v>377.4074</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -4724,10 +4724,10 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>-8.1</v>
+        <v>-8.050000000000001</v>
       </c>
       <c r="Z20" t="n">
-        <v>46.12</v>
+        <v>46.21</v>
       </c>
       <c r="AA20" t="n">
         <v>30.57</v>
@@ -4736,7 +4736,7 @@
         <v>-29.81</v>
       </c>
       <c r="AC20" t="n">
-        <v>16.98</v>
+        <v>16.97</v>
       </c>
       <c r="AD20" t="n">
         <v>22.79</v>
@@ -4755,50 +4755,50 @@
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="n">
-        <v>-5.39</v>
+        <v>-5.33</v>
       </c>
       <c r="AM20" t="n">
-        <v>13.53</v>
+        <v>13.6</v>
       </c>
       <c r="AN20" t="n">
-        <v>36.1</v>
+        <v>36.13</v>
       </c>
       <c r="AO20" t="n">
         <v>1.18</v>
       </c>
       <c r="AP20" t="n">
-        <v>348.5694</v>
+        <v>348.3498</v>
       </c>
       <c r="AQ20" t="n">
-        <v>335.7109</v>
+        <v>335.4963</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>65</v>
       </c>
       <c r="AT20" t="n">
-        <v>58.3</v>
+        <v>58.4</v>
       </c>
       <c r="AU20" t="n">
         <v>39.5</v>
       </c>
       <c r="AV20" t="n">
-        <v>75.40000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="AW20" t="n">
         <v>754</v>
       </c>
       <c r="AX20" t="n">
-        <v>335.02</v>
+        <v>334.8048</v>
       </c>
       <c r="AY20" t="n">
-        <v>357.52</v>
+        <v>357.2903</v>
       </c>
       <c r="AZ20" t="n">
-        <v>-2.9</v>
+        <v>-2.84</v>
       </c>
       <c r="BA20" t="n">
-        <v>0.82</v>
+        <v>0.88</v>
       </c>
       <c r="BB20" t="inlineStr">
         <is>
@@ -4832,16 +4832,16 @@
         <v>100</v>
       </c>
       <c r="BK20" t="n">
-        <v>58.3</v>
+        <v>58.4</v>
       </c>
       <c r="BL20" t="n">
-        <v>75.90000000000001</v>
+        <v>76</v>
       </c>
       <c r="BM20" t="n">
         <v>39.5</v>
       </c>
       <c r="BN20" t="n">
-        <v>75.40000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="BO20" t="inlineStr"/>
       <c r="BP20" t="inlineStr">
@@ -4868,10 +4868,10 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>61.5</v>
+        <v>62.1</v>
       </c>
       <c r="F21" t="n">
-        <v>63.8</v>
+        <v>64.5</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>score 61.5; priority 63.8; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 62.1; priority 64.5; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -4905,7 +4905,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 61.5, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 62.1, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.3%.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4956,13 +4956,13 @@
         </is>
       </c>
       <c r="Y21" t="n">
-        <v>1.67</v>
+        <v>5.73</v>
       </c>
       <c r="Z21" t="n">
-        <v>26.52</v>
+        <v>23.95</v>
       </c>
       <c r="AA21" t="n">
-        <v>18.89</v>
+        <v>18.98</v>
       </c>
       <c r="AB21" t="n">
         <v>-22.72</v>
@@ -4980,53 +4980,53 @@
         </is>
       </c>
       <c r="AG21" t="n">
-        <v>367.42</v>
+        <v>363.41</v>
       </c>
       <c r="AH21" t="n">
-        <v>67.3</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AI21" t="n">
-        <v>51.3</v>
+        <v>54.5</v>
       </c>
       <c r="AJ21" t="n">
-        <v>59.2</v>
+        <v>59</v>
       </c>
       <c r="AK21" t="n">
         <v>78.2</v>
       </c>
       <c r="AL21" t="n">
-        <v>3.65</v>
+        <v>0.34</v>
       </c>
       <c r="AM21" t="n">
-        <v>-12.76</v>
+        <v>-15.91</v>
       </c>
       <c r="AN21" t="n">
-        <v>28.34</v>
+        <v>28.01</v>
       </c>
       <c r="AO21" t="n">
-        <v>1.5</v>
+        <v>1.48</v>
       </c>
       <c r="AP21" t="n">
-        <v>354.0998</v>
+        <v>355.163</v>
       </c>
       <c r="AQ21" t="n">
-        <v>373.6235</v>
+        <v>373.9259</v>
       </c>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="n">
         <v>55</v>
       </c>
       <c r="AT21" t="n">
-        <v>51.3</v>
+        <v>54.5</v>
       </c>
       <c r="AU21" t="n">
-        <v>59.2</v>
+        <v>59</v>
       </c>
       <c r="AV21" t="n">
         <v>78.2</v>
       </c>
       <c r="AW21" t="n">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AX21" t="n">
         <v>362.11</v>
@@ -5035,10 +5035,10 @@
         <v>384.93</v>
       </c>
       <c r="AZ21" t="n">
-        <v>3.76</v>
+        <v>2.32</v>
       </c>
       <c r="BA21" t="n">
-        <v>-1.66</v>
+        <v>-2.81</v>
       </c>
       <c r="BB21" t="inlineStr"/>
       <c r="BC21" t="inlineStr"/>
@@ -5078,7 +5078,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>74.3</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="F22" t="n">
         <v>48.6</v>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>score 74.3; priority 48.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 74.4; priority 48.6; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>NVDA: scenario base Accumulate Carefully, score 74.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.4%.</t>
+          <t>NVDA: scenario base Accumulate Carefully, score 74.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.4%.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -5177,7 +5177,7 @@
         <v>29.16</v>
       </c>
       <c r="AD22" t="n">
-        <v>14.9</v>
+        <v>14.84</v>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
@@ -5264,7 +5264,7 @@
         <v>16.97</v>
       </c>
       <c r="BI22" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="BJ22" t="n">
         <v>100</v>
@@ -5273,7 +5273,7 @@
         <v>93.7</v>
       </c>
       <c r="BL22" t="n">
-        <v>73</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="BM22" t="n">
         <v>14.2</v>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v11_live_value_cockpit_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Action_Plan.xlsx
+++ b/AlphaForge_Action_Plan.xlsx
@@ -776,10 +776,10 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>69.2</v>
+        <v>64.5</v>
       </c>
       <c r="F2" t="n">
-        <v>72.59999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score 69.2; priority 72.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
+          <t>score 64.5; priority 68.9; trend: Constructive; entry zone: Constructive entry zone; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 69.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
+          <t>RBOT.MI: scenario base Hold / Monitor, score 64.5, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.3%.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S2" t="n">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>7.49</v>
+        <v>4.97</v>
       </c>
       <c r="Z2" t="n">
-        <v>41.96</v>
+        <v>40.13</v>
       </c>
       <c r="AA2" t="n">
-        <v>22.5</v>
+        <v>22.51</v>
       </c>
       <c r="AB2" t="n">
         <v>-29.37</v>
@@ -888,50 +888,50 @@
         </is>
       </c>
       <c r="AG2" t="n">
-        <v>18.372</v>
+        <v>18.13</v>
       </c>
       <c r="AH2" t="n">
-        <v>51.7</v>
+        <v>51.5</v>
       </c>
       <c r="AI2" t="n">
-        <v>88.8</v>
+        <v>84.3</v>
       </c>
       <c r="AJ2" t="n">
         <v>44.5</v>
       </c>
       <c r="AK2" t="n">
-        <v>82.8</v>
+        <v>79.3</v>
       </c>
       <c r="AL2" t="n">
-        <v>-2.13</v>
+        <v>-3.08</v>
       </c>
       <c r="AM2" t="n">
-        <v>29.71</v>
+        <v>28.87</v>
       </c>
       <c r="AN2" t="n">
-        <v>20</v>
+        <v>19.74</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="AP2" t="n">
-        <v>18.2049</v>
+        <v>18.1845</v>
       </c>
       <c r="AQ2" t="n">
-        <v>15.9218</v>
+        <v>15.9452</v>
       </c>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT2" t="n">
-        <v>88.8</v>
+        <v>84.3</v>
       </c>
       <c r="AU2" t="n">
         <v>49.5</v>
       </c>
       <c r="AV2" t="n">
-        <v>82.8</v>
+        <v>79.3</v>
       </c>
       <c r="AW2" t="n">
         <v>756</v>
@@ -943,10 +943,10 @@
         <v>19.25</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.92</v>
+        <v>-0.3</v>
       </c>
       <c r="BA2" t="n">
-        <v>15.39</v>
+        <v>13.7</v>
       </c>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
@@ -1178,24 +1178,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASML.AS</t>
+          <t>WCLD.MI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ASML Holding N.V.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>67.7</v>
+        <v>58.9</v>
       </c>
       <c r="F4" t="n">
-        <v>55.6</v>
+        <v>52.4</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1209,7 +1205,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>score 67.7; priority 55.6; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 58.9; priority 52.4; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1229,17 +1225,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 67.7, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -0.3%.</t>
+          <t>WCLD.MI: scenario base Hold / Monitor, score 58.9, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 4.6%.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1719.33 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 36.89 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 1362.20 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1254,153 +1250,131 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Constructive</t>
+          <t>Bullish</t>
         </is>
       </c>
       <c r="S4" t="n">
-        <v>1362.2</v>
+        <v>24.785</v>
       </c>
       <c r="T4" t="n">
-        <v>1719.3295</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>ASML Holding N.V.</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+        <v>36.89</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Thematic</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>0.84</v>
+        <v>28.65</v>
       </c>
       <c r="Z4" t="n">
-        <v>124.63</v>
+        <v>10.64</v>
       </c>
       <c r="AA4" t="n">
-        <v>39.58</v>
+        <v>35.15</v>
       </c>
       <c r="AB4" t="n">
-        <v>-44.77</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>59.86</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>29.35</v>
-      </c>
+        <v>-48.6</v>
+      </c>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr"/>
+          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
       <c r="AG4" t="n">
-        <v>1518</v>
-      </c>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
+        <v>33.385</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>80.3</v>
+      </c>
       <c r="AL4" t="n">
-        <v>1.27</v>
+        <v>-1.59</v>
       </c>
       <c r="AM4" t="n">
-        <v>26.93</v>
+        <v>37.39</v>
       </c>
       <c r="AN4" t="n">
-        <v>37.96</v>
+        <v>4.41</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.96</v>
+        <v>0.13</v>
       </c>
       <c r="AP4" t="n">
-        <v>1522.5573</v>
+        <v>31.913</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1284.1927</v>
+        <v>27.1811</v>
       </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="AT4" t="n">
-        <v>98.5</v>
+        <v>100</v>
       </c>
       <c r="AU4" t="n">
-        <v>16.7</v>
+        <v>18.9</v>
       </c>
       <c r="AV4" t="n">
-        <v>79.3</v>
+        <v>80.3</v>
       </c>
       <c r="AW4" t="n">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="AX4" t="n">
-        <v>1423.4</v>
+        <v>33.385</v>
       </c>
       <c r="AY4" t="n">
-        <v>1621.2</v>
+        <v>36.89</v>
       </c>
       <c r="AZ4" t="n">
-        <v>-0.3</v>
+        <v>4.61</v>
       </c>
       <c r="BA4" t="n">
-        <v>18.21</v>
-      </c>
-      <c r="BB4" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="BC4" t="inlineStr">
-        <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
-        </is>
-      </c>
-      <c r="BD4" t="n">
-        <v>583063830528</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>30.11</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>53.94</v>
-      </c>
-      <c r="BG4" t="n">
-        <v>21.3</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>9.09</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>52</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>98.5</v>
-      </c>
-      <c r="BL4" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="BM4" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="BN4" t="n">
-        <v>79.3</v>
-      </c>
+        <v>22.82</v>
+      </c>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
       <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr">
-        <is>
-          <t>Europe / Semiconductors</t>
-        </is>
-      </c>
+      <c r="BP4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1410,17 +1384,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>ASML.AS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>ASML Holding N.V.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
       <c r="E5" t="n">
-        <v>44.3</v>
+        <v>64.5</v>
       </c>
       <c r="F5" t="n">
         <v>51.7</v>
@@ -1437,17 +1415,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>score 44.3; priority 51.7; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
+          <t>score 64.5; priority 51.7; trend: Constructive; entry zone: Monitor / partial entry only; risk flag: High risk</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Wait for trend repair</t>
+          <t>Monitor / partial entry only</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Medium-high risk</t>
+          <t>High risk</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1457,17 +1435,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Avoid for Now, score 44.3, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.9%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 64.5, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.0%.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 10.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1719.33 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+          <t>Scenario negativo: perdita area 1362.20 o peggioramento trend; rischio attuale: High risk.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1477,136 +1455,158 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Avoid for Now</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>8.541</v>
+        <v>1362.2</v>
       </c>
       <c r="T5" t="n">
-        <v>10.872</v>
-      </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Thematic</t>
-        </is>
-      </c>
+        <v>1719.3295</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>ASML Holding N.V.</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr">
         <is>
           <t>Ridurre size / solo monitoraggio</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>-8.49</v>
+        <v>-5.55</v>
       </c>
       <c r="Z5" t="n">
-        <v>29.69</v>
+        <v>118.15</v>
       </c>
       <c r="AA5" t="n">
-        <v>24.21</v>
+        <v>39.58</v>
       </c>
       <c r="AB5" t="n">
-        <v>-34.52</v>
-      </c>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
+        <v>-44.77</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>58.65</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>28.75</v>
+      </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Rischio elevato: usare solo come quota satellite e con size ridotta.</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>Energia pulita</t>
-        </is>
-      </c>
+          <t>Rischio elevato: volatilità/drawdown richiedono prudenza.</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="n">
-        <v>9.073</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>45.6</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>73.90000000000001</v>
-      </c>
+        <v>1486.8</v>
+      </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="n">
-        <v>-0.23</v>
+        <v>-1.78</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.13</v>
+        <v>24.45</v>
       </c>
       <c r="AN5" t="n">
-        <v>4.24</v>
+        <v>37.75</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.18</v>
+        <v>0.95</v>
       </c>
       <c r="AP5" t="n">
-        <v>9.1576</v>
+        <v>1517.9067</v>
       </c>
       <c r="AQ5" t="n">
-        <v>9.289899999999999</v>
+        <v>1287.353</v>
       </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="AT5" t="n">
-        <v>45.6</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AU5" t="n">
-        <v>43.3</v>
+        <v>16.7</v>
       </c>
       <c r="AV5" t="n">
-        <v>73.90000000000001</v>
+        <v>76.7</v>
       </c>
       <c r="AW5" t="n">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="AX5" t="n">
-        <v>8.541</v>
+        <v>1423.4</v>
       </c>
       <c r="AY5" t="n">
-        <v>9.217000000000001</v>
+        <v>1621.2</v>
       </c>
       <c r="AZ5" t="n">
-        <v>-0.92</v>
+        <v>-2.05</v>
       </c>
       <c r="BA5" t="n">
-        <v>-2.33</v>
-      </c>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
-      <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
-      <c r="BJ5" t="inlineStr"/>
-      <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="inlineStr"/>
-      <c r="BM5" t="inlineStr"/>
-      <c r="BN5" t="inlineStr"/>
+        <v>15.49</v>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>Semiconductor Equipment &amp; Materials</t>
+        </is>
+      </c>
+      <c r="BD5" t="n">
+        <v>571079917568</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>30.11</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>52</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>76.7</v>
+      </c>
       <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>Europe / Semiconductors</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1616,20 +1616,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WCLD.MI</t>
+          <t>INRG.MI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>58.4</v>
+        <v>43.5</v>
       </c>
       <c r="F6" t="n">
-        <v>51.4</v>
+        <v>50.9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1643,17 +1643,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>score 58.4; priority 51.4; trend: Bullish; entry zone: Monitor / partial entry only; risk flag: High risk</t>
+          <t>score 43.5; priority 50.9; trend: Weak; entry zone: Wait for trend repair; risk flag: Medium-high risk</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Monitor / partial entry only</t>
+          <t>Wait for trend repair</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>High risk</t>
+          <t>Medium-high risk</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1663,17 +1663,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>WCLD.MI: scenario base Hold / Monitor, score 58.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 5.4%.</t>
+          <t>INRG.MI: scenario base Avoid for Now, score 43.5, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -0.8%.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 36.89 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 10.87 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 24.79 o peggioramento trend; rischio attuale: High risk.</t>
+          <t>Scenario negativo: perdita area 8.54 o peggioramento trend; rischio attuale: Medium-high risk.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1683,24 +1683,24 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Hold / Monitor</t>
+          <t>Avoid for Now</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>24.785</v>
+        <v>8.541</v>
       </c>
       <c r="T6" t="n">
-        <v>36.89</v>
+        <v>10.872</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>WisdomTree Cloud Computing UCITS ETF - USD Acc</t>
+          <t>iShares Global Clean Energy Transition UCITS ETF USD (Dist)</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1714,16 +1714,16 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>26.36</v>
+        <v>-10.14</v>
       </c>
       <c r="Z6" t="n">
-        <v>12.73</v>
+        <v>27.79</v>
       </c>
       <c r="AA6" t="n">
-        <v>35.17</v>
+        <v>24.17</v>
       </c>
       <c r="AB6" t="n">
-        <v>-48.6</v>
+        <v>-34.52</v>
       </c>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -1734,69 +1734,69 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Energia pulita</t>
         </is>
       </c>
       <c r="AG6" t="n">
-        <v>33.51</v>
+        <v>9.06</v>
       </c>
       <c r="AH6" t="n">
-        <v>25.3</v>
+        <v>35.6</v>
       </c>
       <c r="AI6" t="n">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="AJ6" t="n">
-        <v>13.9</v>
+        <v>38.4</v>
       </c>
       <c r="AK6" t="n">
-        <v>77</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AL6" t="n">
-        <v>1.44</v>
+        <v>0.72</v>
       </c>
       <c r="AM6" t="n">
-        <v>36.44</v>
+        <v>-1.3</v>
       </c>
       <c r="AN6" t="n">
-        <v>4.62</v>
+        <v>4.06</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="AP6" t="n">
-        <v>31.7802</v>
+        <v>9.129300000000001</v>
       </c>
       <c r="AQ6" t="n">
-        <v>27.1553</v>
+        <v>9.293100000000001</v>
       </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="AT6" t="n">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="AU6" t="n">
-        <v>18.9</v>
+        <v>43.4</v>
       </c>
       <c r="AV6" t="n">
-        <v>77</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AW6" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AX6" t="n">
-        <v>33.51</v>
+        <v>8.541</v>
       </c>
       <c r="AY6" t="n">
-        <v>36.89</v>
+        <v>9.217000000000001</v>
       </c>
       <c r="AZ6" t="n">
-        <v>5.44</v>
+        <v>-0.76</v>
       </c>
       <c r="BA6" t="n">
-        <v>23.4</v>
+        <v>-2.51</v>
       </c>
       <c r="BB6" t="inlineStr"/>
       <c r="BC6" t="inlineStr"/>
@@ -1932,7 +1932,7 @@
         <v>-34.15</v>
       </c>
       <c r="AC7" t="n">
-        <v>23.13</v>
+        <v>23.1</v>
       </c>
       <c r="AD7" t="n">
         <v>17.55</v>
@@ -2164,7 +2164,7 @@
         <v>-53.77</v>
       </c>
       <c r="AC8" t="n">
-        <v>334.69</v>
+        <v>344.07</v>
       </c>
       <c r="AD8" t="n">
         <v>170.56</v>
@@ -2294,10 +2294,10 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>82</v>
+        <v>81.2</v>
       </c>
       <c r="F9" t="n">
-        <v>82</v>
+        <v>81.2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>score 82.0; priority 82.0; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 81.2; priority 81.2; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2326,17 +2326,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>prezzo vicino a MA50: monitorare conferma; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Buy Watchlist, score 82.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.3%.</t>
+          <t>XDEV.MI: scenario base Buy Watchlist, score 81.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.5%.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 74.14 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 74.49 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -2363,7 +2363,7 @@
         <v>69.45</v>
       </c>
       <c r="T9" t="n">
-        <v>74.14</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>7.59</v>
+        <v>6.27</v>
       </c>
       <c r="Z9" t="n">
-        <v>58.87</v>
+        <v>57.5</v>
       </c>
       <c r="AA9" t="n">
-        <v>14.14</v>
+        <v>14.16</v>
       </c>
       <c r="AB9" t="n">
         <v>-17.8</v>
@@ -2406,13 +2406,13 @@
         </is>
       </c>
       <c r="AG9" t="n">
-        <v>74.12</v>
+        <v>73.56999999999999</v>
       </c>
       <c r="AH9" t="n">
-        <v>78.5</v>
+        <v>77.7</v>
       </c>
       <c r="AI9" t="n">
-        <v>93.8</v>
+        <v>91.2</v>
       </c>
       <c r="AJ9" t="n">
         <v>68.8</v>
@@ -2421,29 +2421,29 @@
         <v>82.8</v>
       </c>
       <c r="AL9" t="n">
-        <v>2.89</v>
+        <v>2.21</v>
       </c>
       <c r="AM9" t="n">
-        <v>30.75</v>
+        <v>30.07</v>
       </c>
       <c r="AN9" t="n">
-        <v>26.63</v>
+        <v>26.11</v>
       </c>
       <c r="AO9" t="n">
-        <v>1.88</v>
+        <v>1.84</v>
       </c>
       <c r="AP9" t="n">
-        <v>71.7392</v>
+        <v>71.776</v>
       </c>
       <c r="AQ9" t="n">
-        <v>62.3373</v>
+        <v>62.4594</v>
       </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="n">
         <v>85</v>
       </c>
       <c r="AT9" t="n">
-        <v>93.8</v>
+        <v>91.2</v>
       </c>
       <c r="AU9" t="n">
         <v>68.8</v>
@@ -2458,13 +2458,13 @@
         <v>71.86</v>
       </c>
       <c r="AY9" t="n">
-        <v>74.14</v>
+        <v>74.48999999999999</v>
       </c>
       <c r="AZ9" t="n">
-        <v>3.32</v>
+        <v>2.5</v>
       </c>
       <c r="BA9" t="n">
-        <v>18.9</v>
+        <v>17.79</v>
       </c>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
@@ -2500,10 +2500,10 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>74.7</v>
+        <v>73.8</v>
       </c>
       <c r="F10" t="n">
-        <v>75.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>score 74.7; priority 75.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 73.8; priority 74.8; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Accumulate Carefully, score 74.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.6%.</t>
+          <t>EIMI.MI: scenario base Accumulate Carefully, score 73.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.0%.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2584,14 +2584,14 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>5.7</v>
+        <v>3.95</v>
       </c>
       <c r="Z10" t="n">
-        <v>39.17</v>
+        <v>37.75</v>
       </c>
       <c r="AA10" t="n">
         <v>17.07</v>
@@ -2612,13 +2612,13 @@
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>48.565</v>
+        <v>48.26</v>
       </c>
       <c r="AH10" t="n">
-        <v>68.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AI10" t="n">
-        <v>77.7</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AJ10" t="n">
         <v>64.2</v>
@@ -2627,29 +2627,29 @@
         <v>82.8</v>
       </c>
       <c r="AL10" t="n">
-        <v>4.33</v>
+        <v>3.99</v>
       </c>
       <c r="AM10" t="n">
-        <v>16.6</v>
+        <v>16.51</v>
       </c>
       <c r="AN10" t="n">
-        <v>20.15</v>
+        <v>19.69</v>
       </c>
       <c r="AO10" t="n">
-        <v>1.18</v>
+        <v>1.15</v>
       </c>
       <c r="AP10" t="n">
-        <v>46.8561</v>
+        <v>46.8418</v>
       </c>
       <c r="AQ10" t="n">
-        <v>43.6118</v>
+        <v>43.6631</v>
       </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="n">
         <v>85</v>
       </c>
       <c r="AT10" t="n">
-        <v>77.7</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AU10" t="n">
         <v>64.2</v>
@@ -2664,13 +2664,13 @@
         <v>46.37</v>
       </c>
       <c r="AY10" t="n">
-        <v>48.565</v>
+        <v>48.415</v>
       </c>
       <c r="AZ10" t="n">
-        <v>3.65</v>
+        <v>3.03</v>
       </c>
       <c r="BA10" t="n">
-        <v>11.36</v>
+        <v>10.53</v>
       </c>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2696,20 +2696,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EXSA.DE</t>
+          <t>VWCE.DE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>75</v>
+        <v>74.2</v>
       </c>
       <c r="F11" t="n">
-        <v>75.5</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2718,12 +2718,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 65.95. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>score 75.0; priority 75.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 74.2; priority 74.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2743,17 +2743,17 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 75.0, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.3%.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 65.95 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 169.62 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 63.18 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 162.02 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -2772,15 +2772,15 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>63.18</v>
+        <v>162.02</v>
       </c>
       <c r="T11" t="n">
-        <v>65.95</v>
+        <v>169.62</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
+          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -2790,20 +2790,20 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>5.62</v>
+        <v>4.44</v>
       </c>
       <c r="Z11" t="n">
-        <v>21.34</v>
+        <v>22.93</v>
       </c>
       <c r="AA11" t="n">
-        <v>12.77</v>
+        <v>13.01</v>
       </c>
       <c r="AB11" t="n">
-        <v>-16.33</v>
+        <v>-21.07</v>
       </c>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
@@ -2814,69 +2814,69 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>Europa</t>
+          <t>Azionario globale</t>
         </is>
       </c>
       <c r="AG11" t="n">
-        <v>64.93000000000001</v>
+        <v>166.64</v>
       </c>
       <c r="AH11" t="n">
-        <v>73</v>
+        <v>72.8</v>
       </c>
       <c r="AI11" t="n">
-        <v>68.90000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="AJ11" t="n">
-        <v>71.59999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="AK11" t="n">
         <v>82.8</v>
       </c>
       <c r="AL11" t="n">
-        <v>-1.5</v>
+        <v>-1.09</v>
       </c>
       <c r="AM11" t="n">
-        <v>9.42</v>
+        <v>12.59</v>
       </c>
       <c r="AN11" t="n">
-        <v>15.71</v>
+        <v>17.44</v>
       </c>
       <c r="AO11" t="n">
-        <v>1.23</v>
+        <v>1.34</v>
       </c>
       <c r="AP11" t="n">
-        <v>64.82640000000001</v>
+        <v>166.1392</v>
       </c>
       <c r="AQ11" t="n">
-        <v>60.9925</v>
+        <v>154.9367</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
         <v>85</v>
       </c>
       <c r="AT11" t="n">
-        <v>68.90000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="AU11" t="n">
-        <v>71.59999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="AV11" t="n">
         <v>82.8</v>
       </c>
       <c r="AW11" t="n">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="AX11" t="n">
-        <v>64.53</v>
+        <v>165.62</v>
       </c>
       <c r="AY11" t="n">
-        <v>65.95</v>
+        <v>169.62</v>
       </c>
       <c r="AZ11" t="n">
-        <v>0.16</v>
+        <v>0.3</v>
       </c>
       <c r="BA11" t="n">
-        <v>6.46</v>
+        <v>7.55</v>
       </c>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
@@ -2902,20 +2902,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VWCE.DE</t>
+          <t>SWDA.MI</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>74.7</v>
+        <v>70.2</v>
       </c>
       <c r="F12" t="n">
-        <v>75.09999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 169.62. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>score 74.7; priority 75.1; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 70.2; priority 71.9; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2949,17 +2949,17 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 74.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.9%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 70.2, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 169.62 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 162.02 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 123.69 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -2974,19 +2974,19 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>162.02</v>
+        <v>123.69</v>
       </c>
       <c r="T12" t="n">
-        <v>169.62</v>
+        <v>129.38</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Vanguard FTSE All-World UCITS ETF USD Accumulation</t>
+          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -2996,20 +2996,20 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Priorità watchlist</t>
+          <t>Monitorare ingresso graduale</t>
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>5.24</v>
+        <v>4.56</v>
       </c>
       <c r="Z12" t="n">
-        <v>22.97</v>
+        <v>20.9</v>
       </c>
       <c r="AA12" t="n">
-        <v>13</v>
+        <v>13.21</v>
       </c>
       <c r="AB12" t="n">
-        <v>-21.07</v>
+        <v>-21.63</v>
       </c>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
@@ -3020,69 +3020,69 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>Azionario globale</t>
+          <t>Azionario globale sviluppato</t>
         </is>
       </c>
       <c r="AG12" t="n">
-        <v>167.58</v>
+        <v>126.4</v>
       </c>
       <c r="AH12" t="n">
-        <v>73.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="AI12" t="n">
-        <v>70.8</v>
+        <v>69</v>
       </c>
       <c r="AJ12" t="n">
-        <v>67.5</v>
+        <v>66.8</v>
       </c>
       <c r="AK12" t="n">
-        <v>82.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AL12" t="n">
-        <v>-0.48</v>
+        <v>-1.83</v>
       </c>
       <c r="AM12" t="n">
-        <v>12.82</v>
+        <v>12.25</v>
       </c>
       <c r="AN12" t="n">
-        <v>17.67</v>
+        <v>17.14</v>
       </c>
       <c r="AO12" t="n">
-        <v>1.36</v>
+        <v>1.3</v>
       </c>
       <c r="AP12" t="n">
-        <v>166.1068</v>
+        <v>126.5392</v>
       </c>
       <c r="AQ12" t="n">
-        <v>154.8094</v>
+        <v>118.0113</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT12" t="n">
-        <v>70.8</v>
+        <v>69</v>
       </c>
       <c r="AU12" t="n">
-        <v>67.5</v>
+        <v>66.8</v>
       </c>
       <c r="AV12" t="n">
-        <v>82.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AW12" t="n">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="AX12" t="n">
-        <v>165.62</v>
+        <v>126.18</v>
       </c>
       <c r="AY12" t="n">
-        <v>169.62</v>
+        <v>129.38</v>
       </c>
       <c r="AZ12" t="n">
-        <v>0.89</v>
+        <v>-0.11</v>
       </c>
       <c r="BA12" t="n">
-        <v>8.25</v>
+        <v>7.11</v>
       </c>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -3108,20 +3108,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SWDA.MI</t>
+          <t>EXSA.DE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>74.09999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="F13" t="n">
-        <v>74.59999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3130,12 +3130,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Imposta alert prezzo/news. Resistenza 60D: 129.38. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
+          <t>Imposta alert prezzo/news. Resistenza 60D: 65.95. Trigger: prezzo vicino a MA50: monitorare conferma; vicino a supporto 60D: controllare tenuta e volumi.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>score 74.1; priority 74.6; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 70.2; priority 71.7; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3155,17 +3155,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 74.1, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.5%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 70.2, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.0%.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 129.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 65.95 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 123.69 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 63.18 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -3180,19 +3180,19 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>123.69</v>
+        <v>63.18</v>
       </c>
       <c r="T13" t="n">
-        <v>129.38</v>
+        <v>65.95</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>iShares Core MSCI World UCITS ETF USD (Acc)</t>
+          <t>iShares STOXX Europe 600 UCITS ETF (DE) EUR (Dist)</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -3206,16 +3206,16 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>5.33</v>
+        <v>3.7</v>
       </c>
       <c r="Z13" t="n">
-        <v>20.82</v>
+        <v>19.36</v>
       </c>
       <c r="AA13" t="n">
-        <v>13.2</v>
+        <v>12.79</v>
       </c>
       <c r="AB13" t="n">
-        <v>-21.63</v>
+        <v>-16.33</v>
       </c>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
@@ -3226,69 +3226,69 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>Azionario globale sviluppato</t>
+          <t>Europa</t>
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>127.17</v>
+        <v>64.16</v>
       </c>
       <c r="AH13" t="n">
         <v>72.09999999999999</v>
       </c>
       <c r="AI13" t="n">
-        <v>70.2</v>
+        <v>65.3</v>
       </c>
       <c r="AJ13" t="n">
-        <v>66.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AK13" t="n">
-        <v>82.8</v>
+        <v>78.2</v>
       </c>
       <c r="AL13" t="n">
-        <v>-1.17</v>
+        <v>-2.64</v>
       </c>
       <c r="AM13" t="n">
-        <v>12.53</v>
+        <v>8.73</v>
       </c>
       <c r="AN13" t="n">
-        <v>17.37</v>
+        <v>15.13</v>
       </c>
       <c r="AO13" t="n">
-        <v>1.32</v>
+        <v>1.18</v>
       </c>
       <c r="AP13" t="n">
-        <v>126.5098</v>
+        <v>64.83159999999999</v>
       </c>
       <c r="AQ13" t="n">
-        <v>117.9214</v>
+        <v>61.0385</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT13" t="n">
-        <v>70.2</v>
+        <v>65.3</v>
       </c>
       <c r="AU13" t="n">
-        <v>66.90000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AV13" t="n">
-        <v>82.8</v>
+        <v>78.2</v>
       </c>
       <c r="AW13" t="n">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="AX13" t="n">
-        <v>126.18</v>
+        <v>64.16</v>
       </c>
       <c r="AY13" t="n">
-        <v>129.38</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="AZ13" t="n">
-        <v>0.52</v>
+        <v>-1.04</v>
       </c>
       <c r="BA13" t="n">
-        <v>7.84</v>
+        <v>5.11</v>
       </c>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -3324,10 +3324,10 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>72.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>73.5</v>
+        <v>71</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>score 72.8; priority 73.5; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 69.1; priority 71.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3361,7 +3361,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 72.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 69.1, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.2%.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S14" t="n">
@@ -3412,10 +3412,10 @@
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>4.6</v>
+        <v>4.25</v>
       </c>
       <c r="Z14" t="n">
-        <v>20.07</v>
+        <v>20.64</v>
       </c>
       <c r="AA14" t="n">
         <v>14.26</v>
@@ -3436,50 +3436,50 @@
         </is>
       </c>
       <c r="AG14" t="n">
-        <v>713.04</v>
+        <v>710.22</v>
       </c>
       <c r="AH14" t="n">
-        <v>69.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AI14" t="n">
-        <v>69.5</v>
+        <v>69</v>
       </c>
       <c r="AJ14" t="n">
         <v>64.2</v>
       </c>
       <c r="AK14" t="n">
-        <v>82.8</v>
+        <v>79.5</v>
       </c>
       <c r="AL14" t="n">
-        <v>-1.38</v>
+        <v>-1.88</v>
       </c>
       <c r="AM14" t="n">
-        <v>13.4</v>
+        <v>13.09</v>
       </c>
       <c r="AN14" t="n">
-        <v>17.78</v>
+        <v>17.71</v>
       </c>
       <c r="AO14" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="AP14" t="n">
-        <v>711.2744</v>
+        <v>711.3988000000001</v>
       </c>
       <c r="AQ14" t="n">
-        <v>661.5055</v>
+        <v>661.9877</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT14" t="n">
-        <v>69.5</v>
+        <v>69</v>
       </c>
       <c r="AU14" t="n">
         <v>64.2</v>
       </c>
       <c r="AV14" t="n">
-        <v>82.8</v>
+        <v>79.5</v>
       </c>
       <c r="AW14" t="n">
         <v>758</v>
@@ -3491,10 +3491,10 @@
         <v>727.1799999999999</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0.25</v>
+        <v>-0.17</v>
       </c>
       <c r="BA14" t="n">
-        <v>7.79</v>
+        <v>7.29</v>
       </c>
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
@@ -3530,10 +3530,10 @@
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>71.3</v>
+        <v>67.8</v>
       </c>
       <c r="F15" t="n">
-        <v>73.3</v>
+        <v>71</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>score 71.3; priority 73.3; trend: Bullish; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 67.8; priority 71.0; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 71.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.2%.</t>
+          <t>MVOL.MI: scenario base Hold / Monitor, score 67.8, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.1%.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -3587,12 +3587,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Accumulate Carefully</t>
+          <t>Hold / Monitor</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Bullish</t>
+          <t>Constructive</t>
         </is>
       </c>
       <c r="S15" t="n">
@@ -3618,13 +3618,13 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>4.08</v>
+        <v>3.65</v>
       </c>
       <c r="Z15" t="n">
-        <v>5.96</v>
+        <v>6.59</v>
       </c>
       <c r="AA15" t="n">
-        <v>9.710000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AB15" t="n">
         <v>-12.85</v>
@@ -3642,65 +3642,65 @@
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>66.8</v>
+        <v>66.66</v>
       </c>
       <c r="AH15" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
       <c r="AI15" t="n">
-        <v>58.9</v>
+        <v>58.7</v>
       </c>
       <c r="AJ15" t="n">
         <v>78.09999999999999</v>
       </c>
       <c r="AK15" t="n">
-        <v>82.8</v>
+        <v>79.7</v>
       </c>
       <c r="AL15" t="n">
-        <v>-1.08</v>
+        <v>-1.46</v>
       </c>
       <c r="AM15" t="n">
-        <v>2.77</v>
+        <v>3.22</v>
       </c>
       <c r="AN15" t="n">
-        <v>7.78</v>
+        <v>7.69</v>
       </c>
       <c r="AO15" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="AP15" t="n">
-        <v>66.6572</v>
+        <v>66.7012</v>
       </c>
       <c r="AQ15" t="n">
-        <v>64.20699999999999</v>
+        <v>64.2291</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="AT15" t="n">
-        <v>58.9</v>
+        <v>58.7</v>
       </c>
       <c r="AU15" t="n">
         <v>78.09999999999999</v>
       </c>
       <c r="AV15" t="n">
-        <v>82.8</v>
+        <v>79.7</v>
       </c>
       <c r="AW15" t="n">
         <v>756</v>
       </c>
       <c r="AX15" t="n">
-        <v>66.8</v>
+        <v>66.66</v>
       </c>
       <c r="AY15" t="n">
         <v>67.81999999999999</v>
       </c>
       <c r="AZ15" t="n">
-        <v>0.21</v>
+        <v>-0.06</v>
       </c>
       <c r="BA15" t="n">
-        <v>4.04</v>
+        <v>3.78</v>
       </c>
       <c r="BB15" t="inlineStr"/>
       <c r="BC15" t="inlineStr"/>
@@ -3839,7 +3839,7 @@
         <v>36.18</v>
       </c>
       <c r="AD16" t="n">
-        <v>33.03</v>
+        <v>33.02</v>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
@@ -3968,10 +3968,10 @@
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>67.90000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="F17" t="n">
-        <v>70.5</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>score 67.9; priority 70.5; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 67.5; priority 69.9; trend: Constructive; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Hold / Monitor, score 67.9, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -0.6%.</t>
+          <t>IWQU.MI: scenario base Hold / Monitor, score 67.5, trend Constructive. Entry zone: Constructive entry zone. Distanza da MA50: -1.0%.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -4056,13 +4056,13 @@
         </is>
       </c>
       <c r="Y17" t="n">
-        <v>4.07</v>
+        <v>3.11</v>
       </c>
       <c r="Z17" t="n">
-        <v>19.23</v>
+        <v>19.87</v>
       </c>
       <c r="AA17" t="n">
-        <v>12.86</v>
+        <v>12.87</v>
       </c>
       <c r="AB17" t="n">
         <v>-20.6</v>
@@ -4080,65 +4080,65 @@
         </is>
       </c>
       <c r="AG17" t="n">
-        <v>77.02</v>
+        <v>76.67</v>
       </c>
       <c r="AH17" t="n">
         <v>64.5</v>
       </c>
       <c r="AI17" t="n">
-        <v>66.5</v>
+        <v>65.3</v>
       </c>
       <c r="AJ17" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AK17" t="n">
-        <v>78.90000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AL17" t="n">
-        <v>-1.9</v>
+        <v>-2.52</v>
       </c>
       <c r="AM17" t="n">
-        <v>10.03</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="AN17" t="n">
-        <v>14.69</v>
+        <v>14.61</v>
       </c>
       <c r="AO17" t="n">
         <v>1.14</v>
       </c>
       <c r="AP17" t="n">
-        <v>77.4716</v>
+        <v>77.4736</v>
       </c>
       <c r="AQ17" t="n">
-        <v>72.29770000000001</v>
+        <v>72.3518</v>
       </c>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="n">
         <v>65</v>
       </c>
       <c r="AT17" t="n">
-        <v>66.5</v>
+        <v>65.3</v>
       </c>
       <c r="AU17" t="n">
         <v>68.09999999999999</v>
       </c>
       <c r="AV17" t="n">
-        <v>78.90000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="AW17" t="n">
         <v>756</v>
       </c>
       <c r="AX17" t="n">
-        <v>77.02</v>
+        <v>76.67</v>
       </c>
       <c r="AY17" t="n">
         <v>78.87</v>
       </c>
       <c r="AZ17" t="n">
-        <v>-0.58</v>
+        <v>-1.04</v>
       </c>
       <c r="BA17" t="n">
-        <v>6.53</v>
+        <v>5.97</v>
       </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
@@ -4504,7 +4504,7 @@
         <v>-29.81</v>
       </c>
       <c r="AC19" t="n">
-        <v>16.97</v>
+        <v>16.98</v>
       </c>
       <c r="AD19" t="n">
         <v>22.78</v>
@@ -4636,10 +4636,10 @@
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>62.2</v>
+        <v>62.5</v>
       </c>
       <c r="F20" t="n">
-        <v>64.59999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>score 62.2; priority 64.6; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
+          <t>score 62.5; priority 64.9; trend: Recovery; entry zone: Constructive entry zone; risk flag: Normal risk</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>SGLD.MI: scenario base Hold / Monitor, score 62.2, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.6%.</t>
+          <t>SGLD.MI: scenario base Hold / Monitor, score 62.5, trend Recovery. Entry zone: Constructive entry zone. Distanza da MA50: 2.2%.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -4724,10 +4724,10 @@
         </is>
       </c>
       <c r="Y20" t="n">
-        <v>5.98</v>
+        <v>6.62</v>
       </c>
       <c r="Z20" t="n">
-        <v>24.24</v>
+        <v>23.5</v>
       </c>
       <c r="AA20" t="n">
         <v>18.99</v>
@@ -4748,13 +4748,13 @@
         </is>
       </c>
       <c r="AG20" t="n">
-        <v>364.27</v>
+        <v>363.39</v>
       </c>
       <c r="AH20" t="n">
         <v>66.90000000000001</v>
       </c>
       <c r="AI20" t="n">
-        <v>55</v>
+        <v>55.9</v>
       </c>
       <c r="AJ20" t="n">
         <v>59</v>
@@ -4763,29 +4763,29 @@
         <v>78.2</v>
       </c>
       <c r="AL20" t="n">
-        <v>0.58</v>
+        <v>0.34</v>
       </c>
       <c r="AM20" t="n">
-        <v>-15.72</v>
+        <v>-15.45</v>
       </c>
       <c r="AN20" t="n">
-        <v>28.15</v>
+        <v>28.14</v>
       </c>
       <c r="AO20" t="n">
         <v>1.48</v>
       </c>
       <c r="AP20" t="n">
-        <v>355.1802</v>
+        <v>355.6742</v>
       </c>
       <c r="AQ20" t="n">
-        <v>373.9302</v>
+        <v>374.0494</v>
       </c>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="n">
         <v>55</v>
       </c>
       <c r="AT20" t="n">
-        <v>55</v>
+        <v>55.9</v>
       </c>
       <c r="AU20" t="n">
         <v>59</v>
@@ -4803,10 +4803,10 @@
         <v>384.93</v>
       </c>
       <c r="AZ20" t="n">
-        <v>2.56</v>
+        <v>2.17</v>
       </c>
       <c r="BA20" t="n">
-        <v>-2.58</v>
+        <v>-2.85</v>
       </c>
       <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
         <v>16.97</v>
       </c>
       <c r="BI22" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="BJ22" t="n">
         <v>100</v>

</xml_diff>